<commit_message>
Add rotting oranges to tracker and emphasize initial fresh count check
</commit_message>
<xml_diff>
--- a/leetcode_hot100/LeetCode Hot100与高频题目刷题清单与进度追踪表.xlsx
+++ b/leetcode_hot100/LeetCode Hot100与高频题目刷题清单与进度追踪表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hot100与高频题目" sheetId="1" r:id="Rfc8cf4d7a326477e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hot100与高频题目" sheetId="1" r:id="Rd8e30cef1a514d8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="17">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -72,14 +72,14 @@
       <x:name val="微软雅黑"/>
     </x:font>
     <x:font>
-      <x:sz val="9"/>
-      <x:color rgb="FF000000"/>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F4E79"/>
       <x:name val="微软雅黑"/>
     </x:font>
     <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF1F4E79"/>
+      <x:sz val="9"/>
+      <x:color rgb="FF000000"/>
       <x:name val="微软雅黑"/>
     </x:font>
     <x:font>
@@ -99,6 +99,12 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FFC00000"/>
+      <x:name val="微软雅黑"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFF0000"/>
       <x:name val="微软雅黑"/>
     </x:font>
     <x:font>
@@ -205,7 +211,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="94">
+  <x:cellXfs count="104">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -346,9 +352,20 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -357,10 +374,7 @@
     <x:xf numFmtId="200" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="11" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="201" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -408,6 +422,20 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -620,8 +648,8 @@
     <col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="34" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="9" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="8" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="11" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="8" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="42" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="14" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="10" hidden="0" customWidth="1"/>
@@ -631,7 +659,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="5" t="str">
-        <v>LeetCode Hot 100 与高频题目总数：103</v>
+        <v>LeetCode Hot 100 与高频题目总数：104</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -709,7 +737,7 @@
       <c r="A4" s="28" t="str">
         <v>哈希</v>
       </c>
-      <c r="B4" s="93" t="str">
+      <c r="B4" s="103" t="str">
         <v>分组哈希</v>
       </c>
       <c r="C4" s="34" t="n">
@@ -718,7 +746,7 @@
       <c r="D4" s="34" t="n">
         <v>49</v>
       </c>
-      <c r="E4" s="67" t="str">
+      <c r="E4" s="72" t="str">
         <v>49. 字母异位词分组</v>
       </c>
       <c r="F4" s="45" t="str">
@@ -729,21 +757,21 @@
       <c r="I4" s="56" t="str">
         <v>leetcode.cn/problems/group-anagrams/</v>
       </c>
-      <c r="J4" s="68" t="str">
+      <c r="J4" s="73" t="str">
         <v>√</v>
       </c>
-      <c r="K4" s="70" t="n">
+      <c r="K4" s="74" t="n">
         <f>LEN(J4)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J4,"√",""),"×",""),"✓",""))</f>
         <v>1</v>
       </c>
-      <c r="L4" s="66" t="str">
+      <c r="L4" s="71" t="str">
         <v>if goal not in dict 与 if goal not in dict.keys()在性能上有较大区别，dict.keys()先生成一个字典键的列表，然后在这个列表里线性查找，时间复杂度为o(n),而in d…</v>
       </c>
-      <c r="M4" s="66"/>
+      <c r="M4" s="71"/>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="28"/>
-      <c r="B5" s="93" t="str">
+      <c r="B5" s="103" t="str">
         <v>集合查找</v>
       </c>
       <c r="C5" s="34" t="n">
@@ -752,7 +780,7 @@
       <c r="D5" s="34" t="n">
         <v>128</v>
       </c>
-      <c r="E5" s="67" t="str">
+      <c r="E5" s="72" t="str">
         <v>128. 最长连续序列</v>
       </c>
       <c r="F5" s="45" t="str">
@@ -763,21 +791,21 @@
       <c r="I5" s="56" t="str">
         <v>leetcode.cn/problems/longest-consecutive-sequence/</v>
       </c>
-      <c r="J5" s="68"/>
-      <c r="K5" s="70" t="n">
+      <c r="J5" s="73"/>
+      <c r="K5" s="74" t="n">
         <f>LEN(J5)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J5,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L5" s="66" t="str">
+      <c r="L5" s="71" t="str">
         <v>用 HashSet 实现 $O(1)$ 查找，只对“没有前驱数”的数字作为起点向后累加计算长度，确保每个数字最多只被遍历常数次，从而在 $O(n)$ 时间内找到最长连续序列。</v>
       </c>
-      <c r="M5" s="66"/>
+      <c r="M5" s="71"/>
     </row>
     <row r="6" ht="50" customHeight="1">
       <c r="A6" s="28" t="str">
         <v>双指针</v>
       </c>
-      <c r="B6" s="93" t="str">
+      <c r="B6" s="103" t="str">
         <v>同向双指针</v>
       </c>
       <c r="C6" s="34" t="n">
@@ -786,10 +814,10 @@
       <c r="D6" s="34" t="n">
         <v>283</v>
       </c>
-      <c r="E6" s="67" t="str">
+      <c r="E6" s="72" t="str">
         <v>283. 移动零</v>
       </c>
-      <c r="F6" s="76" t="str">
+      <c r="F6" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G6" s="51"/>
@@ -797,19 +825,19 @@
       <c r="I6" s="56" t="str">
         <v>leetcode.cn/problems/move-zeroes/</v>
       </c>
-      <c r="J6" s="68"/>
-      <c r="K6" s="70" t="n">
+      <c r="J6" s="73"/>
+      <c r="K6" s="74" t="n">
         <f>LEN(J6)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J6,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L6" s="81" t="str">
+      <c r="L6" s="85" t="str">
         <v>保证下标[left,right-1]区域都是0,其中left指向第一个0元素;当遇到一个非0数字后,将left与right位置元素互换;然后将left+1,保证该区间内仍是非0元素</v>
       </c>
-      <c r="M6" s="81"/>
+      <c r="M6" s="85"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="28"/>
-      <c r="B7" s="93" t="str">
+      <c r="B7" s="103" t="str">
         <v>相向双指针</v>
       </c>
       <c r="C7" s="34" t="n">
@@ -818,7 +846,7 @@
       <c r="D7" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="E7" s="67" t="str">
+      <c r="E7" s="72" t="str">
         <v>15. 三数之和</v>
       </c>
       <c r="F7" s="45" t="str">
@@ -829,26 +857,26 @@
       <c r="I7" s="56" t="str">
         <v>leetcode.cn/problems/3sum/</v>
       </c>
-      <c r="J7" s="68"/>
-      <c r="K7" s="70" t="n">
+      <c r="J7" s="73"/>
+      <c r="K7" s="74" t="n">
         <f>LEN(J7)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J7,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L7" s="66" t="str">
+      <c r="L7" s="71" t="str">
         <v>固定第一个数x，剩余区间相向双指针；i、j、k 三处都要跳过重复元素去重;注意sum求和要写在循环里面</v>
       </c>
-      <c r="M7" s="66"/>
+      <c r="M7" s="71"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="28"/>
-      <c r="B8" s="93"/>
+      <c r="B8" s="103"/>
       <c r="C8" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>167</v>
       </c>
-      <c r="E8" s="67" t="str">
+      <c r="E8" s="72" t="str">
         <v>167. 两数之和 II - 输入有序数组</v>
       </c>
       <c r="F8" s="45" t="str">
@@ -859,19 +887,19 @@
       <c r="I8" s="56" t="str">
         <v>leetcode.cn/problems/two-sum-ii-input-array-is-sorted/</v>
       </c>
-      <c r="J8" s="68"/>
-      <c r="K8" s="70" t="n">
+      <c r="J8" s="73"/>
+      <c r="K8" s="74" t="n">
         <f>LEN(J8)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J8,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L8" s="66" t="str">
+      <c r="L8" s="71" t="str">
         <v>相向双指针：数组有序，和&lt;target左指针右移，和&gt;target右指针左移（题目下标从1开始）</v>
       </c>
-      <c r="M8" s="66"/>
+      <c r="M8" s="71"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="28"/>
-      <c r="B9" s="93" t="str">
+      <c r="B9" s="103" t="str">
         <v>接雨水</v>
       </c>
       <c r="C9" s="34" t="n">
@@ -880,10 +908,10 @@
       <c r="D9" s="34" t="n">
         <v>42</v>
       </c>
-      <c r="E9" s="67" t="str">
+      <c r="E9" s="72" t="str">
         <v>42. 接雨水</v>
       </c>
-      <c r="F9" s="87" t="str">
+      <c r="F9" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G9" s="51"/>
@@ -891,21 +919,21 @@
       <c r="I9" s="56" t="str">
         <v>leetcode.cn/problems/trapping-rain-water/</v>
       </c>
-      <c r="J9" s="68"/>
-      <c r="K9" s="70" t="n">
+      <c r="J9" s="73"/>
+      <c r="K9" s="74" t="n">
         <f>LEN(J9)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J9,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L9" s="66" t="str">
+      <c r="L9" s="71" t="str">
         <v>三种解法：前后缀最大值 / 相向双指针 / 单调栈；每格存水量=min(左最高,右最高)-height,短板效应</v>
       </c>
-      <c r="M9" s="66"/>
+      <c r="M9" s="71"/>
     </row>
     <row r="10" ht="78" customHeight="1">
       <c r="A10" s="28" t="str">
         <v>滑动窗口</v>
       </c>
-      <c r="B10" s="93" t="str">
+      <c r="B10" s="103" t="str">
         <v>不定长窗口</v>
       </c>
       <c r="C10" s="34" t="n">
@@ -914,7 +942,7 @@
       <c r="D10" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="67" t="str">
+      <c r="E10" s="72" t="str">
         <v>3. 无重复字符的最长子串</v>
       </c>
       <c r="F10" s="45" t="str">
@@ -925,26 +953,26 @@
       <c r="I10" s="56" t="str">
         <v>leetcode.cn/problems/longest-substring-without-repeating-characters/</v>
       </c>
-      <c r="J10" s="68"/>
-      <c r="K10" s="70" t="n">
+      <c r="J10" s="73"/>
+      <c r="K10" s="74" t="n">
         <f>LEN(J10)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J10,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L10" s="66" t="str">
+      <c r="L10" s="71" t="str">
         <v>注意当题目要求返回长度的时候，不一定需要创建一个变量来记录长度，使用左右指针同样可以做到 要特别注意索引在求解数组，字符串长度时的重要作用 这个题是从不满足条件到满足条件，因此从循环退出来后再去判断子串的最大长度;同时注意是要判断最新进来的字符串计数是否超过1!而不是判断是否不等于1</v>
       </c>
-      <c r="M10" s="66"/>
+      <c r="M10" s="71"/>
     </row>
     <row r="11" ht="78" customHeight="1">
       <c r="A11" s="28"/>
-      <c r="B11" s="93"/>
+      <c r="B11" s="103"/>
       <c r="C11" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="34" t="n">
         <v>209</v>
       </c>
-      <c r="E11" s="67" t="str">
+      <c r="E11" s="72" t="str">
         <v>209. 长度最小的子数组</v>
       </c>
       <c r="F11" s="45" t="str">
@@ -955,26 +983,26 @@
       <c r="I11" s="56" t="str">
         <v>leetcode.cn/problems/minimum-size-subarray-sum/</v>
       </c>
-      <c r="J11" s="68"/>
-      <c r="K11" s="70" t="n">
+      <c r="J11" s="73"/>
+      <c r="K11" s="74" t="n">
         <f>LEN(J11)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J11,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L11" s="66" t="str">
+      <c r="L11" s="71" t="str">
         <v>（这个题进入循环意味着满足条件，因此在满足条件的情况下去判断数组长度的最小值） 对于这个题而言，一个很关键的条件是数组全是正整数，满足单调性，即数越多值越大，数越少值越小，所以可以使用不定长滑动窗口算法 左指针的移动原理…</v>
       </c>
-      <c r="M11" s="66"/>
+      <c r="M11" s="71"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="28"/>
-      <c r="B12" s="93"/>
+      <c r="B12" s="103"/>
       <c r="C12" s="34" t="n">
         <v>3</v>
       </c>
       <c r="D12" s="34" t="n">
         <v>713</v>
       </c>
-      <c r="E12" s="67" t="str">
+      <c r="E12" s="72" t="str">
         <v>713. 乘积小于 K 的子数组</v>
       </c>
       <c r="F12" s="45" t="str">
@@ -985,19 +1013,19 @@
       <c r="I12" s="56" t="str">
         <v>leetcode.cn/problems/subarray-product-less-than-k/</v>
       </c>
-      <c r="J12" s="68"/>
-      <c r="K12" s="70" t="n">
+      <c r="J12" s="73"/>
+      <c r="K12" s="74" t="n">
         <f>LEN(J12)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J12,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L12" s="66" t="str">
+      <c r="L12" s="71" t="str">
         <v>这个题也用到了单调性这个重要的概念，对于一个正数数组而言，数越多乘积越大，反之相反</v>
       </c>
-      <c r="M12" s="66"/>
+      <c r="M12" s="71"/>
     </row>
     <row r="13" ht="50" customHeight="1">
       <c r="A13" s="28"/>
-      <c r="B13" s="93" t="str">
+      <c r="B13" s="103" t="str">
         <v>异位词窗口</v>
       </c>
       <c r="C13" s="34" t="n">
@@ -1006,7 +1034,7 @@
       <c r="D13" s="34" t="n">
         <v>438</v>
       </c>
-      <c r="E13" s="67" t="str">
+      <c r="E13" s="72" t="str">
         <v>438. 找到字符串中所有字母异位词</v>
       </c>
       <c r="F13" s="45" t="str">
@@ -1017,21 +1045,21 @@
       <c r="I13" s="56" t="str">
         <v>leetcode.cn/problems/find-all-anagrams-in-a-string/</v>
       </c>
-      <c r="J13" s="68"/>
-      <c r="K13" s="70" t="n">
+      <c r="J13" s="73"/>
+      <c r="K13" s="74" t="n">
         <f>LEN(J13)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J13,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L13" s="66" t="str">
+      <c r="L13" s="71" t="str">
         <v>（定长滑动窗口） 思路就是先构建一个定长滑动窗口，然后逐渐加入右边的值，删除左边的值，保证滑动窗口的长度不变，然后进行判断</v>
       </c>
-      <c r="M13" s="66"/>
+      <c r="M13" s="71"/>
     </row>
     <row r="14" ht="50" customHeight="1">
       <c r="A14" s="28" t="str">
         <v>子串</v>
       </c>
-      <c r="B14" s="93" t="str">
+      <c r="B14" s="103" t="str">
         <v>前缀和与计数</v>
       </c>
       <c r="C14" s="34" t="n">
@@ -1040,7 +1068,7 @@
       <c r="D14" s="34" t="n">
         <v>560</v>
       </c>
-      <c r="E14" s="67" t="str">
+      <c r="E14" s="72" t="str">
         <v>560. 和为 K 的子数组</v>
       </c>
       <c r="F14" s="45" t="str">
@@ -1051,21 +1079,21 @@
       <c r="I14" s="56" t="str">
         <v>leetcode.cn/problems/subarray-sum-equals-k/</v>
       </c>
-      <c r="J14" s="68"/>
-      <c r="K14" s="70" t="n">
+      <c r="J14" s="73"/>
+      <c r="K14" s="74" t="n">
         <f>LEN(J14)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J14,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L14" s="66" t="str">
+      <c r="L14" s="71" t="str">
         <v>这个题不能采用滑动窗口算法，因为不满足单调性，数组中存在负数，思路与二叉树中的路径之和III相似，使用哈希表与前缀求和的方式，具体参考路径之和III。</v>
       </c>
-      <c r="M14" s="66" t="str">
+      <c r="M14" s="71" t="str">
         <v>做错一次,彻底没有想起来</v>
       </c>
     </row>
     <row r="15" ht="78" customHeight="1">
       <c r="A15" s="28"/>
-      <c r="B15" s="93" t="str">
+      <c r="B15" s="103" t="str">
         <v>单调队列窗口</v>
       </c>
       <c r="C15" s="34" t="n">
@@ -1074,10 +1102,10 @@
       <c r="D15" s="34" t="n">
         <v>239</v>
       </c>
-      <c r="E15" s="67" t="str">
+      <c r="E15" s="72" t="str">
         <v>239. 滑动窗口最大值</v>
       </c>
-      <c r="F15" s="87" t="str">
+      <c r="F15" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G15" s="51"/>
@@ -1085,21 +1113,21 @@
       <c r="I15" s="56" t="str">
         <v>leetcode.cn/problems/sliding-window-maximum/</v>
       </c>
-      <c r="J15" s="68"/>
-      <c r="K15" s="70" t="n">
+      <c r="J15" s="73"/>
+      <c r="K15" s="74" t="n">
         <f>LEN(J15)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J15,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L15" s="66" t="str">
+      <c r="L15" s="71" t="str">
         <v>算法的核心思想是维护一个单调递减的队列，当新元素的值大于等于队尾的值的时候，那么末尾元素就不可能作为后续的最大值了，（但这个元素可能作为以它为结尾的最大值，但后续因为滑动窗口始终包含新旧元素，因此旧元素不可能是最大…</v>
       </c>
-      <c r="M15" s="66" t="str">
+      <c r="M15" s="71" t="str">
         <v>最近一次做错,条件应该是i - queue[0] == k,而不是k-1</v>
       </c>
     </row>
     <row r="16" ht="71" customHeight="1">
       <c r="A16" s="28"/>
-      <c r="B16" s="93" t="str">
+      <c r="B16" s="103" t="str">
         <v>覆盖窗口</v>
       </c>
       <c r="C16" s="34" t="n">
@@ -1108,10 +1136,10 @@
       <c r="D16" s="34" t="n">
         <v>76</v>
       </c>
-      <c r="E16" s="67" t="str">
+      <c r="E16" s="72" t="str">
         <v>76. 最小覆盖子串</v>
       </c>
-      <c r="F16" s="87" t="str">
+      <c r="F16" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G16" s="51"/>
@@ -1119,15 +1147,15 @@
       <c r="I16" s="56" t="str">
         <v>leetcode.cn/problems/minimum-window-substring/</v>
       </c>
-      <c r="J16" s="68"/>
-      <c r="K16" s="70" t="n">
+      <c r="J16" s="73"/>
+      <c r="K16" s="74" t="n">
         <f>LEN(J16)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J16,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L16" s="66" t="str">
+      <c r="L16" s="71" t="str">
         <v>不定长滑动窗口的思路,内部循环是从满足条件到不满足条件,使用diff来统计当前窗口中 c 的数量 − t 中 c 的数量;使用ge_num来统计s是否覆盖t,当要删除左侧元素也就是left的时候,首先要判断diff[left] == 0,如果成立的话说明删除后s中对应的字符串数量小于t中,应该将ge_num-1.</v>
       </c>
-      <c r="M16" s="66" t="str">
+      <c r="M16" s="71" t="str">
         <v>最近一次做错,当判断当前滑动窗口左侧的元素对应数值为0是,应该使用s[left]而不是left</v>
       </c>
     </row>
@@ -1135,7 +1163,7 @@
       <c r="A17" s="28" t="str">
         <v>普通数组</v>
       </c>
-      <c r="B17" s="93" t="str">
+      <c r="B17" s="103" t="str">
         <v>连续子数组</v>
       </c>
       <c r="C17" s="34" t="n">
@@ -1144,7 +1172,7 @@
       <c r="D17" s="34" t="n">
         <v>53</v>
       </c>
-      <c r="E17" s="67" t="str">
+      <c r="E17" s="72" t="str">
         <v>53. 最大子数组和</v>
       </c>
       <c r="F17" s="45" t="str">
@@ -1155,19 +1183,19 @@
       <c r="I17" s="56" t="str">
         <v>leetcode.cn/problems/maximum-subarray/</v>
       </c>
-      <c r="J17" s="68"/>
-      <c r="K17" s="70" t="n">
+      <c r="J17" s="73"/>
+      <c r="K17" s="74" t="n">
         <f>LEN(J17)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J17,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L17" s="66" t="str">
+      <c r="L17" s="71" t="str">
         <v>Kadane算法的核心思想是：动态规划 遍历数组，对于每个位置，决定是继续扩展当前子数组，还是从当前位置开始新的子数组 通过比较"当前元素值"与"当前元素值+之前子数组和"来做出决策</v>
       </c>
-      <c r="M17" s="66"/>
+      <c r="M17" s="71"/>
     </row>
     <row r="18" ht="45.79999923706055" customHeight="1">
       <c r="A18" s="28"/>
-      <c r="B18" s="93" t="str">
+      <c r="B18" s="103" t="str">
         <v>区间合并</v>
       </c>
       <c r="C18" s="34" t="n">
@@ -1176,7 +1204,7 @@
       <c r="D18" s="34" t="n">
         <v>56</v>
       </c>
-      <c r="E18" s="67" t="str">
+      <c r="E18" s="72" t="str">
         <v>56. 合并区间</v>
       </c>
       <c r="F18" s="45" t="str">
@@ -1187,21 +1215,21 @@
       <c r="I18" s="56" t="str">
         <v>leetcode.cn/problems/merge-intervals/</v>
       </c>
-      <c r="J18" s="68" t="str">
+      <c r="J18" s="73" t="str">
         <v>√</v>
       </c>
-      <c r="K18" s="70" t="n">
+      <c r="K18" s="74" t="n">
         <f>LEN(J18)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J18,"√",""),"×",""),"✓",""))</f>
         <v>1</v>
       </c>
-      <c r="L18" s="66" t="str">
+      <c r="L18" s="71" t="str">
         <v>思路很简单,先按照第一个值进行排序,然后如果两个区间根本没有交集的话,直接加入区间,如果说有交集的话,区间的结束点取最大值,进行合并.</v>
       </c>
-      <c r="M18" s="66"/>
+      <c r="M18" s="71"/>
     </row>
     <row r="19" ht="78" customHeight="1">
       <c r="A19" s="28"/>
-      <c r="B19" s="93" t="str">
+      <c r="B19" s="103" t="str">
         <v>原地变换</v>
       </c>
       <c r="C19" s="34" t="n">
@@ -1210,7 +1238,7 @@
       <c r="D19" s="34" t="n">
         <v>189</v>
       </c>
-      <c r="E19" s="67" t="str">
+      <c r="E19" s="72" t="str">
         <v>189. 轮转数组</v>
       </c>
       <c r="F19" s="45" t="str">
@@ -1221,19 +1249,19 @@
       <c r="I19" s="56" t="str">
         <v>leetcode.cn/problems/rotate-array/</v>
       </c>
-      <c r="J19" s="68"/>
-      <c r="K19" s="70" t="n">
+      <c r="J19" s="73"/>
+      <c r="K19" s="74" t="n">
         <f>LEN(J19)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J19,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L19" s="66" t="str">
-        <v>1. nums[:] = nums[length-k:]+nums[:length-k] 2. nums = nums[length-k:]+nums[:length-k] 这是两个完全不同的操作，操作1对nums指向的…</v>
-      </c>
-      <c r="M19" s="66"/>
+      <c r="L19" s="96" t="str">
+        <v>使用三次反转法,同时需要注意对k的处理:k = k % n,避免k的值不合理</v>
+      </c>
+      <c r="M19" s="71"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="28"/>
-      <c r="B20" s="93" t="str">
+      <c r="B20" s="103" t="str">
         <v>前后缀乘积</v>
       </c>
       <c r="C20" s="34" t="n">
@@ -1242,7 +1270,7 @@
       <c r="D20" s="34" t="n">
         <v>238</v>
       </c>
-      <c r="E20" s="67" t="str">
+      <c r="E20" s="72" t="str">
         <v>238. 除自身以外数组的乘积</v>
       </c>
       <c r="F20" s="45" t="str">
@@ -1253,19 +1281,19 @@
       <c r="I20" s="56" t="str">
         <v>leetcode.cn/problems/product-of-array-except-self/</v>
       </c>
-      <c r="J20" s="68"/>
-      <c r="K20" s="70" t="n">
+      <c r="J20" s="73"/>
+      <c r="K20" s="74" t="n">
         <f>LEN(J20)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J20,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L20" s="66" t="str">
+      <c r="L20" s="71" t="str">
         <v>思路：求每个数组元素的前缀与后缀乘积，然后令前后缀相乘</v>
       </c>
-      <c r="M20" s="66"/>
+      <c r="M20" s="71"/>
     </row>
     <row r="21" ht="78" customHeight="1">
       <c r="A21" s="28"/>
-      <c r="B21" s="93" t="str">
+      <c r="B21" s="103" t="str">
         <v>原地哈希</v>
       </c>
       <c r="C21" s="34" t="n">
@@ -1274,10 +1302,10 @@
       <c r="D21" s="34" t="n">
         <v>41</v>
       </c>
-      <c r="E21" s="67" t="str">
+      <c r="E21" s="72" t="str">
         <v>41. 缺失的第一个正数</v>
       </c>
-      <c r="F21" s="87" t="str">
+      <c r="F21" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G21" s="51"/>
@@ -1285,21 +1313,21 @@
       <c r="I21" s="56" t="str">
         <v>leetcode.cn/problems/first-missing-positive/</v>
       </c>
-      <c r="J21" s="68"/>
-      <c r="K21" s="70" t="n">
+      <c r="J21" s="73"/>
+      <c r="K21" s="74" t="n">
         <f>LEN(J21)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J21,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L21" s="66" t="str">
-        <v>思想： 看学号为1到n的学生是否坐在了0到n-1的位置上 对于一个长度为n的数组，它的索引范围为[0,n-1],缺失的第一个正数一定在[1,n+1]的范围内，所以对于一个学号为nums[i]的学生，他应该坐在nums[i…</v>
-      </c>
-      <c r="M21" s="66"/>
-    </row>
-    <row r="22" ht="36" customHeight="1">
+      <c r="L21" s="71" t="str">
+        <v>思想： 看学号为1到n的学生是否坐在了0到n-1的位置上 对于一个长度为n的数组，它的索引范围为[0,n-1],缺失的第一个正数一定在[1,n+1]的范围内，所以对于一个学号为nums[i]的学生，他应该坐在nums[i-1]位置;</v>
+      </c>
+      <c r="M21" s="71"/>
+    </row>
+    <row r="22" ht="45.79999923706055" customHeight="1">
       <c r="A22" s="28" t="str">
         <v>矩阵</v>
       </c>
-      <c r="B22" s="93" t="str">
+      <c r="B22" s="103" t="str">
         <v>标记置零</v>
       </c>
       <c r="C22" s="34" t="n">
@@ -1308,7 +1336,7 @@
       <c r="D22" s="34" t="n">
         <v>73</v>
       </c>
-      <c r="E22" s="67" t="str">
+      <c r="E22" s="72" t="str">
         <v>73. 矩阵置零</v>
       </c>
       <c r="F22" s="45" t="str">
@@ -1319,19 +1347,23 @@
       <c r="I22" s="56" t="str">
         <v>leetcode.cn/problems/set-matrix-zeroes/</v>
       </c>
-      <c r="J22" s="68"/>
-      <c r="K22" s="70" t="n">
+      <c r="J22" s="73" t="str">
+        <v>×</v>
+      </c>
+      <c r="K22" s="74" t="n">
         <f>LEN(J22)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J22,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
-      </c>
-      <c r="L22" s="66" t="str">
-        <v>用首行首列作为标记数组记录含0的行列，再二次遍历置零；注意首行首列本身要先处理</v>
-      </c>
-      <c r="M22" s="66"/>
+        <v>1</v>
+      </c>
+      <c r="L22" s="71" t="str">
+        <v>用首行首列作为标记数组记录含0的行列，再二次遍历置零；注意首行首列本身要先处理;倒序就是为了防止 matrix[0][0] = 0 在处理第 0 列时提前把 matrix[i][0] 改成 0，进而误伤整行。</v>
+      </c>
+      <c r="M22" s="71" t="str">
+        <v>注意外部循环从1开始</v>
+      </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="28"/>
-      <c r="B23" s="93" t="str">
+      <c r="B23" s="103" t="str">
         <v>边界模拟</v>
       </c>
       <c r="C23" s="34" t="n">
@@ -1340,7 +1372,7 @@
       <c r="D23" s="34" t="n">
         <v>54</v>
       </c>
-      <c r="E23" s="67" t="str">
+      <c r="E23" s="72" t="str">
         <v>54. 螺旋矩阵</v>
       </c>
       <c r="F23" s="45" t="str">
@@ -1351,19 +1383,19 @@
       <c r="I23" s="56" t="str">
         <v>leetcode.cn/problems/spiral-matrix/</v>
       </c>
-      <c r="J23" s="68"/>
-      <c r="K23" s="70" t="n">
+      <c r="J23" s="73"/>
+      <c r="K23" s="74" t="n">
         <f>LEN(J23)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J23,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L23" s="66" t="str">
+      <c r="L23" s="71" t="str">
         <v>按上、右、下、左四条边界循环收缩；防止m*n为奇数时中心元素遗漏</v>
       </c>
-      <c r="M23" s="66"/>
+      <c r="M23" s="71"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="28"/>
-      <c r="B24" s="93" t="str">
+      <c r="B24" s="103" t="str">
         <v>转置与反转</v>
       </c>
       <c r="C24" s="34" t="n">
@@ -1372,7 +1404,7 @@
       <c r="D24" s="34" t="n">
         <v>48</v>
       </c>
-      <c r="E24" s="67" t="str">
+      <c r="E24" s="72" t="str">
         <v>48. 旋转图像</v>
       </c>
       <c r="F24" s="45" t="str">
@@ -1383,19 +1415,19 @@
       <c r="I24" s="56" t="str">
         <v>leetcode.cn/problems/rotate-image/</v>
       </c>
-      <c r="J24" s="68"/>
-      <c r="K24" s="70" t="n">
+      <c r="J24" s="73"/>
+      <c r="K24" s="74" t="n">
         <f>LEN(J24)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J24,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L24" s="66" t="str">
+      <c r="L24" s="71" t="str">
         <v>先转置（沿主对角线），再逐行反转</v>
       </c>
-      <c r="M24" s="66"/>
+      <c r="M24" s="71"/>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="28"/>
-      <c r="B25" s="93" t="str">
+      <c r="B25" s="103" t="str">
         <v>二维有序查找</v>
       </c>
       <c r="C25" s="34" t="n">
@@ -1404,7 +1436,7 @@
       <c r="D25" s="34" t="n">
         <v>240</v>
       </c>
-      <c r="E25" s="67" t="str">
+      <c r="E25" s="72" t="str">
         <v>240. 搜索二维矩阵 II</v>
       </c>
       <c r="F25" s="45" t="str">
@@ -1415,21 +1447,21 @@
       <c r="I25" s="56" t="str">
         <v>https://leetcode.cn/problems/search-a-2d-matrix-ii/</v>
       </c>
-      <c r="J25" s="68"/>
-      <c r="K25" s="70" t="n">
+      <c r="J25" s="73"/>
+      <c r="K25" s="74" t="n">
         <f>LEN(J25)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J25,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L25" s="66" t="str">
+      <c r="L25" s="71" t="str">
         <v>行、列分别有序，从右上角逐行或逐列排除；区别于74题的整体有序条件。</v>
       </c>
-      <c r="M25" s="66"/>
+      <c r="M25" s="71"/>
     </row>
     <row r="26" ht="78" customHeight="1">
       <c r="A26" s="28" t="str">
         <v>链表</v>
       </c>
-      <c r="B26" s="93" t="str">
+      <c r="B26" s="103" t="str">
         <v>相交与环</v>
       </c>
       <c r="C26" s="34" t="n">
@@ -1438,10 +1470,10 @@
       <c r="D26" s="34" t="n">
         <v>160</v>
       </c>
-      <c r="E26" s="67" t="str">
+      <c r="E26" s="72" t="str">
         <v>160. 相交链表</v>
       </c>
-      <c r="F26" s="76" t="str">
+      <c r="F26" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G26" s="51"/>
@@ -1449,29 +1481,29 @@
       <c r="I26" s="56" t="str">
         <v>leetcode.cn/problems/intersection-of-two-linked-lists/</v>
       </c>
-      <c r="J26" s="68"/>
-      <c r="K26" s="70" t="n">
+      <c r="J26" s="73"/>
+      <c r="K26" s="74" t="n">
         <f>LEN(J26)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J26,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L26" s="66" t="str">
+      <c r="L26" s="71" t="str">
         <v>使用集合而非列表存储节点，因为在后续的环节，使用列表的话时间复杂度为0(n),而对于集合而言，时间复杂度为0(1),对于集合与字典而言，哪怕是值与后继都相同的两个节点，地址不同的话仍然可以存放进去。 if right i…</v>
       </c>
-      <c r="M26" s="66"/>
+      <c r="M26" s="71"/>
     </row>
     <row r="27" ht="50" customHeight="1">
       <c r="A27" s="28"/>
-      <c r="B27" s="93"/>
+      <c r="B27" s="103"/>
       <c r="C27" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D27" s="34" t="n">
         <v>141</v>
       </c>
-      <c r="E27" s="67" t="str">
+      <c r="E27" s="72" t="str">
         <v>141. 环形链表</v>
       </c>
-      <c r="F27" s="76" t="str">
+      <c r="F27" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G27" s="51"/>
@@ -1479,26 +1511,26 @@
       <c r="I27" s="56" t="str">
         <v>leetcode.cn/problems/linked-list-cycle/</v>
       </c>
-      <c r="J27" s="68"/>
-      <c r="K27" s="70" t="n">
+      <c r="J27" s="73"/>
+      <c r="K27" s="74" t="n">
         <f>LEN(J27)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J27,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L27" s="66" t="str">
+      <c r="L27" s="71" t="str">
         <v>佛洛依德判圈算法：使用快慢指针检测是否存在环，快指针每次走两步，慢指针每次走一步，如果最终快指针追上慢指针，证明有环。</v>
       </c>
-      <c r="M27" s="66"/>
+      <c r="M27" s="71"/>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="28"/>
-      <c r="B28" s="93"/>
+      <c r="B28" s="103"/>
       <c r="C28" s="34" t="n">
         <v>3</v>
       </c>
       <c r="D28" s="34" t="n">
         <v>142</v>
       </c>
-      <c r="E28" s="67" t="str">
+      <c r="E28" s="72" t="str">
         <v>142. 环形链表 II</v>
       </c>
       <c r="F28" s="45" t="str">
@@ -1509,19 +1541,19 @@
       <c r="I28" s="56" t="str">
         <v>leetcode.cn/problems/linked-list-cycle-ii/</v>
       </c>
-      <c r="J28" s="68"/>
-      <c r="K28" s="70" t="n">
+      <c r="J28" s="73"/>
+      <c r="K28" s="74" t="n">
         <f>LEN(J28)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J28,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L28" s="66" t="str">
+      <c r="L28" s="71" t="str">
         <v>详见题解</v>
       </c>
-      <c r="M28" s="66"/>
+      <c r="M28" s="71"/>
     </row>
     <row r="29" ht="50" customHeight="1">
       <c r="A29" s="28"/>
-      <c r="B29" s="93" t="str">
+      <c r="B29" s="103" t="str">
         <v>链表反转</v>
       </c>
       <c r="C29" s="34" t="n">
@@ -1530,10 +1562,10 @@
       <c r="D29" s="34" t="n">
         <v>206</v>
       </c>
-      <c r="E29" s="67" t="str">
+      <c r="E29" s="72" t="str">
         <v>206. 反转链表</v>
       </c>
-      <c r="F29" s="76" t="str">
+      <c r="F29" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G29" s="51"/>
@@ -1541,29 +1573,29 @@
       <c r="I29" s="56" t="str">
         <v>leetcode.cn/problems/reverse-linked-list/</v>
       </c>
-      <c r="J29" s="68"/>
-      <c r="K29" s="70" t="n">
+      <c r="J29" s="73"/>
+      <c r="K29" s="74" t="n">
         <f>LEN(J29)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J29,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L29" s="66" t="str">
+      <c r="L29" s="71" t="str">
         <v>迭代：prev/curr指针逐个反转next；递归：先反转后续，再 head.next.next=head</v>
       </c>
-      <c r="M29" s="66"/>
+      <c r="M29" s="71"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="28"/>
-      <c r="B30" s="93"/>
+      <c r="B30" s="103"/>
       <c r="C30" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D30" s="34" t="n">
         <v>25</v>
       </c>
-      <c r="E30" s="67" t="str">
+      <c r="E30" s="72" t="str">
         <v>25. K 个一组翻转链表</v>
       </c>
-      <c r="F30" s="87" t="str">
+      <c r="F30" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G30" s="51"/>
@@ -1571,19 +1603,19 @@
       <c r="I30" s="56" t="str">
         <v>leetcode.cn/problems/reverse-nodes-in-k-group/</v>
       </c>
-      <c r="J30" s="68"/>
-      <c r="K30" s="70" t="n">
+      <c r="J30" s="73"/>
+      <c r="K30" s="74" t="n">
         <f>LEN(J30)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J30,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L30" s="66" t="str">
+      <c r="L30" s="71" t="str">
         <v>注意每个group的pre以及end</v>
       </c>
-      <c r="M30" s="66"/>
+      <c r="M30" s="71"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="28"/>
-      <c r="B31" s="93" t="str">
+      <c r="B31" s="103" t="str">
         <v>快慢指针</v>
       </c>
       <c r="C31" s="34" t="n">
@@ -1592,10 +1624,10 @@
       <c r="D31" s="34" t="n">
         <v>234</v>
       </c>
-      <c r="E31" s="67" t="str">
+      <c r="E31" s="72" t="str">
         <v>234. 回文链表</v>
       </c>
-      <c r="F31" s="76" t="str">
+      <c r="F31" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G31" s="51"/>
@@ -1603,26 +1635,26 @@
       <c r="I31" s="56" t="str">
         <v>leetcode.cn/problems/palindrome-linked-list/</v>
       </c>
-      <c r="J31" s="68"/>
-      <c r="K31" s="70" t="n">
+      <c r="J31" s="73"/>
+      <c r="K31" s="74" t="n">
         <f>LEN(J31)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J31,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L31" s="66" t="str">
+      <c r="L31" s="71" t="str">
         <v>回文链表问题使用快慢指针方法解答最优，其中，慢指针每次走一步，快指针每次走两步。</v>
       </c>
-      <c r="M31" s="66"/>
+      <c r="M31" s="71"/>
     </row>
     <row r="32" ht="45.79999923706055" customHeight="1">
       <c r="A32" s="28"/>
-      <c r="B32" s="93"/>
+      <c r="B32" s="103"/>
       <c r="C32" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D32" s="34" t="n">
         <v>19</v>
       </c>
-      <c r="E32" s="67" t="str">
+      <c r="E32" s="72" t="str">
         <v>19.删除链表的倒数第N个节点</v>
       </c>
       <c r="F32" s="45" t="str">
@@ -1633,19 +1665,19 @@
       <c r="I32" s="56" t="str">
         <v>leetcode.cn/problems/remove-nth-node-from-end-of-list/description/</v>
       </c>
-      <c r="J32" s="68"/>
-      <c r="K32" s="70" t="n">
+      <c r="J32" s="73"/>
+      <c r="K32" s="74" t="n">
         <f>LEN(J32)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J32,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L32" s="66" t="str">
+      <c r="L32" s="71" t="str">
         <v>dummy节点的使用,同时注意当右指针指向最后一个结点的时候,左指针指向的是倒数第(1+n)个节点,也就是说左指针的下一个节点就是倒数第n个节点</v>
       </c>
-      <c r="M32" s="66"/>
+      <c r="M32" s="71"/>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="28"/>
-      <c r="B33" s="93" t="str">
+      <c r="B33" s="103" t="str">
         <v>数位运算</v>
       </c>
       <c r="C33" s="34" t="n">
@@ -1654,7 +1686,7 @@
       <c r="D33" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="E33" s="67" t="str">
+      <c r="E33" s="72" t="str">
         <v>2.两数相加</v>
       </c>
       <c r="F33" s="45" t="str">
@@ -1662,22 +1694,22 @@
       </c>
       <c r="G33" s="51"/>
       <c r="H33" s="51"/>
-      <c r="I33" s="92" t="str">
+      <c r="I33" s="101" t="str">
         <v>leetcode.cn/problems/add-two-numbers/</v>
       </c>
-      <c r="J33" s="68"/>
-      <c r="K33" s="70" t="n">
+      <c r="J33" s="73"/>
+      <c r="K33" s="74" t="n">
         <f>LEN(J33)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J33,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L33" s="66" t="str">
+      <c r="L33" s="71" t="str">
         <v>注意l1.val以及l1.next的赋值方法,里面包含判断,二者紧密结合</v>
       </c>
-      <c r="M33" s="66"/>
+      <c r="M33" s="71"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="28"/>
-      <c r="B34" s="93" t="str">
+      <c r="B34" s="103" t="str">
         <v>节点交换</v>
       </c>
       <c r="C34" s="34" t="n">
@@ -1686,7 +1718,7 @@
       <c r="D34" s="34" t="n">
         <v>24</v>
       </c>
-      <c r="E34" s="67" t="str">
+      <c r="E34" s="72" t="str">
         <v>24. 两两交换链表中的节点</v>
       </c>
       <c r="F34" s="45" t="str">
@@ -1697,19 +1729,19 @@
       <c r="I34" s="56" t="str">
         <v>leetcode.cn/problems/swap-nodes-in-pairs/</v>
       </c>
-      <c r="J34" s="68"/>
-      <c r="K34" s="70" t="n">
+      <c r="J34" s="73"/>
+      <c r="K34" s="74" t="n">
         <f>LEN(J34)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J34,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L34" s="66" t="str">
+      <c r="L34" s="71" t="str">
         <v>需要dummy节点；pre指向每组前驱，两两交换a、b后移动指针</v>
       </c>
-      <c r="M34" s="66"/>
+      <c r="M34" s="71"/>
     </row>
     <row r="35" ht="50" customHeight="1">
       <c r="A35" s="28"/>
-      <c r="B35" s="93" t="str">
+      <c r="B35" s="103" t="str">
         <v>深拷贝</v>
       </c>
       <c r="C35" s="34" t="n">
@@ -1718,7 +1750,7 @@
       <c r="D35" s="34" t="n">
         <v>138</v>
       </c>
-      <c r="E35" s="67" t="str">
+      <c r="E35" s="72" t="str">
         <v>138. 随机链表的复制</v>
       </c>
       <c r="F35" s="45" t="str">
@@ -1729,19 +1761,19 @@
       <c r="I35" s="56" t="str">
         <v>leetcode.cn/problems/copy-list-with-random-pointer/</v>
       </c>
-      <c r="J35" s="68"/>
-      <c r="K35" s="70" t="n">
+      <c r="J35" s="73"/>
+      <c r="K35" s="74" t="n">
         <f>LEN(J35)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J35,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L35" s="66" t="str">
+      <c r="L35" s="71" t="str">
         <v>想要完成链表的深拷贝要求先创建所有的节点，在进行next与random的设置，使用哈希表构建原节点与新节点的映射，在构建新节点的next与random。</v>
       </c>
-      <c r="M35" s="66"/>
+      <c r="M35" s="71"/>
     </row>
     <row r="36" ht="78" customHeight="1">
       <c r="A36" s="28"/>
-      <c r="B36" s="93" t="str">
+      <c r="B36" s="103" t="str">
         <v>归并排序</v>
       </c>
       <c r="C36" s="34" t="n">
@@ -1750,7 +1782,7 @@
       <c r="D36" s="34" t="n">
         <v>148</v>
       </c>
-      <c r="E36" s="67" t="str">
+      <c r="E36" s="72" t="str">
         <v>148. 排序链表</v>
       </c>
       <c r="F36" s="45" t="str">
@@ -1761,19 +1793,19 @@
       <c r="I36" s="56" t="str">
         <v>leetcode.cn/problems/sort-list/</v>
       </c>
-      <c r="J36" s="68"/>
-      <c r="K36" s="70" t="n">
+      <c r="J36" s="73"/>
+      <c r="K36" s="74" t="n">
         <f>LEN(J36)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J36,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L36" s="66" t="str">
+      <c r="L36" s="71" t="str">
         <v>使用快慢指针方法找到中点,然后使用归并排序方法进行排序.</v>
       </c>
-      <c r="M36" s="66"/>
+      <c r="M36" s="71"/>
     </row>
     <row r="37" ht="64" customHeight="1">
       <c r="A37" s="28"/>
-      <c r="B37" s="93" t="str">
+      <c r="B37" s="103" t="str">
         <v>多路归并</v>
       </c>
       <c r="C37" s="34" t="n">
@@ -1782,10 +1814,10 @@
       <c r="D37" s="34" t="n">
         <v>23</v>
       </c>
-      <c r="E37" s="67" t="str">
+      <c r="E37" s="72" t="str">
         <v>23. 合并 K 个升序链表</v>
       </c>
-      <c r="F37" s="87" t="str">
+      <c r="F37" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G37" s="51"/>
@@ -1793,19 +1825,19 @@
       <c r="I37" s="56" t="str">
         <v>leetcode.cn/problems/merge-k-sorted-lists/</v>
       </c>
-      <c r="J37" s="68"/>
-      <c r="K37" s="70" t="n">
+      <c r="J37" s="73"/>
+      <c r="K37" s="74" t="n">
         <f>LEN(J37)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J37,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L37" s="66" t="str">
+      <c r="L37" s="71" t="str">
         <v>此题的思路与链表的归并排序以及两个链表的合并有关，思想是先对链表数组进行递归拆分，然后将单个链表返回并对返回的链表采用链表的合并策略，总体而言相较于链表的直接归并排序要简单一些，因为不需要自己手动将链表拆解。</v>
       </c>
-      <c r="M37" s="66"/>
+      <c r="M37" s="71"/>
     </row>
     <row r="38" ht="36" customHeight="1">
       <c r="A38" s="28"/>
-      <c r="B38" s="93" t="str">
+      <c r="B38" s="103" t="str">
         <v>缓存设计</v>
       </c>
       <c r="C38" s="34" t="n">
@@ -1814,7 +1846,7 @@
       <c r="D38" s="34" t="n">
         <v>146</v>
       </c>
-      <c r="E38" s="67" t="str">
+      <c r="E38" s="72" t="str">
         <v>146.LRU缓存</v>
       </c>
       <c r="F38" s="45" t="str">
@@ -1825,21 +1857,21 @@
       <c r="I38" s="56" t="str">
         <v>leetcode.cn/problems/lru-cache/description/</v>
       </c>
-      <c r="J38" s="68"/>
-      <c r="K38" s="70" t="n">
+      <c r="J38" s="73"/>
+      <c r="K38" s="74" t="n">
         <f>LEN(J38)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J38,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L38" s="66" t="str">
+      <c r="L38" s="71" t="str">
         <v>注意self.hashtable是一个字典,value为双向链表节点,通过.next以及.pre属性构建双向链表</v>
       </c>
-      <c r="M38" s="66"/>
+      <c r="M38" s="71"/>
     </row>
     <row r="39" ht="58.400001525878906" customHeight="1">
       <c r="A39" s="28" t="str">
         <v>二叉树</v>
       </c>
-      <c r="B39" s="93" t="str">
+      <c r="B39" s="103" t="str">
         <v>遍历</v>
       </c>
       <c r="C39" s="34" t="n">
@@ -1848,10 +1880,10 @@
       <c r="D39" s="34" t="n">
         <v>94</v>
       </c>
-      <c r="E39" s="67" t="str">
+      <c r="E39" s="72" t="str">
         <v>94.二叉树中序遍历</v>
       </c>
-      <c r="F39" s="76" t="str">
+      <c r="F39" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G39" s="51"/>
@@ -1859,26 +1891,26 @@
       <c r="I39" s="56" t="str">
         <v>leetcode.cn/problems/binary-tree-inorder-traversal/description/</v>
       </c>
-      <c r="J39" s="68"/>
-      <c r="K39" s="70" t="n">
+      <c r="J39" s="73"/>
+      <c r="K39" s="74" t="n">
         <f>LEN(J39)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J39,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L39" s="66" t="str">
+      <c r="L39" s="71" t="str">
         <v>中序遍历的迭代实现以及前序后序遍历的迭代方法,对于中序方法来说,因为在需要在拆桥(根节点有左子树遍历完)和没有左子树的时候添加,因此可以不使用else,但是对于前序和后序遍历来说,在拆桥的时候不能再次添加,因此需要使用else.</v>
       </c>
-      <c r="M39" s="66"/>
+      <c r="M39" s="71"/>
     </row>
     <row r="40" ht="64" customHeight="1">
       <c r="A40" s="28"/>
-      <c r="B40" s="93"/>
+      <c r="B40" s="103"/>
       <c r="C40" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D40" s="34" t="n">
         <v>102</v>
       </c>
-      <c r="E40" s="67" t="str">
+      <c r="E40" s="72" t="str">
         <v>102. 二叉树的层序遍历</v>
       </c>
       <c r="F40" s="45" t="str">
@@ -1889,19 +1921,19 @@
       <c r="I40" s="56" t="str">
         <v>leetcode.cn/problems/binary-tree-level-order-traversal/</v>
       </c>
-      <c r="J40" s="68"/>
-      <c r="K40" s="70" t="n">
+      <c r="J40" s="73"/>
+      <c r="K40" s="74" t="n">
         <f>LEN(J40)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J40,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L40" s="66" t="str">
+      <c r="L40" s="71" t="str">
         <v>树的层序遍历：树的层序遍历不需要提前知道树的深度 注意：使用 res = [[]nums] 并不能生成一个含有nums个列表的二维列表，应该使用: res = [[] for in range(nums)]</v>
       </c>
-      <c r="M40" s="66"/>
+      <c r="M40" s="71"/>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="28"/>
-      <c r="B41" s="93" t="str">
+      <c r="B41" s="103" t="str">
         <v>深度与结构</v>
       </c>
       <c r="C41" s="34" t="n">
@@ -1910,10 +1942,10 @@
       <c r="D41" s="34" t="n">
         <v>104</v>
       </c>
-      <c r="E41" s="67" t="str">
+      <c r="E41" s="72" t="str">
         <v>104. 二叉树的最大深度</v>
       </c>
-      <c r="F41" s="76" t="str">
+      <c r="F41" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G41" s="51"/>
@@ -1921,29 +1953,29 @@
       <c r="I41" s="56" t="str">
         <v>leetcode.cn/problems/maximum-depth-of-binary-tree/</v>
       </c>
-      <c r="J41" s="68"/>
-      <c r="K41" s="70" t="n">
+      <c r="J41" s="73"/>
+      <c r="K41" s="74" t="n">
         <f>LEN(J41)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J41,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L41" s="66" t="str">
+      <c r="L41" s="71" t="str">
         <v>递归：max(左子树深度, 右子树深度)+1；空节点返回0</v>
       </c>
-      <c r="M41" s="66"/>
+      <c r="M41" s="71"/>
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="28"/>
-      <c r="B42" s="93"/>
+      <c r="B42" s="103"/>
       <c r="C42" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D42" s="34" t="n">
         <v>226</v>
       </c>
-      <c r="E42" s="67" t="str">
+      <c r="E42" s="72" t="str">
         <v>226. 翻转二叉树</v>
       </c>
-      <c r="F42" s="76" t="str">
+      <c r="F42" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G42" s="51"/>
@@ -1951,29 +1983,29 @@
       <c r="I42" s="56" t="str">
         <v>leetcode.cn/problems/invert-binary-tree/</v>
       </c>
-      <c r="J42" s="68"/>
-      <c r="K42" s="70" t="n">
+      <c r="J42" s="73"/>
+      <c r="K42" s="74" t="n">
         <f>LEN(J42)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J42,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L42" s="66" t="str">
+      <c r="L42" s="71" t="str">
         <v>递归交换左右孩子；或层序遍历逐层交换</v>
       </c>
-      <c r="M42" s="66"/>
+      <c r="M42" s="71"/>
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="28"/>
-      <c r="B43" s="93"/>
+      <c r="B43" s="103"/>
       <c r="C43" s="34" t="n">
         <v>3</v>
       </c>
       <c r="D43" s="34" t="n">
         <v>101</v>
       </c>
-      <c r="E43" s="67" t="str">
+      <c r="E43" s="72" t="str">
         <v>101. 对称二叉树</v>
       </c>
-      <c r="F43" s="76" t="str">
+      <c r="F43" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G43" s="51"/>
@@ -1981,19 +2013,19 @@
       <c r="I43" s="56" t="str">
         <v>leetcode.cn/problems/symmetric-tree/</v>
       </c>
-      <c r="J43" s="68"/>
-      <c r="K43" s="70" t="n">
+      <c r="J43" s="73"/>
+      <c r="K43" s="74" t="n">
         <f>LEN(J43)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J43,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L43" s="66" t="str">
+      <c r="L43" s="71" t="str">
         <v>递归：两棵子树镜像对称（左.左==右.右 且 左.右==右.左）;注意需要判断根节点是否为空</v>
       </c>
-      <c r="M43" s="66"/>
+      <c r="M43" s="71"/>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="28"/>
-      <c r="B44" s="93" t="str">
+      <c r="B44" s="103" t="str">
         <v>树的直径（一般树扩展）</v>
       </c>
       <c r="C44" s="34" t="n">
@@ -2002,10 +2034,10 @@
       <c r="D44" s="34" t="n">
         <v>543</v>
       </c>
-      <c r="E44" s="67" t="str">
+      <c r="E44" s="72" t="str">
         <v>543. 二叉树的直径</v>
       </c>
-      <c r="F44" s="76" t="str">
+      <c r="F44" s="80" t="str">
         <v>简单</v>
       </c>
       <c r="G44" s="51"/>
@@ -2013,29 +2045,29 @@
       <c r="I44" s="56" t="str">
         <v>leetcode.cn/problems/diameter-of-binary-tree/</v>
       </c>
-      <c r="J44" s="68"/>
-      <c r="K44" s="70" t="n">
+      <c r="J44" s="73"/>
+      <c r="K44" s="74" t="n">
         <f>LEN(J44)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J44,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L44" s="66" t="str">
+      <c r="L44" s="71" t="str">
         <v>递归求每个节点左右子树深度，全局max(左深+右深)；直径不一定要过根</v>
       </c>
-      <c r="M44" s="66"/>
+      <c r="M44" s="71"/>
     </row>
     <row r="45" ht="78" customHeight="1">
       <c r="A45" s="28"/>
-      <c r="B45" s="93"/>
+      <c r="B45" s="103"/>
       <c r="C45" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D45" s="34" t="n">
         <v>1617</v>
       </c>
-      <c r="E45" s="67" t="str">
+      <c r="E45" s="72" t="str">
         <v>1617. 统计子树中城市之间的最大距离</v>
       </c>
-      <c r="F45" s="87" t="str">
+      <c r="F45" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G45" s="51"/>
@@ -2043,29 +2075,29 @@
       <c r="I45" s="56" t="str">
         <v>leetcode.cn/problems/count-subtrees-with-max-distance-between-cities/</v>
       </c>
-      <c r="J45" s="68"/>
-      <c r="K45" s="70" t="n">
+      <c r="J45" s="73"/>
+      <c r="K45" s="74" t="n">
         <f>LEN(J45)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J45,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L45" s="66" t="str">
+      <c r="L45" s="71" t="str">
         <v>思想：利用枚举子集的思想以及求树的直径的思路，首先创建一个inset数组来对每个节点进行选与不选的操作，当i==n的时候，对前n个节点我们都已经做出了选择，接下来就是判断由这些节点构成的inset是否是一个子集，以及是子…</v>
       </c>
-      <c r="M45" s="66"/>
+      <c r="M45" s="71"/>
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="28"/>
-      <c r="B46" s="93"/>
+      <c r="B46" s="103"/>
       <c r="C46" s="34" t="n">
         <v>3</v>
       </c>
       <c r="D46" s="34" t="n">
         <v>2246</v>
       </c>
-      <c r="E46" s="67" t="str">
+      <c r="E46" s="72" t="str">
         <v>2246. 相邻字符不同的最长路径</v>
       </c>
-      <c r="F46" s="87" t="str">
+      <c r="F46" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G46" s="51"/>
@@ -2073,29 +2105,29 @@
       <c r="I46" s="56" t="str">
         <v>leetcode.cn/problems/longest-path-with-different-adjacent-characters/</v>
       </c>
-      <c r="J46" s="68"/>
-      <c r="K46" s="70" t="n">
+      <c r="J46" s="73"/>
+      <c r="K46" s="74" t="n">
         <f>LEN(J46)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J46,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L46" s="66" t="str">
+      <c r="L46" s="71" t="str">
         <v>树形DP：求经过每个节点的最长路径，仅相邻字符不同才可连边；维护第一大/第二大分支</v>
       </c>
-      <c r="M46" s="66"/>
+      <c r="M46" s="71"/>
     </row>
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="28"/>
-      <c r="B47" s="93"/>
+      <c r="B47" s="103"/>
       <c r="C47" s="34" t="n">
         <v>4</v>
       </c>
       <c r="D47" s="34" t="n">
         <v>2538</v>
       </c>
-      <c r="E47" s="67" t="str">
+      <c r="E47" s="72" t="str">
         <v>2538. 最大价值和与最小价值和的差值</v>
       </c>
-      <c r="F47" s="87" t="str">
+      <c r="F47" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G47" s="51"/>
@@ -2103,19 +2135,19 @@
       <c r="I47" s="56" t="str">
         <v>leetcode.cn/problems/difference-between-maximum-and-minimum-price-sum/</v>
       </c>
-      <c r="J47" s="68"/>
-      <c r="K47" s="70" t="n">
+      <c r="J47" s="73"/>
+      <c r="K47" s="74" t="n">
         <f>LEN(J47)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J47,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L47" s="66" t="str">
+      <c r="L47" s="71" t="str">
         <v>树形DP：维护每个节点向下的路径价值最大和与最小和；答案为max-min，可在节点处拼接两条路径</v>
       </c>
-      <c r="M47" s="66"/>
+      <c r="M47" s="71"/>
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="28"/>
-      <c r="B48" s="93" t="str">
+      <c r="B48" s="103" t="str">
         <v>二叉搜索树</v>
       </c>
       <c r="C48" s="34" t="n">
@@ -2124,7 +2156,7 @@
       <c r="D48" s="34" t="n">
         <v>98</v>
       </c>
-      <c r="E48" s="67" t="str">
+      <c r="E48" s="72" t="str">
         <v>98. 验证二叉搜索树</v>
       </c>
       <c r="F48" s="45" t="str">
@@ -2135,19 +2167,19 @@
       <c r="I48" s="56" t="str">
         <v>leetcode.cn/problems/validate-binary-search-tree/</v>
       </c>
-      <c r="J48" s="68"/>
-      <c r="K48" s="70" t="n">
+      <c r="J48" s="73"/>
+      <c r="K48" s="74" t="n">
         <f>LEN(J48)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J48,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L48" s="66" t="str">
+      <c r="L48" s="71" t="str">
         <v>中序遍历结果严格递增；或递归传递(lower, upper)上下界校验</v>
       </c>
-      <c r="M48" s="66"/>
+      <c r="M48" s="71"/>
     </row>
     <row r="49" ht="64" customHeight="1">
       <c r="A49" s="28"/>
-      <c r="B49" s="93" t="str">
+      <c r="B49" s="103" t="str">
         <v>结构变换</v>
       </c>
       <c r="C49" s="34" t="n">
@@ -2156,7 +2188,7 @@
       <c r="D49" s="34" t="n">
         <v>114</v>
       </c>
-      <c r="E49" s="67" t="str">
+      <c r="E49" s="72" t="str">
         <v>114. 二叉树展开为链表</v>
       </c>
       <c r="F49" s="45" t="str">
@@ -2167,19 +2199,19 @@
       <c r="I49" s="56" t="str">
         <v>leetcode.cn/problems/flatten-binary-tree-to-linked-list/</v>
       </c>
-      <c r="J49" s="68"/>
-      <c r="K49" s="70" t="n">
+      <c r="J49" s="73"/>
+      <c r="K49" s="74" t="n">
         <f>LEN(J49)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J49,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L49" s="66" t="str">
+      <c r="L49" s="71" t="str">
         <v>while 栈非空: 1. 弹出当前节点 = 栈.pop() 2. 连接操作：if pre: pre.right = 当前节点; pre.left = None 3. 入栈操作：先右后左（因为栈是后进先出）</v>
       </c>
-      <c r="M49" s="66"/>
+      <c r="M49" s="71"/>
     </row>
     <row r="50" ht="78" customHeight="1">
       <c r="A50" s="28"/>
-      <c r="B50" s="93" t="str">
+      <c r="B50" s="103" t="str">
         <v>构造二叉树</v>
       </c>
       <c r="C50" s="34" t="n">
@@ -2188,7 +2220,7 @@
       <c r="D50" s="34" t="n">
         <v>105</v>
       </c>
-      <c r="E50" s="67" t="str">
+      <c r="E50" s="72" t="str">
         <v>105. 从前序与中序遍历序列构造二叉树</v>
       </c>
       <c r="F50" s="45" t="str">
@@ -2199,19 +2231,19 @@
       <c r="I50" s="56" t="str">
         <v>leetcode.cn/problems/construct-binary-tree-from-preorder-and-inorder-traversal/</v>
       </c>
-      <c r="J50" s="68"/>
-      <c r="K50" s="70" t="n">
+      <c r="J50" s="73"/>
+      <c r="K50" s="74" t="n">
         <f>LEN(J50)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J50,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L50" s="66" t="str">
+      <c r="L50" s="71" t="str">
         <v>方法一： 这个方法从递归的角度入手，先获取先序遍历中根节点在中序遍历中的索引，然后根据索引确定根节点的左子树和右子树有多少节点，在递归调用构建左右子树 例如，对于这个例子而言，根节点3在中序中对应的位置为1，也就说明了左…</v>
       </c>
-      <c r="M50" s="66"/>
+      <c r="M50" s="71"/>
     </row>
     <row r="51" ht="83.5999984741211" customHeight="1">
       <c r="A51" s="28"/>
-      <c r="B51" s="93" t="str">
+      <c r="B51" s="103" t="str">
         <v>前缀和路径</v>
       </c>
       <c r="C51" s="34" t="n">
@@ -2220,7 +2252,7 @@
       <c r="D51" s="34" t="n">
         <v>437</v>
       </c>
-      <c r="E51" s="67" t="str">
+      <c r="E51" s="72" t="str">
         <v>437. 路径总和 III</v>
       </c>
       <c r="F51" s="45" t="str">
@@ -2231,19 +2263,19 @@
       <c r="I51" s="56" t="str">
         <v>leetcode.cn/problems/path-sum-iii/</v>
       </c>
-      <c r="J51" s="68"/>
-      <c r="K51" s="70" t="n">
+      <c r="J51" s="73"/>
+      <c r="K51" s="74" t="n">
         <f>LEN(J51)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J51,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L51" s="66" t="str">
+      <c r="L51" s="71" t="str">
         <v>采用前缀和的思想，最后在单次函数执行完之前(也就意味着这个节点作为路径终点的所有路径遍历完成)，将字典当中从根节点到当前节点的数量-1，避免对其他分支造成影响。此题可以看作是560.和为k的子数组的升级版本;同时对于使用前缀和的题目来说,有两点需要注意:1.首先设置cnt[0]=1,避免漏算 2.先判断时候有cnt[curr_sum - target_sum]存在,在更新cnt.</v>
       </c>
-      <c r="M51" s="66"/>
+      <c r="M51" s="71"/>
     </row>
     <row r="52" ht="45.79999923706055" customHeight="1">
       <c r="A52" s="28"/>
-      <c r="B52" s="93" t="str">
+      <c r="B52" s="103" t="str">
         <v>最近公共祖先</v>
       </c>
       <c r="C52" s="34" t="n">
@@ -2252,7 +2284,7 @@
       <c r="D52" s="34" t="n">
         <v>236</v>
       </c>
-      <c r="E52" s="67" t="str">
+      <c r="E52" s="72" t="str">
         <v>236. 二叉树的最近公共祖先</v>
       </c>
       <c r="F52" s="45" t="str">
@@ -2263,26 +2295,26 @@
       <c r="I52" s="56" t="str">
         <v>leetcode.cn/problems/lowest-common-ancestor-of-a-binary-tree/</v>
       </c>
-      <c r="J52" s="68"/>
-      <c r="K52" s="70" t="n">
+      <c r="J52" s="73"/>
+      <c r="K52" s="74" t="n">
         <f>LEN(J52)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J52,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L52" s="66" t="str">
+      <c r="L52" s="71" t="str">
         <v>递归：节点为p或q为空都返回自身；左右子树返回值均非空时当前节点即最近公共祖先;否则执行return left if left else right判断</v>
       </c>
-      <c r="M52" s="66"/>
+      <c r="M52" s="71"/>
     </row>
     <row r="53" ht="36" customHeight="1">
       <c r="A53" s="28"/>
-      <c r="B53" s="93"/>
+      <c r="B53" s="103"/>
       <c r="C53" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D53" s="34" t="n">
         <v>235</v>
       </c>
-      <c r="E53" s="67" t="str">
+      <c r="E53" s="72" t="str">
         <v>235. 二叉搜索树的最近公共祖先</v>
       </c>
       <c r="F53" s="45" t="str">
@@ -2293,19 +2325,19 @@
       <c r="I53" s="56" t="str">
         <v>https://leetcode.cn/problems/lowest-common-ancestor-of-a-binary-search-tree/</v>
       </c>
-      <c r="J53" s="68"/>
-      <c r="K53" s="70" t="n">
+      <c r="J53" s="73"/>
+      <c r="K53" s="74" t="n">
         <f>LEN(J53)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J53,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L53" s="66" t="str">
+      <c r="L53" s="71" t="str">
         <v>利用BST有序性：p、q都较小时向左，都较大时向右，否则当前节点为最近公共祖先。</v>
       </c>
-      <c r="M53" s="66"/>
+      <c r="M53" s="71"/>
     </row>
     <row r="54" ht="36" customHeight="1">
       <c r="A54" s="28"/>
-      <c r="B54" s="93" t="str">
+      <c r="B54" s="103" t="str">
         <v>树形DP</v>
       </c>
       <c r="C54" s="34" t="n">
@@ -2314,10 +2346,10 @@
       <c r="D54" s="34" t="n">
         <v>124</v>
       </c>
-      <c r="E54" s="67" t="str">
+      <c r="E54" s="72" t="str">
         <v>124. 二叉树中的最大路径和</v>
       </c>
-      <c r="F54" s="87" t="str">
+      <c r="F54" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G54" s="51"/>
@@ -2325,26 +2357,26 @@
       <c r="I54" s="56" t="str">
         <v>leetcode.cn/problems/binary-tree-maximum-path-sum/</v>
       </c>
-      <c r="J54" s="68"/>
-      <c r="K54" s="70" t="n">
+      <c r="J54" s="73"/>
+      <c r="K54" s="74" t="n">
         <f>LEN(J54)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J54,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L54" s="66" t="str">
+      <c r="L54" s="71" t="str">
         <v>递归返回单边最大路径和 node.val+max(左,右,0)；全局max记录经过当前节点的最大路径和</v>
       </c>
-      <c r="M54" s="66"/>
+      <c r="M54" s="71"/>
     </row>
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="28"/>
-      <c r="B55" s="93"/>
+      <c r="B55" s="103"/>
       <c r="C55" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D55" s="34" t="n">
         <v>337</v>
       </c>
-      <c r="E55" s="67" t="str">
+      <c r="E55" s="72" t="str">
         <v>337. 打家劫舍 III</v>
       </c>
       <c r="F55" s="45" t="str">
@@ -2355,29 +2387,29 @@
       <c r="I55" s="56" t="str">
         <v>leetcode.cn/problems/house-robber-iii/</v>
       </c>
-      <c r="J55" s="68"/>
-      <c r="K55" s="70" t="n">
+      <c r="J55" s="73"/>
+      <c r="K55" s="74" t="n">
         <f>LEN(J55)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J55,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L55" s="66" t="str">
+      <c r="L55" s="71" t="str">
         <v>树形DP：每个节点返回[偷,不偷]；偷则子节点不能偷，不偷取子节点最大值；后序遍历</v>
       </c>
-      <c r="M55" s="66"/>
+      <c r="M55" s="71"/>
     </row>
     <row r="56" ht="78" customHeight="1">
       <c r="A56" s="28"/>
-      <c r="B56" s="93"/>
+      <c r="B56" s="103"/>
       <c r="C56" s="34" t="n">
         <v>3</v>
       </c>
       <c r="D56" s="34" t="n">
         <v>968</v>
       </c>
-      <c r="E56" s="67" t="str">
+      <c r="E56" s="72" t="str">
         <v>968. 监控二叉树</v>
       </c>
-      <c r="F56" s="87" t="str">
+      <c r="F56" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G56" s="51"/>
@@ -2385,21 +2417,21 @@
       <c r="I56" s="56" t="str">
         <v>leetcode.cn/problems/binary-tree-cameras/</v>
       </c>
-      <c r="J56" s="68"/>
-      <c r="K56" s="70" t="n">
+      <c r="J56" s="73"/>
+      <c r="K56" s="74" t="n">
         <f>LEN(J56)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J56,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L56" s="66" t="str">
+      <c r="L56" s="71" t="str">
         <v>此题的核心是针对每个节点，从节点的不同状态入手，分析节点在不同状态下的最小数目或者最小点权和。 分析一下红色节点的处理逻辑，对于红色节点而言，它必须有一个子节点是蓝色节点，而对于黄色节点而言，它的子节点是由红色与蓝色构成…</v>
       </c>
-      <c r="M56" s="66"/>
+      <c r="M56" s="71"/>
     </row>
     <row r="57" ht="78" customHeight="1">
       <c r="A57" s="28" t="str">
         <v>图论</v>
       </c>
-      <c r="B57" s="93" t="str">
+      <c r="B57" s="103" t="str">
         <v>连通块遍历</v>
       </c>
       <c r="C57" s="34" t="n">
@@ -2408,7 +2440,7 @@
       <c r="D57" s="34" t="n">
         <v>200</v>
       </c>
-      <c r="E57" s="67" t="str">
+      <c r="E57" s="72" t="str">
         <v>200. 岛屿数量</v>
       </c>
       <c r="F57" s="45" t="str">
@@ -2419,29 +2451,29 @@
       <c r="I57" s="56" t="str">
         <v>leetcode.cn/problems/number-of-islands/</v>
       </c>
-      <c r="J57" s="68"/>
-      <c r="K57" s="70" t="n">
+      <c r="J57" s="73"/>
+      <c r="K57" s="74" t="n">
         <f>LEN(J57)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J57,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L57" s="66" t="str">
-        <v>方法一：DFS 方法二：BFS 对于坐标而言，用元组存储更加方便 deque（双端队列数据结构）的用法： 基本操作： quene = deque([i,j]): 初始化 d.appendleft() :从左端添加元素 d…</v>
-      </c>
-      <c r="M57" s="66"/>
-    </row>
-    <row r="58" ht="78" customHeight="1">
+      <c r="L57" s="71" t="str">
+        <v>方法一：DFS 方法二：BFS ,对于BFS算法来说,队列的创建放在bfs函数里面,同时队列里面存储的是已经被探索过的岛屿元素,值由1变为0</v>
+      </c>
+      <c r="M57" s="71"/>
+    </row>
+    <row r="58" ht="140" customHeight="1">
       <c r="A58" s="28"/>
-      <c r="B58" s="93" t="str">
-        <v>拓扑排序</v>
+      <c r="B58" s="103" t="str">
+        <v>多源 BFS</v>
       </c>
       <c r="C58" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D58" s="34" t="n">
-        <v>207</v>
-      </c>
-      <c r="E58" s="67" t="str">
-        <v>207. 课程表</v>
+        <v>994</v>
+      </c>
+      <c r="E58" s="72" t="str">
+        <v>994. 腐烂的橘子</v>
       </c>
       <c r="F58" s="45" t="str">
         <v>中等</v>
@@ -2449,31 +2481,33 @@
       <c r="G58" s="51"/>
       <c r="H58" s="51"/>
       <c r="I58" s="56" t="str">
-        <v>leetcode.cn/problems/course-schedule/</v>
-      </c>
-      <c r="J58" s="68"/>
-      <c r="K58" s="70" t="n">
+        <v>leetcode.cn/problems/rotting-oranges/</v>
+      </c>
+      <c r="J58" s="73"/>
+      <c r="K58" s="74" t="n">
         <f>LEN(J58)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J58,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L58" s="66" t="str">
-        <v>在生成初始列表时： list1 = [] n : 这样操作是不对的，空列表重复n次仍为空列表 list1 = [0] n : 正确 list1 = [[] n] : 错误 list1 = [[] for in range…</v>
-      </c>
-      <c r="M58" s="66"/>
-    </row>
-    <row r="59" ht="36" customHeight="1">
+      <c r="L58" s="71" t="str">
+        <v>多源 BFS：先扫描整个网格，将所有腐烂橘子入队并统计新鲜橘子 num；每层处理当前队列长度，对应 1 分钟。新鲜橘子入队时立即标记为腐烂并将 num 减一，避免重复入队。</v>
+      </c>
+      <c r="M58" s="96" t="str">
+        <v>【曾错重点】首次完整遍历网格后、进入 while queue 前，先判断 num == 0（即 if not num），为 0 立即 return 0！不能只在 BFS 内判断：如 [[0]] 没有新鲜橘子，队列也为空，BFS 不执行，会误走末尾 return -1。</v>
+      </c>
+    </row>
+    <row r="59" ht="83.5999984741211" customHeight="1">
       <c r="A59" s="28"/>
-      <c r="B59" s="93" t="str">
-        <v>前缀树</v>
+      <c r="B59" s="103" t="str">
+        <v>拓扑排序</v>
       </c>
       <c r="C59" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D59" s="34" t="n">
-        <v>208</v>
-      </c>
-      <c r="E59" s="67" t="str">
-        <v>208. 实现 Trie (前缀树)</v>
+        <v>207</v>
+      </c>
+      <c r="E59" s="72" t="str">
+        <v>207. 课程表</v>
       </c>
       <c r="F59" s="45" t="str">
         <v>中等</v>
@@ -2481,33 +2515,31 @@
       <c r="G59" s="51"/>
       <c r="H59" s="51"/>
       <c r="I59" s="56" t="str">
-        <v>leetcode.cn/problems/implement-trie-prefix-tree/</v>
-      </c>
-      <c r="J59" s="68"/>
-      <c r="K59" s="70" t="n">
+        <v>leetcode.cn/problems/course-schedule/</v>
+      </c>
+      <c r="J59" s="73"/>
+      <c r="K59" s="74" t="n">
         <f>LEN(J59)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J59,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L59" s="66" t="str">
-        <v>Trie节点含children字典（或26数组）与isEnd标记；插入/搜索/前缀搜索三步走</v>
-      </c>
-      <c r="M59" s="66"/>
-    </row>
-    <row r="60" ht="78" customHeight="1">
-      <c r="A60" s="28" t="str">
-        <v>回溯</v>
-      </c>
-      <c r="B60" s="93" t="str">
-        <v>排列</v>
+      <c r="L59" s="96" t="str">
+        <v>核心在于构建映射表(从parent到child),然后记录每个child的入度,当一个child的入读为0的时候,将其加入到queue队列当中,然后遍历这个节点作为parent的所有子节点,将他们的入读减1,然后判断是否有入度为0的元素,如果有那么将其加入到队列中;同时需要注意记录数量的时候应该是当讲一个元素从队列中弹出时,而不是加入时</v>
+      </c>
+      <c r="M59" s="71"/>
+    </row>
+    <row r="60" ht="45.79999923706055" customHeight="1">
+      <c r="A60" s="28"/>
+      <c r="B60" s="103" t="str">
+        <v>前缀树</v>
       </c>
       <c r="C60" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="34" t="n">
-        <v>46</v>
-      </c>
-      <c r="E60" s="67" t="str">
-        <v>46. 全排列</v>
+        <v>208</v>
+      </c>
+      <c r="E60" s="72" t="str">
+        <v>208. 实现 Trie (前缀树)</v>
       </c>
       <c r="F60" s="45" t="str">
         <v>中等</v>
@@ -2515,31 +2547,33 @@
       <c r="G60" s="51"/>
       <c r="H60" s="51"/>
       <c r="I60" s="56" t="str">
-        <v>leetcode.cn/problems/permutations/</v>
-      </c>
-      <c r="J60" s="68"/>
-      <c r="K60" s="70" t="n">
+        <v>leetcode.cn/problems/implement-trie-prefix-tree/</v>
+      </c>
+      <c r="J60" s="73"/>
+      <c r="K60" s="74" t="n">
         <f>LEN(J60)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J60,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L60" s="66" t="str">
-        <v>（时间复杂度为O(en!)） 在全排列问题当中，始终都是对path这个列表进行处理，如果添加的是path的话只是对原列表的引用，因此当对path进行修改时，也会影响到加入到res当中的列表，正确的做法是添加当前列表的副本…</v>
-      </c>
-      <c r="M60" s="66"/>
+      <c r="L60" s="71" t="str">
+        <v>TrieNode节点的构建很关键,对于该节点的属性hashtable来说,存储以某个字符为前缀的其他Tridnode,然后flag属性用于判断某个字符是不是结尾.</v>
+      </c>
+      <c r="M60" s="71"/>
     </row>
     <row r="61" ht="78" customHeight="1">
-      <c r="A61" s="28"/>
-      <c r="B61" s="93" t="str">
-        <v>子集</v>
+      <c r="A61" s="28" t="str">
+        <v>回溯</v>
+      </c>
+      <c r="B61" s="103" t="str">
+        <v>排列</v>
       </c>
       <c r="C61" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="34" t="n">
-        <v>78</v>
-      </c>
-      <c r="E61" s="67" t="str">
-        <v>78. 子集</v>
+        <v>46</v>
+      </c>
+      <c r="E61" s="72" t="str">
+        <v>46. 全排列</v>
       </c>
       <c r="F61" s="45" t="str">
         <v>中等</v>
@@ -2547,31 +2581,31 @@
       <c r="G61" s="51"/>
       <c r="H61" s="51"/>
       <c r="I61" s="56" t="str">
-        <v>leetcode.cn/problems/subsets/</v>
-      </c>
-      <c r="J61" s="68"/>
-      <c r="K61" s="70" t="n">
+        <v>leetcode.cn/problems/permutations/</v>
+      </c>
+      <c r="J61" s="73"/>
+      <c r="K61" s="74" t="n">
         <f>LEN(J61)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J61,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L61" s="66" t="str">
-        <v>模板一：每个数的选与不选 回溯三问为： 1.当前的操作是什么：是否选择索引值为i的值并将其加入到path中 2.子问题是什么：索引值=i的剩余数的选择问题 3.下一个子问题：索引值=i+1的剩余数的选择问题 模板二：站在…</v>
-      </c>
-      <c r="M61" s="66"/>
+      <c r="L61" s="71" t="str">
+        <v>（时间复杂度为O(en!)） 在全排列问题当中，始终都是对path这个列表进行处理，如果添加的是path的话只是对原列表的引用，因此当对path进行修改时，也会影响到加入到res当中的列表，正确的做法是添加当前列表的副本…</v>
+      </c>
+      <c r="M61" s="71"/>
     </row>
     <row r="62" ht="78" customHeight="1">
       <c r="A62" s="28"/>
-      <c r="B62" s="93" t="str">
-        <v>组合枚举</v>
+      <c r="B62" s="103" t="str">
+        <v>子集</v>
       </c>
       <c r="C62" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D62" s="34" t="n">
-        <v>17</v>
-      </c>
-      <c r="E62" s="67" t="str">
-        <v>17. 电话号码的字母组合</v>
+        <v>78</v>
+      </c>
+      <c r="E62" s="72" t="str">
+        <v>78. 子集</v>
       </c>
       <c r="F62" s="45" t="str">
         <v>中等</v>
@@ -2579,31 +2613,31 @@
       <c r="G62" s="51"/>
       <c r="H62" s="51"/>
       <c r="I62" s="56" t="str">
-        <v>leetcode.cn/problems/letter-combinations-of-a-phone-number/</v>
-      </c>
-      <c r="J62" s="68"/>
-      <c r="K62" s="70" t="n">
+        <v>leetcode.cn/problems/subsets/</v>
+      </c>
+      <c r="J62" s="73"/>
+      <c r="K62" s="74" t="n">
         <f>LEN(J62)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J62,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L62" s="66" t="str">
-        <v>对这个题而言，回溯三问为： 1.当前正在进行的操作是什么：枚举第i个数字的字母（需要使用循环达到枚举的效果） 2.子问题是什么：构建索引值大于等于i的字符串 3.下一个子问题是什么：构建索引值大于等于i+1的字符串</v>
-      </c>
-      <c r="M62" s="66"/>
+      <c r="L62" s="71" t="str">
+        <v>模板一：每个数的选与不选 回溯三问为： 1.当前的操作是什么：是否选择索引值为i的值并将其加入到path中 2.子问题是什么：索引值=i的剩余数的选择问题 3.下一个子问题：索引值=i+1的剩余数的选择问题 模板二：站在…</v>
+      </c>
+      <c r="M62" s="71"/>
     </row>
     <row r="63" ht="78" customHeight="1">
       <c r="A63" s="28"/>
-      <c r="B63" s="93" t="str">
-        <v>组合总和</v>
+      <c r="B63" s="103" t="str">
+        <v>组合枚举</v>
       </c>
       <c r="C63" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D63" s="34" t="n">
-        <v>39</v>
-      </c>
-      <c r="E63" s="67" t="str">
-        <v>39. 组合总和</v>
+        <v>17</v>
+      </c>
+      <c r="E63" s="72" t="str">
+        <v>17. 电话号码的字母组合</v>
       </c>
       <c r="F63" s="45" t="str">
         <v>中等</v>
@@ -2611,29 +2645,31 @@
       <c r="G63" s="51"/>
       <c r="H63" s="51"/>
       <c r="I63" s="56" t="str">
-        <v>leetcode.cn/problems/combination-sum/</v>
-      </c>
-      <c r="J63" s="68"/>
-      <c r="K63" s="70" t="n">
+        <v>leetcode.cn/problems/letter-combinations-of-a-phone-number/</v>
+      </c>
+      <c r="J63" s="73"/>
+      <c r="K63" s="74" t="n">
         <f>LEN(J63)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J63,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L63" s="66" t="str">
-        <v>回溯三问为： 1.当前操作：从大于等于i的索引中选取一个数，索引为j 2.子问题：从大于等于索引i的数组中选数加入到总和中看是否等于target 3.下一个子问题：从大于等于索引j的数组中选数加入到总和中看是否等于tar…</v>
-      </c>
-      <c r="M63" s="66"/>
-    </row>
-    <row r="64" ht="36" customHeight="1">
+      <c r="L63" s="71" t="str">
+        <v>对这个题而言，回溯三问为： 1.当前正在进行的操作是什么：枚举第i个数字的字母（需要使用循环达到枚举的效果） 2.子问题是什么：构建索引值大于等于i的字符串 3.下一个子问题是什么：构建索引值大于等于i+1的字符串</v>
+      </c>
+      <c r="M63" s="71"/>
+    </row>
+    <row r="64" ht="78" customHeight="1">
       <c r="A64" s="28"/>
-      <c r="B64" s="93"/>
+      <c r="B64" s="103" t="str">
+        <v>组合总和</v>
+      </c>
       <c r="C64" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" s="34" t="n">
-        <v>216</v>
-      </c>
-      <c r="E64" s="67" t="str">
-        <v>216. 组合总和 III</v>
+        <v>39</v>
+      </c>
+      <c r="E64" s="72" t="str">
+        <v>39. 组合总和</v>
       </c>
       <c r="F64" s="45" t="str">
         <v>中等</v>
@@ -2641,31 +2677,29 @@
       <c r="G64" s="51"/>
       <c r="H64" s="51"/>
       <c r="I64" s="56" t="str">
-        <v>leetcode.cn/problems/combination-sum-iii/</v>
-      </c>
-      <c r="J64" s="68"/>
-      <c r="K64" s="70" t="n">
+        <v>leetcode.cn/problems/combination-sum/</v>
+      </c>
+      <c r="J64" s="73"/>
+      <c r="K64" s="74" t="n">
         <f>LEN(J64)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J64,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L64" s="66" t="str">
-        <v>回溯组合：从1~9选k个数和为n；可剪枝（剩余个数不足或和超target）</v>
-      </c>
-      <c r="M64" s="66"/>
+      <c r="L64" s="71" t="str">
+        <v>回溯三问为： 1.当前操作：从大于等于i的索引中选取一个数，索引为j 2.子问题：从大于等于索引i的数组中选数加入到总和中看是否等于target 3.下一个子问题：从大于等于索引j的数组中选数加入到总和中看是否等于tar…</v>
+      </c>
+      <c r="M64" s="71"/>
     </row>
     <row r="65" ht="36" customHeight="1">
       <c r="A65" s="28"/>
-      <c r="B65" s="93" t="str">
-        <v>括号构造</v>
-      </c>
+      <c r="B65" s="103"/>
       <c r="C65" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D65" s="34" t="n">
-        <v>22</v>
-      </c>
-      <c r="E65" s="67" t="str">
-        <v>22. 括号生成</v>
+        <v>216</v>
+      </c>
+      <c r="E65" s="72" t="str">
+        <v>216. 组合总和 III</v>
       </c>
       <c r="F65" s="45" t="str">
         <v>中等</v>
@@ -2673,31 +2707,31 @@
       <c r="G65" s="51"/>
       <c r="H65" s="51"/>
       <c r="I65" s="56" t="str">
-        <v>leetcode.cn/problems/generate-parentheses/</v>
-      </c>
-      <c r="J65" s="68"/>
-      <c r="K65" s="70" t="n">
+        <v>leetcode.cn/problems/combination-sum-iii/</v>
+      </c>
+      <c r="J65" s="73"/>
+      <c r="K65" s="74" t="n">
         <f>LEN(J65)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J65,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L65" s="66" t="str">
-        <v>回溯选与不选：左括号数&lt;n才可加'('，右括号数&lt;左括号数才可加')'</v>
-      </c>
-      <c r="M65" s="66"/>
-    </row>
-    <row r="66" ht="64" customHeight="1">
+      <c r="L65" s="71" t="str">
+        <v>回溯组合：从1~9选k个数和为n；可剪枝（剩余个数不足或和超target）</v>
+      </c>
+      <c r="M65" s="71"/>
+    </row>
+    <row r="66" ht="36" customHeight="1">
       <c r="A66" s="28"/>
-      <c r="B66" s="93" t="str">
-        <v>分割</v>
+      <c r="B66" s="103" t="str">
+        <v>括号构造</v>
       </c>
       <c r="C66" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D66" s="34" t="n">
-        <v>131</v>
-      </c>
-      <c r="E66" s="67" t="str">
-        <v>131. 分割回文串</v>
+        <v>22</v>
+      </c>
+      <c r="E66" s="72" t="str">
+        <v>22. 括号生成</v>
       </c>
       <c r="F66" s="45" t="str">
         <v>中等</v>
@@ -2705,97 +2739,97 @@
       <c r="G66" s="51"/>
       <c r="H66" s="51"/>
       <c r="I66" s="56" t="str">
-        <v>leetcode.cn/problems/palindrome-partitioning/</v>
-      </c>
-      <c r="J66" s="68"/>
-      <c r="K66" s="70" t="n">
+        <v>leetcode.cn/problems/generate-parentheses/</v>
+      </c>
+      <c r="J66" s="73"/>
+      <c r="K66" s="74" t="n">
         <f>LEN(J66)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J66,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L66" s="66" t="str">
-        <v>回溯三问为: 1.当前操作：从索引i开始找一个[i,j]的字符串，判断它是不是回文串 2.子问题：从当前索引开始查找回文子串（枚举从i开始的字符串） 3.下一个子问题：从索引j+1开始查找回文串</v>
-      </c>
-      <c r="M66" s="66"/>
-    </row>
-    <row r="67" ht="36" customHeight="1">
+      <c r="L66" s="71" t="str">
+        <v>回溯选与不选：左括号数&lt;n才可加'('，右括号数&lt;左括号数才可加')'</v>
+      </c>
+      <c r="M66" s="71"/>
+    </row>
+    <row r="67" ht="64" customHeight="1">
       <c r="A67" s="28"/>
-      <c r="B67" s="93" t="str">
-        <v>排列与约束</v>
+      <c r="B67" s="103" t="str">
+        <v>分割</v>
       </c>
       <c r="C67" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D67" s="34" t="n">
-        <v>51</v>
-      </c>
-      <c r="E67" s="67" t="str">
-        <v>51. N 皇后</v>
-      </c>
-      <c r="F67" s="87" t="str">
-        <v>困难</v>
+        <v>131</v>
+      </c>
+      <c r="E67" s="72" t="str">
+        <v>131. 分割回文串</v>
+      </c>
+      <c r="F67" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G67" s="51"/>
       <c r="H67" s="51"/>
       <c r="I67" s="56" t="str">
-        <v>leetcode.cn/problems/n-queens/</v>
-      </c>
-      <c r="J67" s="68"/>
-      <c r="K67" s="70" t="n">
+        <v>leetcode.cn/problems/palindrome-partitioning/</v>
+      </c>
+      <c r="J67" s="73"/>
+      <c r="K67" s="74" t="n">
         <f>LEN(J67)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J67,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L67" s="66" t="str">
-        <v>回溯逐行放皇后；用列、主对角线(i-j)、副对角线(i+j)集合剪枝</v>
-      </c>
-      <c r="M67" s="66"/>
+      <c r="L67" s="71" t="str">
+        <v>回溯三问为: 1.当前操作：从索引i开始找一个[i,j]的字符串，判断它是不是回文串 2.子问题：从当前索引开始查找回文子串（枚举从i开始的字符串） 3.下一个子问题：从索引j+1开始查找回文串</v>
+      </c>
+      <c r="M67" s="71"/>
     </row>
     <row r="68" ht="36" customHeight="1">
-      <c r="A68" s="28" t="str">
-        <v>二分查找</v>
-      </c>
-      <c r="B68" s="93" t="str">
-        <v>二维有序查找</v>
+      <c r="A68" s="28"/>
+      <c r="B68" s="103" t="str">
+        <v>排列与约束</v>
       </c>
       <c r="C68" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D68" s="34" t="n">
-        <v>74</v>
-      </c>
-      <c r="E68" s="67" t="str">
-        <v>74. 搜索二维矩阵</v>
-      </c>
-      <c r="F68" s="45" t="str">
-        <v>中等</v>
+        <v>51</v>
+      </c>
+      <c r="E68" s="72" t="str">
+        <v>51. N 皇后</v>
+      </c>
+      <c r="F68" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G68" s="51"/>
       <c r="H68" s="51"/>
       <c r="I68" s="56" t="str">
-        <v>leetcode.cn/problems/search-a-2d-matrix/</v>
-      </c>
-      <c r="J68" s="68"/>
-      <c r="K68" s="70" t="n">
+        <v>leetcode.cn/problems/n-queens/</v>
+      </c>
+      <c r="J68" s="73"/>
+      <c r="K68" s="74" t="n">
         <f>LEN(J68)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J68,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L68" s="66" t="str">
-        <v>把二维矩阵拉成一维即可,mid对应矩阵的位置为[mid//column][mid%column]</v>
-      </c>
-      <c r="M68" s="66"/>
-    </row>
-    <row r="69" ht="50" customHeight="1">
-      <c r="A69" s="28"/>
-      <c r="B69" s="93" t="str">
-        <v>边界查找</v>
+      <c r="L68" s="71" t="str">
+        <v>回溯逐行放皇后；用列、主对角线(i-j)、副对角线(i+j)集合剪枝</v>
+      </c>
+      <c r="M68" s="71"/>
+    </row>
+    <row r="69" ht="36" customHeight="1">
+      <c r="A69" s="28" t="str">
+        <v>二分查找</v>
+      </c>
+      <c r="B69" s="103" t="str">
+        <v>二维有序查找</v>
       </c>
       <c r="C69" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D69" s="34" t="n">
-        <v>34</v>
-      </c>
-      <c r="E69" s="67" t="str">
-        <v>34. 在排序数组中查找元素的第一个和最后一个位置</v>
+        <v>74</v>
+      </c>
+      <c r="E69" s="72" t="str">
+        <v>74. 搜索二维矩阵</v>
       </c>
       <c r="F69" s="45" t="str">
         <v>中等</v>
@@ -2803,31 +2837,31 @@
       <c r="G69" s="51"/>
       <c r="H69" s="51"/>
       <c r="I69" s="56" t="str">
-        <v>leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/</v>
-      </c>
-      <c r="J69" s="68"/>
-      <c r="K69" s="70" t="n">
+        <v>leetcode.cn/problems/search-a-2d-matrix/</v>
+      </c>
+      <c r="J69" s="73"/>
+      <c r="K69" s="74" t="n">
         <f>LEN(J69)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J69,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L69" s="66" t="str">
-        <v>使用lower_bound方法,lower_bound(x)找到第一个大于等于x的值,使用lower_bound(x+1)-1找到最后一个大于等于0的值,然后再判断是不是目标值;额外关注left的取值范围为[0,len(nums)]</v>
-      </c>
-      <c r="M69" s="66"/>
-    </row>
-    <row r="70" ht="45.79999923706055" customHeight="1">
+      <c r="L69" s="71" t="str">
+        <v>把二维矩阵拉成一维即可,mid对应矩阵的位置为[mid//column][mid%column]</v>
+      </c>
+      <c r="M69" s="71"/>
+    </row>
+    <row r="70" ht="50" customHeight="1">
       <c r="A70" s="28"/>
-      <c r="B70" s="93" t="str">
-        <v>旋转数组与局部性质</v>
+      <c r="B70" s="103" t="str">
+        <v>边界查找</v>
       </c>
       <c r="C70" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D70" s="34" t="n">
-        <v>33</v>
-      </c>
-      <c r="E70" s="67" t="str">
-        <v>33. 搜索旋转排序数组</v>
+        <v>34</v>
+      </c>
+      <c r="E70" s="72" t="str">
+        <v>34. 在排序数组中查找元素的第一个和最后一个位置</v>
       </c>
       <c r="F70" s="45" t="str">
         <v>中等</v>
@@ -2835,29 +2869,31 @@
       <c r="G70" s="51"/>
       <c r="H70" s="51"/>
       <c r="I70" s="56" t="str">
-        <v>leetcode.cn/problems/search-in-rotated-sorted-array/</v>
-      </c>
-      <c r="J70" s="68"/>
-      <c r="K70" s="70" t="n">
+        <v>leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/</v>
+      </c>
+      <c r="J70" s="73"/>
+      <c r="K70" s="74" t="n">
         <f>LEN(J70)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J70,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L70" s="66" t="str">
-        <v>红蓝染色/二分：判断mid在target的左侧还是右侧,然后进行染色,最终返回的left就应该是target出现的位置,但同时需要进行判断验证left的合理性.</v>
-      </c>
-      <c r="M70" s="66"/>
-    </row>
-    <row r="71" ht="64" customHeight="1">
+      <c r="L70" s="71" t="str">
+        <v>使用lower_bound方法,lower_bound(x)找到第一个大于等于x的值,使用lower_bound(x+1)-1找到最后一个大于等于0的值,然后再判断是不是目标值;额外关注left的取值范围为[0,len(nums)]</v>
+      </c>
+      <c r="M70" s="71"/>
+    </row>
+    <row r="71" ht="45.79999923706055" customHeight="1">
       <c r="A71" s="28"/>
-      <c r="B71" s="93"/>
+      <c r="B71" s="103" t="str">
+        <v>旋转数组与局部性质</v>
+      </c>
       <c r="C71" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D71" s="34" t="n">
-        <v>153</v>
-      </c>
-      <c r="E71" s="67" t="str">
-        <v>153. 寻找旋转排序数组中的最小值</v>
+        <v>33</v>
+      </c>
+      <c r="E71" s="72" t="str">
+        <v>33. 搜索旋转排序数组</v>
       </c>
       <c r="F71" s="45" t="str">
         <v>中等</v>
@@ -2865,29 +2901,29 @@
       <c r="G71" s="51"/>
       <c r="H71" s="51"/>
       <c r="I71" s="56" t="str">
-        <v>leetcode.cn/problems/find-minimum-in-rotated-sorted-array/</v>
-      </c>
-      <c r="J71" s="68"/>
-      <c r="K71" s="70" t="n">
+        <v>leetcode.cn/problems/search-in-rotated-sorted-array/</v>
+      </c>
+      <c r="J71" s="73"/>
+      <c r="K71" s="74" t="n">
         <f>LEN(J71)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J71,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L71" s="66" t="str">
-        <v>旋转数组左半部分的元素一定大于右半部分，令中间值与末尾值进行比较，如果中间值大于end，意味着中间值及其左侧的值都在最小值的左侧，染成红色，否则为蓝色，蓝色代表着最小值及其右侧。</v>
-      </c>
-      <c r="M71" s="66"/>
-    </row>
-    <row r="72" ht="36" customHeight="1">
+      <c r="L71" s="71" t="str">
+        <v>红蓝染色/二分：判断mid在target的左侧还是右侧,然后进行染色,最终返回的left就应该是target出现的位置,但同时需要进行判断验证left的合理性.</v>
+      </c>
+      <c r="M71" s="71"/>
+    </row>
+    <row r="72" ht="64" customHeight="1">
       <c r="A72" s="28"/>
-      <c r="B72" s="93"/>
+      <c r="B72" s="103"/>
       <c r="C72" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D72" s="34" t="n">
-        <v>162</v>
-      </c>
-      <c r="E72" s="67" t="str">
-        <v>162. 寻找峰值</v>
+        <v>153</v>
+      </c>
+      <c r="E72" s="72" t="str">
+        <v>153. 寻找旋转排序数组中的最小值</v>
       </c>
       <c r="F72" s="45" t="str">
         <v>中等</v>
@@ -2895,97 +2931,95 @@
       <c r="G72" s="51"/>
       <c r="H72" s="51"/>
       <c r="I72" s="56" t="str">
-        <v>leetcode.cn/problems/find-peak-element/</v>
-      </c>
-      <c r="J72" s="68"/>
-      <c r="K72" s="70" t="n">
+        <v>leetcode.cn/problems/find-minimum-in-rotated-sorted-array/</v>
+      </c>
+      <c r="J72" s="73"/>
+      <c r="K72" s="74" t="n">
         <f>LEN(J72)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J72,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L72" s="66" t="str">
-        <v>红蓝染色：nums[mid]&lt;nums[mid+1] 说明峰在右侧，否则峰在左侧</v>
-      </c>
-      <c r="M72" s="66"/>
-    </row>
-    <row r="73" ht="45.79999923706055" customHeight="1">
+      <c r="L72" s="71" t="str">
+        <v>旋转数组左半部分的元素一定大于右半部分，令中间值与末尾值进行比较，如果中间值大于end，意味着中间值及其左侧的值都在最小值的左侧，染成红色，否则为蓝色，蓝色代表着最小值及其右侧。</v>
+      </c>
+      <c r="M72" s="71"/>
+    </row>
+    <row r="73" ht="36" customHeight="1">
       <c r="A73" s="28"/>
-      <c r="B73" s="93" t="str">
-        <v>中位数划分</v>
-      </c>
+      <c r="B73" s="103"/>
       <c r="C73" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D73" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="E73" s="67" t="str">
-        <v>4. 寻找两个正序数组的中位数</v>
-      </c>
-      <c r="F73" s="87" t="str">
-        <v>困难</v>
+        <v>162</v>
+      </c>
+      <c r="E73" s="72" t="str">
+        <v>162. 寻找峰值</v>
+      </c>
+      <c r="F73" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G73" s="51"/>
       <c r="H73" s="51"/>
       <c r="I73" s="56" t="str">
-        <v>leetcode.cn/problems/median-of-two-sorted-arrays/</v>
-      </c>
-      <c r="J73" s="68"/>
-      <c r="K73" s="70" t="n">
+        <v>leetcode.cn/problems/find-peak-element/</v>
+      </c>
+      <c r="J73" s="73"/>
+      <c r="K73" s="74" t="n">
         <f>LEN(J73)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J73,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L73" s="66" t="str">
-        <v>二分排除：在较短数组上二分划分，保证左半最大&lt;右半最小；注意奇偶长度中位数处理;对于左侧来说,存在a[i]&lt;=b[j+1],右侧则是a[i]&gt;b[j+1</v>
-      </c>
-      <c r="M73" s="66"/>
-    </row>
-    <row r="74" ht="36" customHeight="1">
-      <c r="A74" s="28" t="str">
-        <v>栈</v>
-      </c>
-      <c r="B74" s="93" t="str">
-        <v>辅助栈</v>
+      <c r="L73" s="71" t="str">
+        <v>红蓝染色：nums[mid]&lt;nums[mid+1] 说明峰在右侧，否则峰在左侧</v>
+      </c>
+      <c r="M73" s="71"/>
+    </row>
+    <row r="74" ht="45.79999923706055" customHeight="1">
+      <c r="A74" s="28"/>
+      <c r="B74" s="103" t="str">
+        <v>中位数划分</v>
       </c>
       <c r="C74" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D74" s="34" t="n">
-        <v>155</v>
-      </c>
-      <c r="E74" s="67" t="str">
-        <v>155. 最小栈</v>
-      </c>
-      <c r="F74" s="45" t="str">
-        <v>中等</v>
+        <v>4</v>
+      </c>
+      <c r="E74" s="72" t="str">
+        <v>4. 寻找两个正序数组的中位数</v>
+      </c>
+      <c r="F74" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G74" s="51"/>
       <c r="H74" s="51"/>
       <c r="I74" s="56" t="str">
-        <v>leetcode.cn/problems/min-stack/</v>
-      </c>
-      <c r="J74" s="68"/>
-      <c r="K74" s="70" t="n">
+        <v>leetcode.cn/problems/median-of-two-sorted-arrays/</v>
+      </c>
+      <c r="J74" s="73"/>
+      <c r="K74" s="74" t="n">
         <f>LEN(J74)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J74,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L74" s="66" t="str">
-        <v>辅助栈同步压入当前最小值；或每个元素存(值, 当前最小值)</v>
-      </c>
-      <c r="M74" s="66"/>
-    </row>
-    <row r="75" ht="78" customHeight="1">
-      <c r="A75" s="28"/>
-      <c r="B75" s="93" t="str">
-        <v>嵌套解析</v>
+      <c r="L74" s="71" t="str">
+        <v>二分排除：在较短数组上二分划分，保证左半最大&lt;右半最小；注意奇偶长度中位数处理;对于左侧来说,存在a[i]&lt;=b[j+1],右侧则是a[i]&gt;b[j+1</v>
+      </c>
+      <c r="M74" s="71"/>
+    </row>
+    <row r="75" ht="36" customHeight="1">
+      <c r="A75" s="28" t="str">
+        <v>栈</v>
+      </c>
+      <c r="B75" s="103" t="str">
+        <v>辅助栈</v>
       </c>
       <c r="C75" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D75" s="34" t="n">
-        <v>394</v>
-      </c>
-      <c r="E75" s="67" t="str">
-        <v>394. 字符串解码</v>
+        <v>155</v>
+      </c>
+      <c r="E75" s="72" t="str">
+        <v>155. 最小栈</v>
       </c>
       <c r="F75" s="45" t="str">
         <v>中等</v>
@@ -2993,31 +3027,31 @@
       <c r="G75" s="51"/>
       <c r="H75" s="51"/>
       <c r="I75" s="56" t="str">
-        <v>leetcode.cn/problems/decode-string/</v>
-      </c>
-      <c r="J75" s="68"/>
-      <c r="K75" s="70" t="n">
+        <v>leetcode.cn/problems/min-stack/</v>
+      </c>
+      <c r="J75" s="73"/>
+      <c r="K75" s="74" t="n">
         <f>LEN(J75)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J75,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L75" s="66" t="str">
-        <v>此题的巧妙之处在于使用currsum与currstr来存储会遇到的数字与字符，而不是直接将其加入到栈中，正确的做法是当需要二者入栈的时候，处理到新的字符串（即遇到[时）再将其入栈。 char.isdigit()用来判断一…</v>
-      </c>
-      <c r="M75" s="66"/>
+      <c r="L75" s="71" t="str">
+        <v>辅助栈同步压入当前最小值；或每个元素存(值, 当前最小值)</v>
+      </c>
+      <c r="M75" s="71"/>
     </row>
     <row r="76" ht="78" customHeight="1">
       <c r="A76" s="28"/>
-      <c r="B76" s="93" t="str">
-        <v>单调栈</v>
+      <c r="B76" s="103" t="str">
+        <v>嵌套解析</v>
       </c>
       <c r="C76" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D76" s="34" t="n">
-        <v>739</v>
-      </c>
-      <c r="E76" s="67" t="str">
-        <v>739. 每日温度</v>
+        <v>394</v>
+      </c>
+      <c r="E76" s="72" t="str">
+        <v>394. 字符串解码</v>
       </c>
       <c r="F76" s="45" t="str">
         <v>中等</v>
@@ -3025,221 +3059,221 @@
       <c r="G76" s="51"/>
       <c r="H76" s="51"/>
       <c r="I76" s="56" t="str">
-        <v>leetcode.cn/problems/daily-temperatures/</v>
-      </c>
-      <c r="J76" s="68"/>
-      <c r="K76" s="70" t="n">
+        <v>leetcode.cn/problems/decode-string/</v>
+      </c>
+      <c r="J76" s="73"/>
+      <c r="K76" s="74" t="n">
         <f>LEN(J76)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J76,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L76" s="66" t="str">
-        <v>上一个更大更小是通过单调栈的属性判断出来的，下一个更大更小是通过while循环中的比较判断出来的 判断单调栈是递增还是递减就看在什么情况下会弹栈就行 此题的求解要特别留意数组中每个元素的索引值的作用，用索引值相减来得到天…</v>
-      </c>
-      <c r="M76" s="66"/>
-    </row>
-    <row r="77" ht="36" customHeight="1">
+      <c r="L76" s="71" t="str">
+        <v>此题的巧妙之处在于使用currsum与currstr来存储会遇到的数字与字符，而不是直接将其加入到栈中，正确的做法是当需要二者入栈的时候，处理到新的字符串（即遇到[时）再将其入栈。 char.isdigit()用来判断一…</v>
+      </c>
+      <c r="M76" s="71"/>
+    </row>
+    <row r="77" ht="78" customHeight="1">
       <c r="A77" s="28"/>
-      <c r="B77" s="93"/>
+      <c r="B77" s="103" t="str">
+        <v>单调栈</v>
+      </c>
       <c r="C77" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D77" s="34" t="n">
-        <v>84</v>
-      </c>
-      <c r="E77" s="67" t="str">
-        <v>84. 柱状图中最大的矩形</v>
-      </c>
-      <c r="F77" s="87" t="str">
-        <v>困难</v>
+        <v>739</v>
+      </c>
+      <c r="E77" s="72" t="str">
+        <v>739. 每日温度</v>
+      </c>
+      <c r="F77" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G77" s="51"/>
       <c r="H77" s="51"/>
       <c r="I77" s="56" t="str">
-        <v>leetcode.cn/problems/largest-rectangle-in-histogram/</v>
-      </c>
-      <c r="J77" s="68"/>
-      <c r="K77" s="70" t="n">
+        <v>leetcode.cn/problems/daily-temperatures/</v>
+      </c>
+      <c r="J77" s="73"/>
+      <c r="K77" s="74" t="n">
         <f>LEN(J77)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J77,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L77" s="66" t="str">
-        <v>思想：枚举每个高度，找到它左右两边最小的值 记住两个-1操作</v>
-      </c>
-      <c r="M77" s="66"/>
+      <c r="L77" s="71" t="str">
+        <v>上一个更大更小是通过单调栈的属性判断出来的，下一个更大更小是通过while循环中的比较判断出来的 判断单调栈是递增还是递减就看在什么情况下会弹栈就行 此题的求解要特别留意数组中每个元素的索引值的作用，用索引值相减来得到天…</v>
+      </c>
+      <c r="M77" s="71"/>
     </row>
     <row r="78" ht="36" customHeight="1">
-      <c r="A78" s="28" t="str">
-        <v>堆</v>
-      </c>
-      <c r="B78" s="93" t="str">
-        <v>第K大与快速选择</v>
-      </c>
+      <c r="A78" s="28"/>
+      <c r="B78" s="103"/>
       <c r="C78" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D78" s="34" t="n">
-        <v>215</v>
-      </c>
-      <c r="E78" s="67" t="str">
-        <v>215. 数组中的第 K 个最大元素</v>
-      </c>
-      <c r="F78" s="45" t="str">
-        <v>中等</v>
+        <v>84</v>
+      </c>
+      <c r="E78" s="72" t="str">
+        <v>84. 柱状图中最大的矩形</v>
+      </c>
+      <c r="F78" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G78" s="51"/>
       <c r="H78" s="51"/>
       <c r="I78" s="56" t="str">
-        <v>leetcode.cn/problems/kth-largest-element-in-an-array/</v>
-      </c>
-      <c r="J78" s="68"/>
-      <c r="K78" s="70" t="n">
+        <v>leetcode.cn/problems/largest-rectangle-in-histogram/</v>
+      </c>
+      <c r="J78" s="73"/>
+      <c r="K78" s="74" t="n">
         <f>LEN(J78)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J78,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L78" s="66" t="str">
-        <v>快速选择partition（随机pivot）期望O(n)；或维护大小为k的小顶堆</v>
-      </c>
-      <c r="M78" s="66"/>
-    </row>
-    <row r="79" ht="78" customHeight="1">
-      <c r="A79" s="28"/>
-      <c r="B79" s="93" t="str">
-        <v>对顶堆</v>
+      <c r="L78" s="71" t="str">
+        <v>思想：枚举每个高度，找到它左右两边最小的值 记住两个-1操作</v>
+      </c>
+      <c r="M78" s="71"/>
+    </row>
+    <row r="79" ht="36" customHeight="1">
+      <c r="A79" s="28" t="str">
+        <v>堆</v>
+      </c>
+      <c r="B79" s="103" t="str">
+        <v>第K大与快速选择</v>
       </c>
       <c r="C79" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D79" s="34" t="n">
-        <v>295</v>
-      </c>
-      <c r="E79" s="67" t="str">
-        <v>295. 数据流的中位数</v>
-      </c>
-      <c r="F79" s="87" t="str">
-        <v>困难</v>
+        <v>215</v>
+      </c>
+      <c r="E79" s="72" t="str">
+        <v>215. 数组中的第 K 个最大元素</v>
+      </c>
+      <c r="F79" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G79" s="51"/>
       <c r="H79" s="51"/>
       <c r="I79" s="56" t="str">
-        <v>leetcode.cn/problems/find-median-from-data-stream/</v>
-      </c>
-      <c r="J79" s="68"/>
-      <c r="K79" s="70" t="n">
+        <v>leetcode.cn/problems/kth-largest-element-in-an-array/</v>
+      </c>
+      <c r="J79" s="73"/>
+      <c r="K79" s="74" t="n">
         <f>LEN(J79)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J79,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L79" s="66" t="str">
-        <v>此题的思路时使用最大堆与最小堆存储数据，但因为python只有最小堆，因此采用存储相反数的形式来实现最大堆，取出时记得将数取反即可。 当左右堆大小相等的时候，不要直接向左堆中加入数据，应该先加入到右堆中，然后取出新的右堆…</v>
-      </c>
-      <c r="M79" s="66"/>
-    </row>
-    <row r="80" ht="36" customHeight="1">
-      <c r="A80" s="28" t="str">
-        <v>贪心算法</v>
-      </c>
-      <c r="B80" s="93" t="str">
-        <v>股票买卖（状态机DP扩展）</v>
+      <c r="L79" s="71" t="str">
+        <v>快速选择partition（随机pivot）期望O(n)；或维护大小为k的小顶堆</v>
+      </c>
+      <c r="M79" s="71"/>
+    </row>
+    <row r="80" ht="78" customHeight="1">
+      <c r="A80" s="28"/>
+      <c r="B80" s="103" t="str">
+        <v>对顶堆</v>
       </c>
       <c r="C80" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D80" s="34" t="n">
-        <v>122</v>
-      </c>
-      <c r="E80" s="67" t="str">
-        <v>122. 买卖股票的最佳时机 II</v>
-      </c>
-      <c r="F80" s="45" t="str">
-        <v>中等</v>
+        <v>295</v>
+      </c>
+      <c r="E80" s="72" t="str">
+        <v>295. 数据流的中位数</v>
+      </c>
+      <c r="F80" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G80" s="51"/>
       <c r="H80" s="51"/>
       <c r="I80" s="56" t="str">
-        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/</v>
-      </c>
-      <c r="J80" s="68"/>
-      <c r="K80" s="70" t="n">
+        <v>leetcode.cn/problems/find-median-from-data-stream/</v>
+      </c>
+      <c r="J80" s="73"/>
+      <c r="K80" s="74" t="n">
         <f>LEN(J80)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J80,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L80" s="66" t="str">
-        <v>状态机DP：dp[i][0]不持有、dp[i][1]持有；不限制交易次数，答案=dp[n-1][0]</v>
-      </c>
-      <c r="M80" s="66"/>
+      <c r="L80" s="71" t="str">
+        <v>此题的思路时使用最大堆与最小堆存储数据，但因为python只有最小堆，因此采用存储相反数的形式来实现最大堆，取出时记得将数取反即可。 当左右堆大小相等的时候，不要直接向左堆中加入数据，应该先加入到右堆中，然后取出新的右堆…</v>
+      </c>
+      <c r="M80" s="71"/>
     </row>
     <row r="81" ht="36" customHeight="1">
-      <c r="A81" s="28"/>
-      <c r="B81" s="93"/>
+      <c r="A81" s="28" t="str">
+        <v>贪心算法</v>
+      </c>
+      <c r="B81" s="103" t="str">
+        <v>股票买卖（状态机DP扩展）</v>
+      </c>
       <c r="C81" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D81" s="34" t="n">
-        <v>188</v>
-      </c>
-      <c r="E81" s="67" t="str">
-        <v>188. 买卖股票的最佳时机 IV</v>
-      </c>
-      <c r="F81" s="87" t="str">
-        <v>困难</v>
+        <v>122</v>
+      </c>
+      <c r="E81" s="72" t="str">
+        <v>122. 买卖股票的最佳时机 II</v>
+      </c>
+      <c r="F81" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G81" s="51"/>
       <c r="H81" s="51"/>
       <c r="I81" s="56" t="str">
-        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/</v>
-      </c>
-      <c r="J81" s="68"/>
-      <c r="K81" s="70" t="n">
+        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/</v>
+      </c>
+      <c r="J81" s="73"/>
+      <c r="K81" s="74" t="n">
         <f>LEN(J81)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J81,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L81" s="66" t="str">
-        <v>至多k笔：dp[i][j][0/1]，j为已交易次数；j&lt;0不合法，需k+2维空间</v>
-      </c>
-      <c r="M81" s="66"/>
+      <c r="L81" s="71" t="str">
+        <v>状态机DP：dp[i][0]不持有、dp[i][1]持有；不限制交易次数，答案=dp[n-1][0]</v>
+      </c>
+      <c r="M81" s="71"/>
     </row>
     <row r="82" ht="36" customHeight="1">
       <c r="A82" s="28"/>
-      <c r="B82" s="93"/>
+      <c r="B82" s="103"/>
       <c r="C82" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D82" s="34" t="n">
-        <v>309</v>
-      </c>
-      <c r="E82" s="67" t="str">
-        <v>309. 买卖股票的最佳时机含冷冻期</v>
-      </c>
-      <c r="F82" s="45" t="str">
-        <v>中等</v>
+        <v>188</v>
+      </c>
+      <c r="E82" s="72" t="str">
+        <v>188. 买卖股票的最佳时机 IV</v>
+      </c>
+      <c r="F82" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G82" s="51"/>
       <c r="H82" s="51"/>
       <c r="I82" s="56" t="str">
-        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/</v>
-      </c>
-      <c r="J82" s="68"/>
-      <c r="K82" s="70" t="n">
+        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/</v>
+      </c>
+      <c r="J82" s="73"/>
+      <c r="K82" s="74" t="n">
         <f>LEN(J82)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J82,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L82" s="66" t="str">
-        <v>含冷冻期：买入只能从两天前(f2)转移；f0卖出/f1持有/f2冷冻 滚动更新</v>
-      </c>
-      <c r="M82" s="66"/>
+      <c r="L82" s="71" t="str">
+        <v>至多k笔：dp[i][j][0/1]，j为已交易次数；j&lt;0不合法，需k+2维空间</v>
+      </c>
+      <c r="M82" s="71"/>
     </row>
     <row r="83" ht="36" customHeight="1">
       <c r="A83" s="28"/>
-      <c r="B83" s="93" t="str">
-        <v>覆盖范围</v>
-      </c>
+      <c r="B83" s="103"/>
       <c r="C83" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D83" s="34" t="n">
-        <v>55</v>
-      </c>
-      <c r="E83" s="67" t="str">
-        <v>55. 跳跃游戏</v>
+        <v>309</v>
+      </c>
+      <c r="E83" s="72" t="str">
+        <v>309. 买卖股票的最佳时机含冷冻期</v>
       </c>
       <c r="F83" s="45" t="str">
         <v>中等</v>
@@ -3247,29 +3281,31 @@
       <c r="G83" s="51"/>
       <c r="H83" s="51"/>
       <c r="I83" s="56" t="str">
-        <v>leetcode.cn/problems/jump-game/</v>
-      </c>
-      <c r="J83" s="68"/>
-      <c r="K83" s="70" t="n">
+        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/</v>
+      </c>
+      <c r="J83" s="73"/>
+      <c r="K83" s="74" t="n">
         <f>LEN(J83)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J83,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L83" s="66" t="str">
-        <v>贪心：维护能到达的最远位置reach，遍历时更新；reach&gt;=n-1即成功</v>
-      </c>
-      <c r="M83" s="66"/>
+      <c r="L83" s="71" t="str">
+        <v>含冷冻期：买入只能从两天前(f2)转移；f0卖出/f1持有/f2冷冻 滚动更新</v>
+      </c>
+      <c r="M83" s="71"/>
     </row>
     <row r="84" ht="36" customHeight="1">
       <c r="A84" s="28"/>
-      <c r="B84" s="93"/>
+      <c r="B84" s="103" t="str">
+        <v>覆盖范围</v>
+      </c>
       <c r="C84" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D84" s="34" t="n">
-        <v>45</v>
-      </c>
-      <c r="E84" s="67" t="str">
-        <v>45. 跳跃游戏 II</v>
+        <v>55</v>
+      </c>
+      <c r="E84" s="72" t="str">
+        <v>55. 跳跃游戏</v>
       </c>
       <c r="F84" s="45" t="str">
         <v>中等</v>
@@ -3277,33 +3313,29 @@
       <c r="G84" s="51"/>
       <c r="H84" s="51"/>
       <c r="I84" s="56" t="str">
-        <v>leetcode.cn/problems/jump-game-ii/</v>
-      </c>
-      <c r="J84" s="68"/>
-      <c r="K84" s="70" t="n">
+        <v>leetcode.cn/problems/jump-game/</v>
+      </c>
+      <c r="J84" s="73"/>
+      <c r="K84" s="74" t="n">
         <f>LEN(J84)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J84,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L84" s="66" t="str">
-        <v>条件:从头走到尾 最小子序列:走过的步数最少，涉及到的元素的个数最少，也即最小子序列</v>
-      </c>
-      <c r="M84" s="66"/>
-    </row>
-    <row r="85" ht="64" customHeight="1">
-      <c r="A85" s="28" t="str">
-        <v>动态规划</v>
-      </c>
-      <c r="B85" s="93" t="str">
-        <v>计数递推</v>
-      </c>
+      <c r="L84" s="71" t="str">
+        <v>贪心：维护能到达的最远位置reach，遍历时更新；reach&gt;=n-1即成功</v>
+      </c>
+      <c r="M84" s="71"/>
+    </row>
+    <row r="85" ht="36" customHeight="1">
+      <c r="A85" s="28"/>
+      <c r="B85" s="103"/>
       <c r="C85" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D85" s="34" t="n">
-        <v>2266</v>
-      </c>
-      <c r="E85" s="67" t="str">
-        <v>2266. 统计打字方案数</v>
+        <v>45</v>
+      </c>
+      <c r="E85" s="72" t="str">
+        <v>45. 跳跃游戏 II</v>
       </c>
       <c r="F85" s="45" t="str">
         <v>中等</v>
@@ -3311,31 +3343,33 @@
       <c r="G85" s="51"/>
       <c r="H85" s="51"/>
       <c r="I85" s="56" t="str">
-        <v>leetcode.cn/problems/count-number-of-texts/</v>
-      </c>
-      <c r="J85" s="68"/>
-      <c r="K85" s="70" t="n">
+        <v>leetcode.cn/problems/jump-game-ii/</v>
+      </c>
+      <c r="J85" s="73"/>
+      <c r="K85" s="74" t="n">
         <f>LEN(J85)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J85,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L85" s="66" t="str">
-        <v>组合计数+DP：连续相同数字分组，每组按键方案满足dp[i]=dp[i-1]+dp[i-2]+dp[i-3]+(4字母键再加dp[i-4])；结果取模1e9+7</v>
-      </c>
-      <c r="M85" s="66"/>
-    </row>
-    <row r="86" ht="78" customHeight="1">
-      <c r="A86" s="28"/>
-      <c r="B86" s="93" t="str">
-        <v>线性递推</v>
+      <c r="L85" s="71" t="str">
+        <v>条件:从头走到尾 最小子序列:走过的步数最少，涉及到的元素的个数最少，也即最小子序列</v>
+      </c>
+      <c r="M85" s="71"/>
+    </row>
+    <row r="86" ht="64" customHeight="1">
+      <c r="A86" s="28" t="str">
+        <v>动态规划</v>
+      </c>
+      <c r="B86" s="103" t="str">
+        <v>计数递推</v>
       </c>
       <c r="C86" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D86" s="34" t="n">
-        <v>198</v>
-      </c>
-      <c r="E86" s="67" t="str">
-        <v>198. 打家劫舍</v>
+        <v>2266</v>
+      </c>
+      <c r="E86" s="72" t="str">
+        <v>2266. 统计打字方案数</v>
       </c>
       <c r="F86" s="45" t="str">
         <v>中等</v>
@@ -3343,31 +3377,31 @@
       <c r="G86" s="51"/>
       <c r="H86" s="51"/>
       <c r="I86" s="56" t="str">
-        <v>leetcode.cn/problems/house-robber/</v>
-      </c>
-      <c r="J86" s="68"/>
-      <c r="K86" s="70" t="n">
+        <v>leetcode.cn/problems/count-number-of-texts/</v>
+      </c>
+      <c r="J86" s="73"/>
+      <c r="K86" s="74" t="n">
         <f>LEN(J86)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J86,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L86" s="66" t="str">
-        <v>使用动态规划的方法，而对于偷前i个房子的问题，它的最大值为偷取前i-1个房子与偷取前i-2个房子加上当前房子的价格的最大值，因此实际上只需使用两个变量记录i-1与i-2的值，不需要使用一个列表来完整记录每个索引的最大值</v>
-      </c>
-      <c r="M86" s="66"/>
-    </row>
-    <row r="87" ht="50" customHeight="1">
+      <c r="L86" s="71" t="str">
+        <v>组合计数+DP：连续相同数字分组，每组按键方案满足dp[i]=dp[i-1]+dp[i-2]+dp[i-3]+(4字母键再加dp[i-4])；结果取模1e9+7</v>
+      </c>
+      <c r="M86" s="71"/>
+    </row>
+    <row r="87" ht="78" customHeight="1">
       <c r="A87" s="28"/>
-      <c r="B87" s="93" t="str">
-        <v>背包</v>
+      <c r="B87" s="103" t="str">
+        <v>线性递推</v>
       </c>
       <c r="C87" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D87" s="34" t="n">
-        <v>322</v>
-      </c>
-      <c r="E87" s="67" t="str">
-        <v>322. 零钱兑换</v>
+        <v>198</v>
+      </c>
+      <c r="E87" s="72" t="str">
+        <v>198. 打家劫舍</v>
       </c>
       <c r="F87" s="45" t="str">
         <v>中等</v>
@@ -3375,29 +3409,31 @@
       <c r="G87" s="51"/>
       <c r="H87" s="51"/>
       <c r="I87" s="56" t="str">
-        <v>leetcode.cn/problems/coin-change/</v>
-      </c>
-      <c r="J87" s="68"/>
-      <c r="K87" s="70" t="n">
+        <v>leetcode.cn/problems/house-robber/</v>
+      </c>
+      <c r="J87" s="73"/>
+      <c r="K87" s="74" t="n">
         <f>LEN(J87)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J87,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L87" s="66" t="str">
-        <v>完全背包：f[i]=min(f[i], f[i-coin]+1)；f初始化为inf、f[0]=0，返回时判断是否可达</v>
-      </c>
-      <c r="M87" s="66"/>
-    </row>
-    <row r="88" ht="36" customHeight="1">
+      <c r="L87" s="71" t="str">
+        <v>使用动态规划的方法，而对于偷前i个房子的问题，它的最大值为偷取前i-1个房子与偷取前i-2个房子加上当前房子的价格的最大值，因此实际上只需使用两个变量记录i-1与i-2的值，不需要使用一个列表来完整记录每个索引的最大值</v>
+      </c>
+      <c r="M87" s="71"/>
+    </row>
+    <row r="88" ht="50" customHeight="1">
       <c r="A88" s="28"/>
-      <c r="B88" s="93"/>
+      <c r="B88" s="103" t="str">
+        <v>背包</v>
+      </c>
       <c r="C88" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D88" s="34" t="n">
-        <v>494</v>
-      </c>
-      <c r="E88" s="67" t="str">
-        <v>494. 目标和</v>
+        <v>322</v>
+      </c>
+      <c r="E88" s="72" t="str">
+        <v>322. 零钱兑换</v>
       </c>
       <c r="F88" s="45" t="str">
         <v>中等</v>
@@ -3405,31 +3441,29 @@
       <c r="G88" s="51"/>
       <c r="H88" s="51"/>
       <c r="I88" s="56" t="str">
-        <v>leetcode.cn/problems/target-sum/</v>
-      </c>
-      <c r="J88" s="68"/>
-      <c r="K88" s="70" t="n">
+        <v>leetcode.cn/problems/coin-change/</v>
+      </c>
+      <c r="J88" s="73"/>
+      <c r="K88" s="74" t="n">
         <f>LEN(J88)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J88,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L88" s="66" t="str">
-        <v>01背包：target += sum(nums)，求恰好等于target的方案数（每个数选或不选）</v>
-      </c>
-      <c r="M88" s="66"/>
+      <c r="L88" s="71" t="str">
+        <v>完全背包：f[i]=min(f[i], f[i-coin]+1)；f初始化为inf、f[0]=0，返回时判断是否可达</v>
+      </c>
+      <c r="M88" s="71"/>
     </row>
     <row r="89" ht="36" customHeight="1">
       <c r="A89" s="28"/>
-      <c r="B89" s="93" t="str">
-        <v>字符串划分</v>
-      </c>
+      <c r="B89" s="103"/>
       <c r="C89" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D89" s="34" t="n">
-        <v>139</v>
-      </c>
-      <c r="E89" s="67" t="str">
-        <v>139. 单词拆分</v>
+        <v>494</v>
+      </c>
+      <c r="E89" s="72" t="str">
+        <v>494. 目标和</v>
       </c>
       <c r="F89" s="45" t="str">
         <v>中等</v>
@@ -3437,31 +3471,31 @@
       <c r="G89" s="51"/>
       <c r="H89" s="51"/>
       <c r="I89" s="56" t="str">
-        <v>leetcode.cn/problems/word-break/</v>
-      </c>
-      <c r="J89" s="68"/>
-      <c r="K89" s="70" t="n">
+        <v>leetcode.cn/problems/target-sum/</v>
+      </c>
+      <c r="J89" s="73"/>
+      <c r="K89" s="74" t="n">
         <f>LEN(J89)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J89,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L89" s="66" t="str">
-        <v>f数组代表着索引i之前的字符串能否被拆分，因此只需考虑f[n]是否为True即可。</v>
-      </c>
-      <c r="M89" s="66"/>
-    </row>
-    <row r="90" ht="50" customHeight="1">
+      <c r="L89" s="71" t="str">
+        <v>01背包：target += sum(nums)，求恰好等于target的方案数（每个数选或不选）</v>
+      </c>
+      <c r="M89" s="71"/>
+    </row>
+    <row r="90" ht="36" customHeight="1">
       <c r="A90" s="28"/>
-      <c r="B90" s="93" t="str">
-        <v>递增子序列</v>
+      <c r="B90" s="103" t="str">
+        <v>字符串划分</v>
       </c>
       <c r="C90" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D90" s="34" t="n">
-        <v>300</v>
-      </c>
-      <c r="E90" s="67" t="str">
-        <v>300. 最长递增子序列</v>
+        <v>139</v>
+      </c>
+      <c r="E90" s="72" t="str">
+        <v>139. 单词拆分</v>
       </c>
       <c r="F90" s="45" t="str">
         <v>中等</v>
@@ -3469,249 +3503,251 @@
       <c r="G90" s="51"/>
       <c r="H90" s="51"/>
       <c r="I90" s="56" t="str">
-        <v>leetcode.cn/problems/longest-increasing-subsequence/</v>
-      </c>
-      <c r="J90" s="68"/>
-      <c r="K90" s="70" t="n">
+        <v>leetcode.cn/problems/word-break/</v>
+      </c>
+      <c r="J90" s="73"/>
+      <c r="K90" s="74" t="n">
         <f>LEN(J90)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J90,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L90" s="66" t="str">
-        <v>方法一：使用子集型回溯的枚举选哪个思路 方法二： 在LS相同的情况下我们只保存末尾元素最小的那个值，因为末尾元素越小，后续LS的长度才有可能越大</v>
-      </c>
-      <c r="M90" s="66"/>
+      <c r="L90" s="71" t="str">
+        <v>f数组代表着索引i之前的字符串能否被拆分，因此只需考虑f[n]是否为True即可。</v>
+      </c>
+      <c r="M90" s="71"/>
     </row>
     <row r="91" ht="50" customHeight="1">
       <c r="A91" s="28"/>
-      <c r="B91" s="93"/>
+      <c r="B91" s="103" t="str">
+        <v>递增子序列</v>
+      </c>
       <c r="C91" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D91" s="34" t="n">
-        <v>1187</v>
-      </c>
-      <c r="E91" s="67" t="str">
-        <v>1187. 使数组严格递增</v>
-      </c>
-      <c r="F91" s="87" t="str">
-        <v>困难</v>
+        <v>300</v>
+      </c>
+      <c r="E91" s="72" t="str">
+        <v>300. 最长递增子序列</v>
+      </c>
+      <c r="F91" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G91" s="51"/>
       <c r="H91" s="51"/>
       <c r="I91" s="56" t="str">
-        <v>leetcode.cn/problems/make-array-strictly-increasing/</v>
-      </c>
-      <c r="J91" s="68"/>
-      <c r="K91" s="70" t="n">
+        <v>leetcode.cn/problems/longest-increasing-subsequence/</v>
+      </c>
+      <c r="J91" s="73"/>
+      <c r="K91" s="74" t="n">
         <f>LEN(J91)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J91,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L91" s="66" t="str">
-        <v>f[i] 表示：以 a[i] 结尾（且 a[i] 不被替换）时，前 i+1 个元素中最多能保留多少个不替换的元素</v>
-      </c>
-      <c r="M91" s="66"/>
+      <c r="L91" s="71" t="str">
+        <v>方法一：使用子集型回溯的枚举选哪个思路 方法二： 在LS相同的情况下我们只保存末尾元素最小的那个值，因为末尾元素越小，后续LS的长度才有可能越大</v>
+      </c>
+      <c r="M91" s="71"/>
     </row>
     <row r="92" ht="50" customHeight="1">
       <c r="A92" s="28"/>
-      <c r="B92" s="93"/>
+      <c r="B92" s="103"/>
       <c r="C92" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D92" s="34" t="n">
-        <v>1671</v>
-      </c>
-      <c r="E92" s="67" t="str">
-        <v>1671. 得到山形数组的最少删除次数</v>
-      </c>
-      <c r="F92" s="87" t="str">
+        <v>1187</v>
+      </c>
+      <c r="E92" s="72" t="str">
+        <v>1187. 使数组严格递增</v>
+      </c>
+      <c r="F92" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G92" s="51"/>
       <c r="H92" s="51"/>
       <c r="I92" s="56" t="str">
-        <v>leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/</v>
-      </c>
-      <c r="J92" s="68"/>
-      <c r="K92" s="70" t="n">
+        <v>leetcode.cn/problems/make-array-strictly-increasing/</v>
+      </c>
+      <c r="J92" s="73"/>
+      <c r="K92" s="74" t="n">
         <f>LEN(J92)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J92,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L92" s="66" t="str">
-        <v>山形数组：LIS+LDS，枚举峰顶，删除数=n-max(LIS[i]+LDS[i]-1)；峰两侧都需有元素</v>
-      </c>
-      <c r="M92" s="66"/>
+      <c r="L92" s="71" t="str">
+        <v>f[i] 表示：以 a[i] 结尾（且 a[i] 不被替换）时，前 i+1 个元素中最多能保留多少个不替换的元素</v>
+      </c>
+      <c r="M92" s="71"/>
     </row>
     <row r="93" ht="50" customHeight="1">
       <c r="A93" s="28"/>
-      <c r="B93" s="93"/>
+      <c r="B93" s="103"/>
       <c r="C93" s="34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D93" s="34" t="n">
-        <v>1964</v>
-      </c>
-      <c r="E93" s="67" t="str">
-        <v>1964. 找出到每个位置为止的最长合法障碍赛跑路线</v>
-      </c>
-      <c r="F93" s="87" t="str">
+        <v>1671</v>
+      </c>
+      <c r="E93" s="72" t="str">
+        <v>1671. 得到山形数组的最少删除次数</v>
+      </c>
+      <c r="F93" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G93" s="51"/>
       <c r="H93" s="51"/>
       <c r="I93" s="56" t="str">
-        <v>leetcode.cn/problems/longest-obstacle-course-at-each-position/</v>
-      </c>
-      <c r="J93" s="68"/>
-      <c r="K93" s="70" t="n">
+        <v>leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/</v>
+      </c>
+      <c r="J93" s="73"/>
+      <c r="K93" s="74" t="n">
         <f>LEN(J93)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J93,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L93" s="66" t="str">
-        <v>此题与LIS问题的不同之处在于求解的是以某个元素为止的非递减序列的长度，而不是整个数组的最长递增子序列的长度</v>
-      </c>
-      <c r="M93" s="66"/>
-    </row>
-    <row r="94" ht="78" customHeight="1">
+      <c r="L93" s="71" t="str">
+        <v>山形数组：LIS+LDS，枚举峰顶，删除数=n-max(LIS[i]+LDS[i]-1)；峰两侧都需有元素</v>
+      </c>
+      <c r="M93" s="71"/>
+    </row>
+    <row r="94" ht="50" customHeight="1">
       <c r="A94" s="28"/>
-      <c r="B94" s="93" t="str">
-        <v>连续子数组</v>
-      </c>
+      <c r="B94" s="103"/>
       <c r="C94" s="34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D94" s="34" t="n">
-        <v>152</v>
-      </c>
-      <c r="E94" s="67" t="str">
-        <v>152. 乘积最大子数组</v>
-      </c>
-      <c r="F94" s="45" t="str">
-        <v>中等</v>
+        <v>1964</v>
+      </c>
+      <c r="E94" s="72" t="str">
+        <v>1964. 找出到每个位置为止的最长合法障碍赛跑路线</v>
+      </c>
+      <c r="F94" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G94" s="51"/>
       <c r="H94" s="51"/>
       <c r="I94" s="56" t="str">
-        <v>leetcode.cn/problems/maximum-product-subarray/</v>
-      </c>
-      <c r="J94" s="68"/>
-      <c r="K94" s="70" t="n">
+        <v>leetcode.cn/problems/longest-obstacle-course-at-each-position/</v>
+      </c>
+      <c r="J94" s="73"/>
+      <c r="K94" s="74" t="n">
         <f>LEN(J94)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J94,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L94" s="66" t="str">
-        <v>这个问题的思路与求解最大连续子数组和很像，不同的点在于不仅要记录当前最大值，还要记录当前最小值，因为如果当前的数是一个负数的话，那么它乘以小值反而得到一个更大的值，因此在遇到负数的情况下，首先需要将之前的大值与小值互换…</v>
-      </c>
-      <c r="M94" s="66"/>
-    </row>
-    <row r="95" ht="36" customHeight="1">
+      <c r="L94" s="71" t="str">
+        <v>此题与LIS问题的不同之处在于求解的是以某个元素为止的非递减序列的长度，而不是整个数组的最长递增子序列的长度</v>
+      </c>
+      <c r="M94" s="71"/>
+    </row>
+    <row r="95" ht="78" customHeight="1">
       <c r="A95" s="28"/>
-      <c r="B95" s="93" t="str">
-        <v>括号匹配</v>
+      <c r="B95" s="103" t="str">
+        <v>连续子数组</v>
       </c>
       <c r="C95" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D95" s="34" t="n">
-        <v>32</v>
-      </c>
-      <c r="E95" s="67" t="str">
-        <v>32. 最长有效括号</v>
-      </c>
-      <c r="F95" s="87" t="str">
-        <v>困难</v>
+        <v>152</v>
+      </c>
+      <c r="E95" s="72" t="str">
+        <v>152. 乘积最大子数组</v>
+      </c>
+      <c r="F95" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G95" s="51"/>
       <c r="H95" s="51"/>
       <c r="I95" s="56" t="str">
-        <v>leetcode.cn/problems/longest-valid-parentheses/</v>
-      </c>
-      <c r="J95" s="68"/>
-      <c r="K95" s="70" t="n">
+        <v>leetcode.cn/problems/maximum-product-subarray/</v>
+      </c>
+      <c r="J95" s="73"/>
+      <c r="K95" s="74" t="n">
         <f>LEN(J95)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J95,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L95" s="66" t="str">
-        <v>栈存左括号下标，栈底保留最后一个未匹配的')'作哨兵；遇')'弹出并更新ans</v>
-      </c>
-      <c r="M95" s="66"/>
-    </row>
-    <row r="96" ht="78" customHeight="1">
-      <c r="A96" s="28" t="str">
-        <v>多维动态规划</v>
-      </c>
-      <c r="B96" s="93" t="str">
-        <v>多维状态与路径</v>
+      <c r="L95" s="71" t="str">
+        <v>这个问题的思路与求解最大连续子数组和很像，不同的点在于不仅要记录当前最大值，还要记录当前最小值，因为如果当前的数是一个负数的话，那么它乘以小值反而得到一个更大的值，因此在遇到负数的情况下，首先需要将之前的大值与小值互换…</v>
+      </c>
+      <c r="M95" s="71"/>
+    </row>
+    <row r="96" ht="36" customHeight="1">
+      <c r="A96" s="28"/>
+      <c r="B96" s="103" t="str">
+        <v>括号匹配</v>
       </c>
       <c r="C96" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D96" s="34" t="n">
-        <v>1770</v>
-      </c>
-      <c r="E96" s="67" t="str">
-        <v>1770. 执行乘法运算的最大分数</v>
-      </c>
-      <c r="F96" s="87" t="str">
+        <v>32</v>
+      </c>
+      <c r="E96" s="72" t="str">
+        <v>32. 最长有效括号</v>
+      </c>
+      <c r="F96" s="91" t="str">
         <v>困难</v>
       </c>
       <c r="G96" s="51"/>
       <c r="H96" s="51"/>
       <c r="I96" s="56" t="str">
-        <v>leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/</v>
-      </c>
-      <c r="J96" s="68"/>
-      <c r="K96" s="70" t="n">
+        <v>leetcode.cn/problems/longest-valid-parentheses/</v>
+      </c>
+      <c r="J96" s="73"/>
+      <c r="K96" s="74" t="n">
         <f>LEN(J96)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J96,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L96" s="66" t="str">
-        <v>这个题最难的点在于f数组的理解，f[i][j]计算的是剩余操作的最大分数，也就是从第i+1步操作到第m步的最大分数，而j代表着已经选取了j个左侧的值，同时也指明了当前左指针正指向j这个元素，选取的值不论左右，是不会计入到…</v>
-      </c>
-      <c r="M96" s="66"/>
-    </row>
-    <row r="97" ht="36" customHeight="1">
-      <c r="A97" s="28"/>
-      <c r="B97" s="93" t="str">
-        <v>回文与区间DP</v>
+      <c r="L96" s="71" t="str">
+        <v>栈存左括号下标，栈底保留最后一个未匹配的')'作哨兵；遇')'弹出并更新ans</v>
+      </c>
+      <c r="M96" s="71"/>
+    </row>
+    <row r="97" ht="78" customHeight="1">
+      <c r="A97" s="28" t="str">
+        <v>多维动态规划</v>
+      </c>
+      <c r="B97" s="103" t="str">
+        <v>多维状态与路径</v>
       </c>
       <c r="C97" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D97" s="34" t="n">
-        <v>5</v>
-      </c>
-      <c r="E97" s="67" t="str">
-        <v>5. 最长回文子串</v>
-      </c>
-      <c r="F97" s="45" t="str">
-        <v>中等</v>
+        <v>1770</v>
+      </c>
+      <c r="E97" s="72" t="str">
+        <v>1770. 执行乘法运算的最大分数</v>
+      </c>
+      <c r="F97" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G97" s="51"/>
       <c r="H97" s="51"/>
       <c r="I97" s="56" t="str">
-        <v>leetcode.cn/problems/longest-palindromic-substring/</v>
-      </c>
-      <c r="J97" s="68"/>
-      <c r="K97" s="70" t="n">
+        <v>leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/</v>
+      </c>
+      <c r="J97" s="73"/>
+      <c r="K97" s="74" t="n">
         <f>LEN(J97)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J97,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L97" s="66" t="str">
-        <v>使用这种方法通过一次循环就实现了对每个位置的奇回文串与偶回文串的检查</v>
-      </c>
-      <c r="M97" s="66"/>
-    </row>
-    <row r="98" ht="50" customHeight="1">
+      <c r="L97" s="71" t="str">
+        <v>这个题最难的点在于f数组的理解，f[i][j]计算的是剩余操作的最大分数，也就是从第i+1步操作到第m步的最大分数，而j代表着已经选取了j个左侧的值，同时也指明了当前左指针正指向j这个元素，选取的值不论左右，是不会计入到…</v>
+      </c>
+      <c r="M97" s="71"/>
+    </row>
+    <row r="98" ht="36" customHeight="1">
       <c r="A98" s="28"/>
-      <c r="B98" s="93"/>
+      <c r="B98" s="103" t="str">
+        <v>回文与区间DP</v>
+      </c>
       <c r="C98" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D98" s="34" t="n">
-        <v>516</v>
-      </c>
-      <c r="E98" s="67" t="str">
-        <v>516. 最长回文子序列</v>
+        <v>5</v>
+      </c>
+      <c r="E98" s="72" t="str">
+        <v>5. 最长回文子串</v>
       </c>
       <c r="F98" s="45" t="str">
         <v>中等</v>
@@ -3719,29 +3755,29 @@
       <c r="G98" s="51"/>
       <c r="H98" s="51"/>
       <c r="I98" s="56" t="str">
-        <v>leetcode.cn/problems/longest-palindromic-subsequence/</v>
-      </c>
-      <c r="J98" s="68"/>
-      <c r="K98" s="70" t="n">
+        <v>leetcode.cn/problems/longest-palindromic-substring/</v>
+      </c>
+      <c r="J98" s="73"/>
+      <c r="K98" s="74" t="n">
         <f>LEN(J98)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J98,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L98" s="66" t="str">
-        <v>区间DP：f[i][j]表示s[i..j]的最长回文子序列；s[i]==s[j]则+2，否则取max(去左,去右)</v>
-      </c>
-      <c r="M98" s="66"/>
-    </row>
-    <row r="99" ht="78" customHeight="1">
+      <c r="L98" s="71" t="str">
+        <v>使用这种方法通过一次循环就实现了对每个位置的奇回文串与偶回文串的检查</v>
+      </c>
+      <c r="M98" s="71"/>
+    </row>
+    <row r="99" ht="50" customHeight="1">
       <c r="A99" s="28"/>
-      <c r="B99" s="93"/>
+      <c r="B99" s="103"/>
       <c r="C99" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D99" s="34" t="n">
-        <v>647</v>
-      </c>
-      <c r="E99" s="67" t="str">
-        <v>647. 回文子串</v>
+        <v>516</v>
+      </c>
+      <c r="E99" s="72" t="str">
+        <v>516. 最长回文子序列</v>
       </c>
       <c r="F99" s="45" t="str">
         <v>中等</v>
@@ -3749,29 +3785,29 @@
       <c r="G99" s="51"/>
       <c r="H99" s="51"/>
       <c r="I99" s="56" t="str">
-        <v>leetcode.cn/problems/palindromic-substrings/</v>
-      </c>
-      <c r="J99" s="68"/>
-      <c r="K99" s="70" t="n">
+        <v>leetcode.cn/problems/longest-palindromic-subsequence/</v>
+      </c>
+      <c r="J99" s="73"/>
+      <c r="K99" s="74" t="n">
         <f>LEN(J99)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J99,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L99" s="66" t="str">
-        <v>是用动态规划思路解答这个问题的关键在于想清楚dp数组的含义，[i,j]的含义不是从i到j的字符字串中含有多少回文子串，而是判断这个子串是不是一个回文串，因此dp数组有True与False构成，通过统计True的数量来判断…</v>
-      </c>
-      <c r="M99" s="66"/>
-    </row>
-    <row r="100" ht="50" customHeight="1">
+      <c r="L99" s="71" t="str">
+        <v>区间DP：f[i][j]表示s[i..j]的最长回文子序列；s[i]==s[j]则+2，否则取max(去左,去右)</v>
+      </c>
+      <c r="M99" s="71"/>
+    </row>
+    <row r="100" ht="78" customHeight="1">
       <c r="A100" s="28"/>
-      <c r="B100" s="93"/>
+      <c r="B100" s="103"/>
       <c r="C100" s="34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D100" s="34" t="n">
-        <v>1039</v>
-      </c>
-      <c r="E100" s="67" t="str">
-        <v>1039. 多边形三角剖分的最低得分</v>
+        <v>647</v>
+      </c>
+      <c r="E100" s="72" t="str">
+        <v>647. 回文子串</v>
       </c>
       <c r="F100" s="45" t="str">
         <v>中等</v>
@@ -3779,31 +3815,29 @@
       <c r="G100" s="51"/>
       <c r="H100" s="51"/>
       <c r="I100" s="56" t="str">
-        <v>leetcode.cn/problems/minimum-score-triangulation-of-polygon/</v>
-      </c>
-      <c r="J100" s="68"/>
-      <c r="K100" s="70" t="n">
+        <v>leetcode.cn/problems/palindromic-substrings/</v>
+      </c>
+      <c r="J100" s="73"/>
+      <c r="K100" s="74" t="n">
         <f>LEN(J100)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J100,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L100" s="66" t="str">
-        <v>回溯三问： 1.当前操作：在(i，j)的范围内枚举一个数k 2.子问题：求解(i,j)的最低得分 3.下一个子问题：求解(i,k)与(k,j)的最低得分</v>
-      </c>
-      <c r="M100" s="66"/>
+      <c r="L100" s="71" t="str">
+        <v>是用动态规划思路解答这个问题的关键在于想清楚dp数组的含义，[i,j]的含义不是从i到j的字符字串中含有多少回文子串，而是判断这个子串是不是一个回文串，因此dp数组有True与False构成，通过统计True的数量来判断…</v>
+      </c>
+      <c r="M100" s="71"/>
     </row>
     <row r="101" ht="50" customHeight="1">
       <c r="A101" s="28"/>
-      <c r="B101" s="93" t="str">
-        <v>双序列</v>
-      </c>
+      <c r="B101" s="103"/>
       <c r="C101" s="34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D101" s="34" t="n">
-        <v>1143</v>
-      </c>
-      <c r="E101" s="67" t="str">
-        <v>1143. 最长公共子序列</v>
+        <v>1039</v>
+      </c>
+      <c r="E101" s="72" t="str">
+        <v>1039. 多边形三角剖分的最低得分</v>
       </c>
       <c r="F101" s="45" t="str">
         <v>中等</v>
@@ -3811,29 +3845,31 @@
       <c r="G101" s="51"/>
       <c r="H101" s="51"/>
       <c r="I101" s="56" t="str">
-        <v>leetcode.cn/problems/longest-common-subsequence/</v>
-      </c>
-      <c r="J101" s="68"/>
-      <c r="K101" s="70" t="n">
+        <v>leetcode.cn/problems/minimum-score-triangulation-of-polygon/</v>
+      </c>
+      <c r="J101" s="73"/>
+      <c r="K101" s="74" t="n">
         <f>LEN(J101)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J101,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L101" s="66" t="str">
-        <v>二维DP：text1[i]==text2[j]则f[i][j]=f[i-1][j-1]+1，否则取max(f[i-1][j], f[i][j-1])</v>
-      </c>
-      <c r="M101" s="66"/>
-    </row>
-    <row r="102" ht="36" customHeight="1">
+      <c r="L101" s="71" t="str">
+        <v>回溯三问： 1.当前操作：在(i，j)的范围内枚举一个数k 2.子问题：求解(i,j)的最低得分 3.下一个子问题：求解(i,k)与(k,j)的最低得分</v>
+      </c>
+      <c r="M101" s="71"/>
+    </row>
+    <row r="102" ht="50" customHeight="1">
       <c r="A102" s="28"/>
-      <c r="B102" s="93"/>
+      <c r="B102" s="103" t="str">
+        <v>双序列</v>
+      </c>
       <c r="C102" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D102" s="34" t="n">
-        <v>712</v>
-      </c>
-      <c r="E102" s="67" t="str">
-        <v>712. 两个字符串的最小ASCII删除和</v>
+        <v>1143</v>
+      </c>
+      <c r="E102" s="72" t="str">
+        <v>1143. 最长公共子序列</v>
       </c>
       <c r="F102" s="45" t="str">
         <v>中等</v>
@@ -3841,29 +3877,29 @@
       <c r="G102" s="51"/>
       <c r="H102" s="51"/>
       <c r="I102" s="56" t="str">
-        <v>leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/</v>
-      </c>
-      <c r="J102" s="68"/>
-      <c r="K102" s="70" t="n">
+        <v>leetcode.cn/problems/longest-common-subsequence/</v>
+      </c>
+      <c r="J102" s="73"/>
+      <c r="K102" s="74" t="n">
         <f>LEN(J102)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J102,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L102" s="66" t="str">
-        <v>LCS变式：总ASCII和-2×LCS；或直接DP，两字符不同时取删s1[i]或删s2[j]的较小值</v>
-      </c>
-      <c r="M102" s="66"/>
+      <c r="L102" s="71" t="str">
+        <v>二维DP：text1[i]==text2[j]则f[i][j]=f[i-1][j-1]+1，否则取max(f[i-1][j], f[i][j-1])</v>
+      </c>
+      <c r="M102" s="71"/>
     </row>
     <row r="103" ht="36" customHeight="1">
       <c r="A103" s="28"/>
-      <c r="B103" s="93"/>
+      <c r="B103" s="103"/>
       <c r="C103" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D103" s="34" t="n">
-        <v>72</v>
-      </c>
-      <c r="E103" s="67" t="str">
-        <v>72. 编辑距离</v>
+        <v>712</v>
+      </c>
+      <c r="E103" s="72" t="str">
+        <v>712. 两个字符串的最小ASCII删除和</v>
       </c>
       <c r="F103" s="45" t="str">
         <v>中等</v>
@@ -3871,33 +3907,29 @@
       <c r="G103" s="51"/>
       <c r="H103" s="51"/>
       <c r="I103" s="56" t="str">
-        <v>leetcode.cn/problems/edit-distance/</v>
-      </c>
-      <c r="J103" s="68"/>
-      <c r="K103" s="70" t="n">
+        <v>leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/</v>
+      </c>
+      <c r="J103" s="73"/>
+      <c r="K103" s="74" t="n">
         <f>LEN(J103)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J103,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L103" s="66" t="str">
-        <v>DP：f[i][j]编辑距离；末尾字符相同直接继承，不同则取增/删/改三者最小值+1</v>
-      </c>
-      <c r="M103" s="66"/>
+      <c r="L103" s="71" t="str">
+        <v>LCS变式：总ASCII和-2×LCS；或直接DP，两字符不同时取删s1[i]或删s2[j]的较小值</v>
+      </c>
+      <c r="M103" s="71"/>
     </row>
     <row r="104" ht="36" customHeight="1">
-      <c r="A104" s="28" t="str">
-        <v>技巧</v>
-      </c>
-      <c r="B104" s="93" t="str">
-        <v>三路划分</v>
-      </c>
+      <c r="A104" s="28"/>
+      <c r="B104" s="103"/>
       <c r="C104" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D104" s="34" t="n">
-        <v>75</v>
-      </c>
-      <c r="E104" s="67" t="str">
-        <v>75. 颜色分类</v>
+        <v>72</v>
+      </c>
+      <c r="E104" s="72" t="str">
+        <v>72. 编辑距离</v>
       </c>
       <c r="F104" s="45" t="str">
         <v>中等</v>
@@ -3905,31 +3937,33 @@
       <c r="G104" s="51"/>
       <c r="H104" s="51"/>
       <c r="I104" s="56" t="str">
-        <v>leetcode.cn/problems/sort-colors/</v>
-      </c>
-      <c r="J104" s="68"/>
-      <c r="K104" s="70" t="n">
+        <v>leetcode.cn/problems/edit-distance/</v>
+      </c>
+      <c r="J104" s="73"/>
+      <c r="K104" s="74" t="n">
         <f>LEN(J104)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J104,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L104" s="66" t="str">
-        <v>荷兰国旗三指针：[0,zero]全0、[two,n-1]全2、中间为1；partition交换</v>
-      </c>
-      <c r="M104" s="66"/>
-    </row>
-    <row r="105" ht="64" customHeight="1">
-      <c r="A105" s="28"/>
-      <c r="B105" s="93" t="str">
-        <v>排列变换</v>
+      <c r="L104" s="71" t="str">
+        <v>DP：f[i][j]编辑距离；末尾字符相同直接继承，不同则取增/删/改三者最小值+1</v>
+      </c>
+      <c r="M104" s="71"/>
+    </row>
+    <row r="105" ht="36" customHeight="1">
+      <c r="A105" s="28" t="str">
+        <v>技巧</v>
+      </c>
+      <c r="B105" s="103" t="str">
+        <v>三路划分</v>
       </c>
       <c r="C105" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D105" s="34" t="n">
-        <v>31</v>
-      </c>
-      <c r="E105" s="67" t="str">
-        <v>31. 下一个排列</v>
+        <v>75</v>
+      </c>
+      <c r="E105" s="72" t="str">
+        <v>75. 颜色分类</v>
       </c>
       <c r="F105" s="45" t="str">
         <v>中等</v>
@@ -3937,31 +3971,31 @@
       <c r="G105" s="51"/>
       <c r="H105" s="51"/>
       <c r="I105" s="56" t="str">
-        <v>leetcode.cn/problems/next-permutation/</v>
-      </c>
-      <c r="J105" s="68"/>
-      <c r="K105" s="70" t="n">
+        <v>leetcode.cn/problems/sort-colors/</v>
+      </c>
+      <c r="J105" s="73"/>
+      <c r="K105" s="74" t="n">
         <f>LEN(J105)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J105,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L105" s="66" t="str">
-        <v>思路： 1.从右向左，找第一个小于右侧相邻数字的数 x 2.找 x 右边最小的大于 x 的数 y，交换 x 和 y 3.反转 y 右边的数，把右边的数变成最小的排列</v>
-      </c>
-      <c r="M105" s="66"/>
-    </row>
-    <row r="106" ht="78" customHeight="1">
+      <c r="L105" s="71" t="str">
+        <v>荷兰国旗三指针：[0,zero]全0、[two,n-1]全2、中间为1；partition交换</v>
+      </c>
+      <c r="M105" s="71"/>
+    </row>
+    <row r="106" ht="64" customHeight="1">
       <c r="A106" s="28"/>
-      <c r="B106" s="93" t="str">
-        <v>判圈</v>
+      <c r="B106" s="103" t="str">
+        <v>排列变换</v>
       </c>
       <c r="C106" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D106" s="34" t="n">
-        <v>287</v>
-      </c>
-      <c r="E106" s="67" t="str">
-        <v>287. 寻找重复数</v>
+        <v>31</v>
+      </c>
+      <c r="E106" s="72" t="str">
+        <v>31. 下一个排列</v>
       </c>
       <c r="F106" s="45" t="str">
         <v>中等</v>
@@ -3969,17 +4003,49 @@
       <c r="G106" s="51"/>
       <c r="H106" s="51"/>
       <c r="I106" s="56" t="str">
+        <v>leetcode.cn/problems/next-permutation/</v>
+      </c>
+      <c r="J106" s="73"/>
+      <c r="K106" s="74" t="n">
+        <f>LEN(J106)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J106,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L106" s="71" t="str">
+        <v>思路： 1.从右向左，找第一个小于右侧相邻数字的数 x 2.找 x 右边最小的大于 x 的数 y，交换 x 和 y 3.反转 y 右边的数，把右边的数变成最小的排列</v>
+      </c>
+      <c r="M106" s="71"/>
+    </row>
+    <row r="107" ht="78" customHeight="1">
+      <c r="A107" s="28"/>
+      <c r="B107" s="103" t="str">
+        <v>判圈</v>
+      </c>
+      <c r="C107" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" s="34" t="n">
+        <v>287</v>
+      </c>
+      <c r="E107" s="72" t="str">
+        <v>287. 寻找重复数</v>
+      </c>
+      <c r="F107" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G107" s="51"/>
+      <c r="H107" s="51"/>
+      <c r="I107" s="56" t="str">
         <v>leetcode.cn/problems/find-the-duplicate-number/</v>
       </c>
-      <c r="J106" s="68"/>
-      <c r="K106" s="70" t="n">
-        <f>LEN(J106)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J106,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
-      </c>
-      <c r="L106" s="66" t="str">
+      <c r="J107" s="73"/>
+      <c r="K107" s="74" t="n">
+        <f>LEN(J107)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J107,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L107" s="71" t="str">
         <v>这题的关键在于给出一个包含n+1个数字的数组，且数组的取值位于[1,n],可以这么看待问题，把这n+1个数对应的索引看成是n+1个节点，标号从0到n，构建从i到nums[i]的映射，nums[i]的值就代表了i这个节点指…</v>
       </c>
-      <c r="M106" s="66"/>
+      <c r="M107" s="71"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -3993,15 +4059,15 @@
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A26:A38"/>
     <mergeCell ref="A39:A56"/>
-    <mergeCell ref="A57:A59"/>
-    <mergeCell ref="A60:A67"/>
-    <mergeCell ref="A68:A73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="A78:A79"/>
-    <mergeCell ref="A80:A84"/>
-    <mergeCell ref="A85:A95"/>
-    <mergeCell ref="A96:A103"/>
-    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A57:A60"/>
+    <mergeCell ref="A61:A68"/>
+    <mergeCell ref="A69:A74"/>
+    <mergeCell ref="A75:A78"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="A81:A85"/>
+    <mergeCell ref="A86:A96"/>
+    <mergeCell ref="A97:A104"/>
+    <mergeCell ref="A105:A107"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B26:B28"/>
@@ -4012,18 +4078,18 @@
     <mergeCell ref="B44:B47"/>
     <mergeCell ref="B52:B53"/>
     <mergeCell ref="B54:B56"/>
-    <mergeCell ref="B63:B64"/>
-    <mergeCell ref="B70:B72"/>
-    <mergeCell ref="B76:B77"/>
-    <mergeCell ref="B80:B82"/>
-    <mergeCell ref="B83:B84"/>
-    <mergeCell ref="B87:B88"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="B97:B100"/>
-    <mergeCell ref="B101:B103"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="B71:B73"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="B88:B89"/>
+    <mergeCell ref="B91:B94"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="B102:B104"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="custom" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="只填写做题结果" error="请只填写√或×（兼容✓）。每个符号代表做了一次，例如√×√。" promptTitle="追加本次结果" prompt="双击或F2编辑，在末尾追加√或×。例如√×√表示3次；不要覆盖已有记录。" sqref="J4:J106">
+    <dataValidation type="custom" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="只填写做题结果" error="请只填写√或×（兼容✓）。每个符号代表做了一次，例如√×√。" promptTitle="追加本次结果" prompt="双击或F2编辑，在末尾追加√或×。例如√×√表示3次；不要覆盖已有记录。" sqref="J4:J107">
       <formula1>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J4,"√",""),"×",""),"✓",""))=0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4136,104 +4202,106 @@
     <hyperlink ref="I56" display="leetcode.cn/problems/binary-tree-cameras/" r:id="codexHyperlink106"/>
     <hyperlink ref="E57" display="200. 岛屿数量" tooltip="09_图论.ipynb / lc-200" r:id="codexHyperlink107"/>
     <hyperlink ref="I57" display="leetcode.cn/problems/number-of-islands/" r:id="codexHyperlink108"/>
-    <hyperlink ref="E58" display="207. 课程表" tooltip="09_图论.ipynb / lc-207" r:id="codexHyperlink109"/>
-    <hyperlink ref="I58" display="leetcode.cn/problems/course-schedule/" r:id="codexHyperlink110"/>
-    <hyperlink ref="E59" display="208. 实现 Trie (前缀树)" tooltip="09_图论.ipynb / lc-208" r:id="codexHyperlink111"/>
-    <hyperlink ref="I59" display="leetcode.cn/problems/implement-trie-prefix-tree/" r:id="codexHyperlink112"/>
-    <hyperlink ref="E60" display="46. 全排列" tooltip="10_回溯.ipynb / lc-46" r:id="codexHyperlink113"/>
-    <hyperlink ref="I60" display="leetcode.cn/problems/permutations/" r:id="codexHyperlink114"/>
-    <hyperlink ref="E61" display="78. 子集" tooltip="10_回溯.ipynb / lc-78" r:id="codexHyperlink115"/>
-    <hyperlink ref="I61" display="leetcode.cn/problems/subsets/" r:id="codexHyperlink116"/>
-    <hyperlink ref="E62" display="17. 电话号码的字母组合" tooltip="10_回溯.ipynb / lc-17" r:id="codexHyperlink117"/>
-    <hyperlink ref="I62" display="leetcode.cn/problems/letter-combinations-of-a-phone-number/" r:id="codexHyperlink118"/>
-    <hyperlink ref="E63" display="39. 组合总和" tooltip="10_回溯.ipynb / lc-39" r:id="codexHyperlink119"/>
-    <hyperlink ref="I63" display="leetcode.cn/problems/combination-sum/" r:id="codexHyperlink120"/>
-    <hyperlink ref="E64" display="216. 组合总和 III" tooltip="10_回溯.ipynb / lc-216" r:id="codexHyperlink121"/>
-    <hyperlink ref="I64" display="leetcode.cn/problems/combination-sum-iii/" r:id="codexHyperlink122"/>
-    <hyperlink ref="E65" display="22. 括号生成" tooltip="10_回溯.ipynb / lc-22" r:id="codexHyperlink123"/>
-    <hyperlink ref="I65" display="leetcode.cn/problems/generate-parentheses/" r:id="codexHyperlink124"/>
-    <hyperlink ref="E66" display="131. 分割回文串" tooltip="10_回溯.ipynb / lc-131" r:id="codexHyperlink125"/>
-    <hyperlink ref="I66" display="leetcode.cn/problems/palindrome-partitioning/" r:id="codexHyperlink126"/>
-    <hyperlink ref="E67" display="51. N 皇后" tooltip="10_回溯.ipynb / lc-51" r:id="codexHyperlink127"/>
-    <hyperlink ref="I67" display="leetcode.cn/problems/n-queens/" r:id="codexHyperlink128"/>
-    <hyperlink ref="E68" display="74. 搜索二维矩阵" tooltip="11_二分查找.ipynb / lc-74" r:id="codexHyperlink129"/>
-    <hyperlink ref="I68" display="leetcode.cn/problems/search-a-2d-matrix/" r:id="codexHyperlink130"/>
-    <hyperlink ref="E69" display="34. 在排序数组中查找元素的第一个和最后一个位置" tooltip="11_二分查找.ipynb / lc-34" r:id="codexHyperlink131"/>
-    <hyperlink ref="I69" display="leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/" r:id="codexHyperlink132"/>
-    <hyperlink ref="E70" display="33. 搜索旋转排序数组" tooltip="11_二分查找.ipynb / lc-33" r:id="codexHyperlink133"/>
-    <hyperlink ref="I70" display="leetcode.cn/problems/search-in-rotated-sorted-array/" r:id="codexHyperlink134"/>
-    <hyperlink ref="E71" display="153. 寻找旋转排序数组中的最小值" tooltip="11_二分查找.ipynb / lc-153" r:id="codexHyperlink135"/>
-    <hyperlink ref="I71" display="leetcode.cn/problems/find-minimum-in-rotated-sorted-array/" r:id="codexHyperlink136"/>
-    <hyperlink ref="E72" display="162. 寻找峰值" tooltip="11_二分查找.ipynb / lc-162" r:id="codexHyperlink137"/>
-    <hyperlink ref="I72" display="leetcode.cn/problems/find-peak-element/" r:id="codexHyperlink138"/>
-    <hyperlink ref="E73" display="4. 寻找两个正序数组的中位数" tooltip="11_二分查找.ipynb / lc-4" r:id="codexHyperlink139"/>
-    <hyperlink ref="I73" display="leetcode.cn/problems/median-of-two-sorted-arrays/" r:id="codexHyperlink140"/>
-    <hyperlink ref="E74" display="155. 最小栈" tooltip="12_栈.ipynb / lc-155" r:id="codexHyperlink141"/>
-    <hyperlink ref="I74" display="leetcode.cn/problems/min-stack/" r:id="codexHyperlink142"/>
-    <hyperlink ref="E75" display="394. 字符串解码" tooltip="12_栈.ipynb / lc-394" r:id="codexHyperlink143"/>
-    <hyperlink ref="I75" display="leetcode.cn/problems/decode-string/" r:id="codexHyperlink144"/>
-    <hyperlink ref="E76" display="739. 每日温度" tooltip="12_栈.ipynb / lc-739" r:id="codexHyperlink145"/>
-    <hyperlink ref="I76" display="leetcode.cn/problems/daily-temperatures/" r:id="codexHyperlink146"/>
-    <hyperlink ref="E77" display="84. 柱状图中最大的矩形" tooltip="12_栈.ipynb / lc-84" r:id="codexHyperlink147"/>
-    <hyperlink ref="I77" display="leetcode.cn/problems/largest-rectangle-in-histogram/" r:id="codexHyperlink148"/>
-    <hyperlink ref="E78" display="215. 数组中的第 K 个最大元素" tooltip="13_堆.ipynb / lc-215" r:id="codexHyperlink149"/>
-    <hyperlink ref="I78" display="leetcode.cn/problems/kth-largest-element-in-an-array/" r:id="codexHyperlink150"/>
-    <hyperlink ref="E79" display="295. 数据流的中位数" tooltip="13_堆.ipynb / lc-295" r:id="codexHyperlink151"/>
-    <hyperlink ref="I79" display="leetcode.cn/problems/find-median-from-data-stream/" r:id="codexHyperlink152"/>
-    <hyperlink ref="E80" display="122. 买卖股票的最佳时机 II" tooltip="14_贪心算法.ipynb / lc-122" r:id="codexHyperlink153"/>
-    <hyperlink ref="I80" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/" r:id="codexHyperlink154"/>
-    <hyperlink ref="E81" display="188. 买卖股票的最佳时机 IV" tooltip="14_贪心算法.ipynb / lc-188" r:id="codexHyperlink155"/>
-    <hyperlink ref="I81" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/" r:id="codexHyperlink156"/>
-    <hyperlink ref="E82" display="309. 买卖股票的最佳时机含冷冻期" tooltip="14_贪心算法.ipynb / lc-309" r:id="codexHyperlink157"/>
-    <hyperlink ref="I82" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/" r:id="codexHyperlink158"/>
-    <hyperlink ref="E83" display="55. 跳跃游戏" tooltip="14_贪心算法.ipynb / lc-55" r:id="codexHyperlink159"/>
-    <hyperlink ref="I83" display="leetcode.cn/problems/jump-game/" r:id="codexHyperlink160"/>
-    <hyperlink ref="E84" display="45. 跳跃游戏 II" tooltip="14_贪心算法.ipynb / lc-45" r:id="codexHyperlink161"/>
-    <hyperlink ref="I84" display="leetcode.cn/problems/jump-game-ii/" r:id="codexHyperlink162"/>
-    <hyperlink ref="E85" display="2266. 统计打字方案数" tooltip="15_动态规划.ipynb / lc-2266" r:id="codexHyperlink163"/>
-    <hyperlink ref="I85" display="leetcode.cn/problems/count-number-of-texts/" r:id="codexHyperlink164"/>
-    <hyperlink ref="E86" display="198. 打家劫舍" tooltip="15_动态规划.ipynb / lc-198" r:id="codexHyperlink165"/>
-    <hyperlink ref="I86" display="leetcode.cn/problems/house-robber/" r:id="codexHyperlink166"/>
-    <hyperlink ref="E87" display="322. 零钱兑换" tooltip="15_动态规划.ipynb / lc-322" r:id="codexHyperlink167"/>
-    <hyperlink ref="I87" display="leetcode.cn/problems/coin-change/" r:id="codexHyperlink168"/>
-    <hyperlink ref="E88" display="494. 目标和" tooltip="15_动态规划.ipynb / lc-494" r:id="codexHyperlink169"/>
-    <hyperlink ref="I88" display="leetcode.cn/problems/target-sum/" r:id="codexHyperlink170"/>
-    <hyperlink ref="E89" display="139. 单词拆分" tooltip="15_动态规划.ipynb / lc-139" r:id="codexHyperlink171"/>
-    <hyperlink ref="I89" display="leetcode.cn/problems/word-break/" r:id="codexHyperlink172"/>
-    <hyperlink ref="E90" display="300. 最长递增子序列" tooltip="15_动态规划.ipynb / lc-300" r:id="codexHyperlink173"/>
-    <hyperlink ref="I90" display="leetcode.cn/problems/longest-increasing-subsequence/" r:id="codexHyperlink174"/>
-    <hyperlink ref="E91" display="1187. 使数组严格递增" tooltip="15_动态规划.ipynb / lc-1187" r:id="codexHyperlink175"/>
-    <hyperlink ref="I91" display="leetcode.cn/problems/make-array-strictly-increasing/" r:id="codexHyperlink176"/>
-    <hyperlink ref="E92" display="1671. 得到山形数组的最少删除次数" tooltip="15_动态规划.ipynb / lc-1671" r:id="codexHyperlink177"/>
-    <hyperlink ref="I92" display="leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/" r:id="codexHyperlink178"/>
-    <hyperlink ref="E93" display="1964. 找出到每个位置为止的最长合法障碍赛跑路线" tooltip="15_动态规划.ipynb / lc-1964" r:id="codexHyperlink179"/>
-    <hyperlink ref="I93" display="leetcode.cn/problems/longest-obstacle-course-at-each-position/" r:id="codexHyperlink180"/>
-    <hyperlink ref="E94" display="152. 乘积最大子数组" tooltip="15_动态规划.ipynb / lc-152" r:id="codexHyperlink181"/>
-    <hyperlink ref="I94" display="leetcode.cn/problems/maximum-product-subarray/" r:id="codexHyperlink182"/>
-    <hyperlink ref="E95" display="32. 最长有效括号" tooltip="15_动态规划.ipynb / lc-32" r:id="codexHyperlink183"/>
-    <hyperlink ref="I95" display="leetcode.cn/problems/longest-valid-parentheses/" r:id="codexHyperlink184"/>
-    <hyperlink ref="E96" display="1770. 执行乘法运算的最大分数" tooltip="16_多维动态规划.ipynb / lc-1770" r:id="codexHyperlink185"/>
-    <hyperlink ref="I96" display="leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/" r:id="codexHyperlink186"/>
-    <hyperlink ref="E97" display="5. 最长回文子串" tooltip="16_多维动态规划.ipynb / lc-5" r:id="codexHyperlink187"/>
-    <hyperlink ref="I97" display="leetcode.cn/problems/longest-palindromic-substring/" r:id="codexHyperlink188"/>
-    <hyperlink ref="E98" display="516. 最长回文子序列" tooltip="16_多维动态规划.ipynb / lc-516" r:id="codexHyperlink189"/>
-    <hyperlink ref="I98" display="leetcode.cn/problems/longest-palindromic-subsequence/" r:id="codexHyperlink190"/>
-    <hyperlink ref="E99" display="647. 回文子串" tooltip="16_多维动态规划.ipynb / lc-647" r:id="codexHyperlink191"/>
-    <hyperlink ref="I99" display="leetcode.cn/problems/palindromic-substrings/" r:id="codexHyperlink192"/>
-    <hyperlink ref="E100" display="1039. 多边形三角剖分的最低得分" tooltip="16_多维动态规划.ipynb / lc-1039" r:id="codexHyperlink193"/>
-    <hyperlink ref="I100" display="leetcode.cn/problems/minimum-score-triangulation-of-polygon/" r:id="codexHyperlink194"/>
-    <hyperlink ref="E101" display="1143. 最长公共子序列" tooltip="16_多维动态规划.ipynb / lc-1143" r:id="codexHyperlink195"/>
-    <hyperlink ref="I101" display="leetcode.cn/problems/longest-common-subsequence/" r:id="codexHyperlink196"/>
-    <hyperlink ref="E102" display="712. 两个字符串的最小ASCII删除和" tooltip="16_多维动态规划.ipynb / lc-712" r:id="codexHyperlink197"/>
-    <hyperlink ref="I102" display="leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/" r:id="codexHyperlink198"/>
-    <hyperlink ref="E103" display="72. 编辑距离" tooltip="16_多维动态规划.ipynb / lc-72" r:id="codexHyperlink199"/>
-    <hyperlink ref="I103" display="leetcode.cn/problems/edit-distance/" r:id="codexHyperlink200"/>
-    <hyperlink ref="E104" display="75. 颜色分类" tooltip="17_技巧.ipynb / lc-75" r:id="codexHyperlink201"/>
-    <hyperlink ref="I104" display="leetcode.cn/problems/sort-colors/" r:id="codexHyperlink202"/>
-    <hyperlink ref="E105" display="31. 下一个排列" tooltip="17_技巧.ipynb / lc-31" r:id="codexHyperlink203"/>
-    <hyperlink ref="I105" display="leetcode.cn/problems/next-permutation/" r:id="codexHyperlink204"/>
-    <hyperlink ref="E106" display="287. 寻找重复数" tooltip="17_技巧.ipynb / lc-287" r:id="codexHyperlink205"/>
-    <hyperlink ref="I106" display="leetcode.cn/problems/find-the-duplicate-number/" r:id="codexHyperlink206"/>
+    <hyperlink ref="E58" display="994. 腐烂的橘子" tooltip="09_图论.ipynb / lc-994" r:id="codexHyperlink109"/>
+    <hyperlink ref="I58" display="leetcode.cn/problems/rotting-oranges/" r:id="codexHyperlink110"/>
+    <hyperlink ref="E59" display="207. 课程表" tooltip="09_图论.ipynb / lc-207" r:id="codexHyperlink111"/>
+    <hyperlink ref="I59" display="leetcode.cn/problems/course-schedule/" r:id="codexHyperlink112"/>
+    <hyperlink ref="E60" display="208. 实现 Trie (前缀树)" tooltip="09_图论.ipynb / lc-208" r:id="codexHyperlink113"/>
+    <hyperlink ref="I60" display="leetcode.cn/problems/implement-trie-prefix-tree/" r:id="codexHyperlink114"/>
+    <hyperlink ref="E61" display="46. 全排列" tooltip="10_回溯.ipynb / lc-46" r:id="codexHyperlink115"/>
+    <hyperlink ref="I61" display="leetcode.cn/problems/permutations/" r:id="codexHyperlink116"/>
+    <hyperlink ref="E62" display="78. 子集" tooltip="10_回溯.ipynb / lc-78" r:id="codexHyperlink117"/>
+    <hyperlink ref="I62" display="leetcode.cn/problems/subsets/" r:id="codexHyperlink118"/>
+    <hyperlink ref="E63" display="17. 电话号码的字母组合" tooltip="10_回溯.ipynb / lc-17" r:id="codexHyperlink119"/>
+    <hyperlink ref="I63" display="leetcode.cn/problems/letter-combinations-of-a-phone-number/" r:id="codexHyperlink120"/>
+    <hyperlink ref="E64" display="39. 组合总和" tooltip="10_回溯.ipynb / lc-39" r:id="codexHyperlink121"/>
+    <hyperlink ref="I64" display="leetcode.cn/problems/combination-sum/" r:id="codexHyperlink122"/>
+    <hyperlink ref="E65" display="216. 组合总和 III" tooltip="10_回溯.ipynb / lc-216" r:id="codexHyperlink123"/>
+    <hyperlink ref="I65" display="leetcode.cn/problems/combination-sum-iii/" r:id="codexHyperlink124"/>
+    <hyperlink ref="E66" display="22. 括号生成" tooltip="10_回溯.ipynb / lc-22" r:id="codexHyperlink125"/>
+    <hyperlink ref="I66" display="leetcode.cn/problems/generate-parentheses/" r:id="codexHyperlink126"/>
+    <hyperlink ref="E67" display="131. 分割回文串" tooltip="10_回溯.ipynb / lc-131" r:id="codexHyperlink127"/>
+    <hyperlink ref="I67" display="leetcode.cn/problems/palindrome-partitioning/" r:id="codexHyperlink128"/>
+    <hyperlink ref="E68" display="51. N 皇后" tooltip="10_回溯.ipynb / lc-51" r:id="codexHyperlink129"/>
+    <hyperlink ref="I68" display="leetcode.cn/problems/n-queens/" r:id="codexHyperlink130"/>
+    <hyperlink ref="E69" display="74. 搜索二维矩阵" tooltip="11_二分查找.ipynb / lc-74" r:id="codexHyperlink131"/>
+    <hyperlink ref="I69" display="leetcode.cn/problems/search-a-2d-matrix/" r:id="codexHyperlink132"/>
+    <hyperlink ref="E70" display="34. 在排序数组中查找元素的第一个和最后一个位置" tooltip="11_二分查找.ipynb / lc-34" r:id="codexHyperlink133"/>
+    <hyperlink ref="I70" display="leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/" r:id="codexHyperlink134"/>
+    <hyperlink ref="E71" display="33. 搜索旋转排序数组" tooltip="11_二分查找.ipynb / lc-33" r:id="codexHyperlink135"/>
+    <hyperlink ref="I71" display="leetcode.cn/problems/search-in-rotated-sorted-array/" r:id="codexHyperlink136"/>
+    <hyperlink ref="E72" display="153. 寻找旋转排序数组中的最小值" tooltip="11_二分查找.ipynb / lc-153" r:id="codexHyperlink137"/>
+    <hyperlink ref="I72" display="leetcode.cn/problems/find-minimum-in-rotated-sorted-array/" r:id="codexHyperlink138"/>
+    <hyperlink ref="E73" display="162. 寻找峰值" tooltip="11_二分查找.ipynb / lc-162" r:id="codexHyperlink139"/>
+    <hyperlink ref="I73" display="leetcode.cn/problems/find-peak-element/" r:id="codexHyperlink140"/>
+    <hyperlink ref="E74" display="4. 寻找两个正序数组的中位数" tooltip="11_二分查找.ipynb / lc-4" r:id="codexHyperlink141"/>
+    <hyperlink ref="I74" display="leetcode.cn/problems/median-of-two-sorted-arrays/" r:id="codexHyperlink142"/>
+    <hyperlink ref="E75" display="155. 最小栈" tooltip="12_栈.ipynb / lc-155" r:id="codexHyperlink143"/>
+    <hyperlink ref="I75" display="leetcode.cn/problems/min-stack/" r:id="codexHyperlink144"/>
+    <hyperlink ref="E76" display="394. 字符串解码" tooltip="12_栈.ipynb / lc-394" r:id="codexHyperlink145"/>
+    <hyperlink ref="I76" display="leetcode.cn/problems/decode-string/" r:id="codexHyperlink146"/>
+    <hyperlink ref="E77" display="739. 每日温度" tooltip="12_栈.ipynb / lc-739" r:id="codexHyperlink147"/>
+    <hyperlink ref="I77" display="leetcode.cn/problems/daily-temperatures/" r:id="codexHyperlink148"/>
+    <hyperlink ref="E78" display="84. 柱状图中最大的矩形" tooltip="12_栈.ipynb / lc-84" r:id="codexHyperlink149"/>
+    <hyperlink ref="I78" display="leetcode.cn/problems/largest-rectangle-in-histogram/" r:id="codexHyperlink150"/>
+    <hyperlink ref="E79" display="215. 数组中的第 K 个最大元素" tooltip="13_堆.ipynb / lc-215" r:id="codexHyperlink151"/>
+    <hyperlink ref="I79" display="leetcode.cn/problems/kth-largest-element-in-an-array/" r:id="codexHyperlink152"/>
+    <hyperlink ref="E80" display="295. 数据流的中位数" tooltip="13_堆.ipynb / lc-295" r:id="codexHyperlink153"/>
+    <hyperlink ref="I80" display="leetcode.cn/problems/find-median-from-data-stream/" r:id="codexHyperlink154"/>
+    <hyperlink ref="E81" display="122. 买卖股票的最佳时机 II" tooltip="14_贪心算法.ipynb / lc-122" r:id="codexHyperlink155"/>
+    <hyperlink ref="I81" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/" r:id="codexHyperlink156"/>
+    <hyperlink ref="E82" display="188. 买卖股票的最佳时机 IV" tooltip="14_贪心算法.ipynb / lc-188" r:id="codexHyperlink157"/>
+    <hyperlink ref="I82" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/" r:id="codexHyperlink158"/>
+    <hyperlink ref="E83" display="309. 买卖股票的最佳时机含冷冻期" tooltip="14_贪心算法.ipynb / lc-309" r:id="codexHyperlink159"/>
+    <hyperlink ref="I83" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/" r:id="codexHyperlink160"/>
+    <hyperlink ref="E84" display="55. 跳跃游戏" tooltip="14_贪心算法.ipynb / lc-55" r:id="codexHyperlink161"/>
+    <hyperlink ref="I84" display="leetcode.cn/problems/jump-game/" r:id="codexHyperlink162"/>
+    <hyperlink ref="E85" display="45. 跳跃游戏 II" tooltip="14_贪心算法.ipynb / lc-45" r:id="codexHyperlink163"/>
+    <hyperlink ref="I85" display="leetcode.cn/problems/jump-game-ii/" r:id="codexHyperlink164"/>
+    <hyperlink ref="E86" display="2266. 统计打字方案数" tooltip="15_动态规划.ipynb / lc-2266" r:id="codexHyperlink165"/>
+    <hyperlink ref="I86" display="leetcode.cn/problems/count-number-of-texts/" r:id="codexHyperlink166"/>
+    <hyperlink ref="E87" display="198. 打家劫舍" tooltip="15_动态规划.ipynb / lc-198" r:id="codexHyperlink167"/>
+    <hyperlink ref="I87" display="leetcode.cn/problems/house-robber/" r:id="codexHyperlink168"/>
+    <hyperlink ref="E88" display="322. 零钱兑换" tooltip="15_动态规划.ipynb / lc-322" r:id="codexHyperlink169"/>
+    <hyperlink ref="I88" display="leetcode.cn/problems/coin-change/" r:id="codexHyperlink170"/>
+    <hyperlink ref="E89" display="494. 目标和" tooltip="15_动态规划.ipynb / lc-494" r:id="codexHyperlink171"/>
+    <hyperlink ref="I89" display="leetcode.cn/problems/target-sum/" r:id="codexHyperlink172"/>
+    <hyperlink ref="E90" display="139. 单词拆分" tooltip="15_动态规划.ipynb / lc-139" r:id="codexHyperlink173"/>
+    <hyperlink ref="I90" display="leetcode.cn/problems/word-break/" r:id="codexHyperlink174"/>
+    <hyperlink ref="E91" display="300. 最长递增子序列" tooltip="15_动态规划.ipynb / lc-300" r:id="codexHyperlink175"/>
+    <hyperlink ref="I91" display="leetcode.cn/problems/longest-increasing-subsequence/" r:id="codexHyperlink176"/>
+    <hyperlink ref="E92" display="1187. 使数组严格递增" tooltip="15_动态规划.ipynb / lc-1187" r:id="codexHyperlink177"/>
+    <hyperlink ref="I92" display="leetcode.cn/problems/make-array-strictly-increasing/" r:id="codexHyperlink178"/>
+    <hyperlink ref="E93" display="1671. 得到山形数组的最少删除次数" tooltip="15_动态规划.ipynb / lc-1671" r:id="codexHyperlink179"/>
+    <hyperlink ref="I93" display="leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/" r:id="codexHyperlink180"/>
+    <hyperlink ref="E94" display="1964. 找出到每个位置为止的最长合法障碍赛跑路线" tooltip="15_动态规划.ipynb / lc-1964" r:id="codexHyperlink181"/>
+    <hyperlink ref="I94" display="leetcode.cn/problems/longest-obstacle-course-at-each-position/" r:id="codexHyperlink182"/>
+    <hyperlink ref="E95" display="152. 乘积最大子数组" tooltip="15_动态规划.ipynb / lc-152" r:id="codexHyperlink183"/>
+    <hyperlink ref="I95" display="leetcode.cn/problems/maximum-product-subarray/" r:id="codexHyperlink184"/>
+    <hyperlink ref="E96" display="32. 最长有效括号" tooltip="15_动态规划.ipynb / lc-32" r:id="codexHyperlink185"/>
+    <hyperlink ref="I96" display="leetcode.cn/problems/longest-valid-parentheses/" r:id="codexHyperlink186"/>
+    <hyperlink ref="E97" display="1770. 执行乘法运算的最大分数" tooltip="16_多维动态规划.ipynb / lc-1770" r:id="codexHyperlink187"/>
+    <hyperlink ref="I97" display="leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/" r:id="codexHyperlink188"/>
+    <hyperlink ref="E98" display="5. 最长回文子串" tooltip="16_多维动态规划.ipynb / lc-5" r:id="codexHyperlink189"/>
+    <hyperlink ref="I98" display="leetcode.cn/problems/longest-palindromic-substring/" r:id="codexHyperlink190"/>
+    <hyperlink ref="E99" display="516. 最长回文子序列" tooltip="16_多维动态规划.ipynb / lc-516" r:id="codexHyperlink191"/>
+    <hyperlink ref="I99" display="leetcode.cn/problems/longest-palindromic-subsequence/" r:id="codexHyperlink192"/>
+    <hyperlink ref="E100" display="647. 回文子串" tooltip="16_多维动态规划.ipynb / lc-647" r:id="codexHyperlink193"/>
+    <hyperlink ref="I100" display="leetcode.cn/problems/palindromic-substrings/" r:id="codexHyperlink194"/>
+    <hyperlink ref="E101" display="1039. 多边形三角剖分的最低得分" tooltip="16_多维动态规划.ipynb / lc-1039" r:id="codexHyperlink195"/>
+    <hyperlink ref="I101" display="leetcode.cn/problems/minimum-score-triangulation-of-polygon/" r:id="codexHyperlink196"/>
+    <hyperlink ref="E102" display="1143. 最长公共子序列" tooltip="16_多维动态规划.ipynb / lc-1143" r:id="codexHyperlink197"/>
+    <hyperlink ref="I102" display="leetcode.cn/problems/longest-common-subsequence/" r:id="codexHyperlink198"/>
+    <hyperlink ref="E103" display="712. 两个字符串的最小ASCII删除和" tooltip="16_多维动态规划.ipynb / lc-712" r:id="codexHyperlink199"/>
+    <hyperlink ref="I103" display="leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/" r:id="codexHyperlink200"/>
+    <hyperlink ref="E104" display="72. 编辑距离" tooltip="16_多维动态规划.ipynb / lc-72" r:id="codexHyperlink201"/>
+    <hyperlink ref="I104" display="leetcode.cn/problems/edit-distance/" r:id="codexHyperlink202"/>
+    <hyperlink ref="E105" display="75. 颜色分类" tooltip="17_技巧.ipynb / lc-75" r:id="codexHyperlink203"/>
+    <hyperlink ref="I105" display="leetcode.cn/problems/sort-colors/" r:id="codexHyperlink204"/>
+    <hyperlink ref="E106" display="31. 下一个排列" tooltip="17_技巧.ipynb / lc-31" r:id="codexHyperlink205"/>
+    <hyperlink ref="I106" display="leetcode.cn/problems/next-permutation/" r:id="codexHyperlink206"/>
+    <hyperlink ref="E107" display="287. 寻找重复数" tooltip="17_技巧.ipynb / lc-287" r:id="codexHyperlink207"/>
+    <hyperlink ref="I107" display="leetcode.cn/problems/find-the-duplicate-number/" r:id="codexHyperlink208"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Restore tracker notes and original layout for 114 problems
</commit_message>
<xml_diff>
--- a/leetcode_hot100/LeetCode Hot100与高频题目刷题清单与进度追踪表.xlsx
+++ b/leetcode_hot100/LeetCode Hot100与高频题目刷题清单与进度追踪表.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hot100与高频题目" sheetId="1" r:id="Rd8e30cef1a514d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hot100与高频题目" sheetId="1" r:id="Rc07ced474ad64eb1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -162,27 +162,39 @@
     </x:fill>
   </x:fills>
   <x:borders count="5">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:left>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
+      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:top>
       <x:bottom style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
+      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:right>
@@ -192,6 +204,7 @@
       <x:bottom style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
@@ -206,12 +219,13 @@
       <x:bottom style="thin">
         <x:color rgb="FFB0B0B0"/>
       </x:bottom>
+      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="104">
+  <x:cellXfs count="103">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -433,9 +447,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="201" fontId="9" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -648,8 +659,8 @@
     <col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="34" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="9" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="8" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="11" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="8" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="11" hidden="1" customWidth="1"/>
     <col min="9" max="9" width="42" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="14" hidden="0" customWidth="1"/>
     <col min="11" max="11" width="10" hidden="0" customWidth="1"/>
@@ -659,7 +670,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="5" t="str">
-        <v>LeetCode Hot 100 与高频题目总数：104</v>
+        <v>LeetCode Hot 100 与高频题目总数：114</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -737,7 +748,7 @@
       <c r="A4" s="28" t="str">
         <v>哈希</v>
       </c>
-      <c r="B4" s="103" t="str">
+      <c r="B4" s="102" t="str">
         <v>分组哈希</v>
       </c>
       <c r="C4" s="34" t="n">
@@ -771,7 +782,7 @@
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="28"/>
-      <c r="B5" s="103" t="str">
+      <c r="B5" s="102" t="str">
         <v>集合查找</v>
       </c>
       <c r="C5" s="34" t="n">
@@ -791,21 +802,25 @@
       <c r="I5" s="56" t="str">
         <v>leetcode.cn/problems/longest-consecutive-sequence/</v>
       </c>
-      <c r="J5" s="73"/>
+      <c r="J5" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K5" s="74" t="n">
         <f>LEN(J5)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J5,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" s="71" t="str">
         <v>用 HashSet 实现 $O(1)$ 查找，只对“没有前驱数”的数字作为起点向后累加计算长度，确保每个数字最多只被遍历常数次，从而在 $O(n)$ 时间内找到最长连续序列。</v>
       </c>
-      <c r="M5" s="71"/>
+      <c r="M5" s="71" t="str">
+        <v>请注意需要遍历集合而不是哈希表</v>
+      </c>
     </row>
     <row r="6" ht="50" customHeight="1">
       <c r="A6" s="28" t="str">
         <v>双指针</v>
       </c>
-      <c r="B6" s="103" t="str">
+      <c r="B6" s="102" t="str">
         <v>同向双指针</v>
       </c>
       <c r="C6" s="34" t="n">
@@ -825,10 +840,12 @@
       <c r="I6" s="56" t="str">
         <v>leetcode.cn/problems/move-zeroes/</v>
       </c>
-      <c r="J6" s="73"/>
+      <c r="J6" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K6" s="74" t="n">
         <f>LEN(J6)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J6,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" s="85" t="str">
         <v>保证下标[left,right-1]区域都是0,其中left指向第一个0元素;当遇到一个非0数字后,将left与right位置元素互换;然后将left+1,保证该区间内仍是非0元素</v>
@@ -837,7 +854,7 @@
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="28"/>
-      <c r="B7" s="103" t="str">
+      <c r="B7" s="102" t="str">
         <v>相向双指针</v>
       </c>
       <c r="C7" s="34" t="n">
@@ -869,7 +886,7 @@
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="28"/>
-      <c r="B8" s="103"/>
+      <c r="B8" s="102"/>
       <c r="C8" s="34" t="n">
         <v>2</v>
       </c>
@@ -899,7 +916,7 @@
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="28"/>
-      <c r="B9" s="103" t="str">
+      <c r="B9" s="102" t="str">
         <v>接雨水</v>
       </c>
       <c r="C9" s="34" t="n">
@@ -933,7 +950,7 @@
       <c r="A10" s="28" t="str">
         <v>滑动窗口</v>
       </c>
-      <c r="B10" s="103" t="str">
+      <c r="B10" s="102" t="str">
         <v>不定长窗口</v>
       </c>
       <c r="C10" s="34" t="n">
@@ -965,7 +982,7 @@
     </row>
     <row r="11" ht="78" customHeight="1">
       <c r="A11" s="28"/>
-      <c r="B11" s="103"/>
+      <c r="B11" s="102"/>
       <c r="C11" s="34" t="n">
         <v>2</v>
       </c>
@@ -995,7 +1012,7 @@
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="28"/>
-      <c r="B12" s="103"/>
+      <c r="B12" s="102"/>
       <c r="C12" s="34" t="n">
         <v>3</v>
       </c>
@@ -1023,9 +1040,9 @@
       </c>
       <c r="M12" s="71"/>
     </row>
-    <row r="13" ht="50" customHeight="1">
+    <row r="13" ht="58.400001525878906" customHeight="1">
       <c r="A13" s="28"/>
-      <c r="B13" s="103" t="str">
+      <c r="B13" s="102" t="str">
         <v>异位词窗口</v>
       </c>
       <c r="C13" s="34" t="n">
@@ -1045,13 +1062,15 @@
       <c r="I13" s="56" t="str">
         <v>leetcode.cn/problems/find-all-anagrams-in-a-string/</v>
       </c>
-      <c r="J13" s="73"/>
+      <c r="J13" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K13" s="74" t="n">
         <f>LEN(J13)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J13,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L13" s="71" t="str">
-        <v>（定长滑动窗口） 思路就是先构建一个定长滑动窗口，然后逐渐加入右边的值，删除左边的值，保证滑动窗口的长度不变，然后进行判断</v>
+        <v>这个题目while循环判断的是字符出现的次数是否比p中多,但是少不会判断,因此退出循环需要判断长度是否满足要求,注意使用Conuter(p),然后在s中遇到相同字符的时候,直接减去,while循环里面加1</v>
       </c>
       <c r="M13" s="71"/>
     </row>
@@ -1059,7 +1078,7 @@
       <c r="A14" s="28" t="str">
         <v>子串</v>
       </c>
-      <c r="B14" s="103" t="str">
+      <c r="B14" s="102" t="str">
         <v>前缀和与计数</v>
       </c>
       <c r="C14" s="34" t="n">
@@ -1093,7 +1112,7 @@
     </row>
     <row r="15" ht="78" customHeight="1">
       <c r="A15" s="28"/>
-      <c r="B15" s="103" t="str">
+      <c r="B15" s="102" t="str">
         <v>单调队列窗口</v>
       </c>
       <c r="C15" s="34" t="n">
@@ -1113,21 +1132,23 @@
       <c r="I15" s="56" t="str">
         <v>leetcode.cn/problems/sliding-window-maximum/</v>
       </c>
-      <c r="J15" s="73"/>
+      <c r="J15" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K15" s="74" t="n">
         <f>LEN(J15)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J15,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" s="71" t="str">
-        <v>算法的核心思想是维护一个单调递减的队列，当新元素的值大于等于队尾的值的时候，那么末尾元素就不可能作为后续的最大值了，（但这个元素可能作为以它为结尾的最大值，但后续因为滑动窗口始终包含新旧元素，因此旧元素不可能是最大…</v>
+        <v>算法的核心思想是维护一个单调递减的双端队列,保证队列头部元素为滑动窗口最大值</v>
       </c>
       <c r="M15" s="71" t="str">
-        <v>最近一次做错,条件应该是i - queue[0] == k,而不是k-1</v>
+        <v>最近一次做错,条件应该是i - queue[0] == k,而不是k-1;要先判断是否超出范围在进行值的添加</v>
       </c>
     </row>
     <row r="16" ht="71" customHeight="1">
       <c r="A16" s="28"/>
-      <c r="B16" s="103" t="str">
+      <c r="B16" s="102" t="str">
         <v>覆盖窗口</v>
       </c>
       <c r="C16" s="34" t="n">
@@ -1156,14 +1177,14 @@
         <v>不定长滑动窗口的思路,内部循环是从满足条件到不满足条件,使用diff来统计当前窗口中 c 的数量 − t 中 c 的数量;使用ge_num来统计s是否覆盖t,当要删除左侧元素也就是left的时候,首先要判断diff[left] == 0,如果成立的话说明删除后s中对应的字符串数量小于t中,应该将ge_num-1.</v>
       </c>
       <c r="M16" s="71" t="str">
-        <v>最近一次做错,当判断当前滑动窗口左侧的元素对应数值为0是,应该使用s[left]而不是left</v>
+        <v>ans_left以及ans_right的初始化,同时注意在每次循环开始的时候判断最小值</v>
       </c>
     </row>
     <row r="17" ht="64" customHeight="1">
       <c r="A17" s="28" t="str">
         <v>普通数组</v>
       </c>
-      <c r="B17" s="103" t="str">
+      <c r="B17" s="102" t="str">
         <v>连续子数组</v>
       </c>
       <c r="C17" s="34" t="n">
@@ -1195,7 +1216,7 @@
     </row>
     <row r="18" ht="45.79999923706055" customHeight="1">
       <c r="A18" s="28"/>
-      <c r="B18" s="103" t="str">
+      <c r="B18" s="102" t="str">
         <v>区间合并</v>
       </c>
       <c r="C18" s="34" t="n">
@@ -1229,7 +1250,7 @@
     </row>
     <row r="19" ht="78" customHeight="1">
       <c r="A19" s="28"/>
-      <c r="B19" s="103" t="str">
+      <c r="B19" s="102" t="str">
         <v>原地变换</v>
       </c>
       <c r="C19" s="34" t="n">
@@ -1249,19 +1270,23 @@
       <c r="I19" s="56" t="str">
         <v>leetcode.cn/problems/rotate-array/</v>
       </c>
-      <c r="J19" s="73"/>
+      <c r="J19" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K19" s="74" t="n">
         <f>LEN(J19)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J19,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" s="96" t="str">
         <v>使用三次反转法,同时需要注意对k的处理:k = k % n,避免k的值不合理</v>
       </c>
-      <c r="M19" s="71"/>
+      <c r="M19" s="71" t="str">
+        <v>忽略对k的处理</v>
+      </c>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="28"/>
-      <c r="B20" s="103" t="str">
+      <c r="B20" s="102" t="str">
         <v>前后缀乘积</v>
       </c>
       <c r="C20" s="34" t="n">
@@ -1281,19 +1306,21 @@
       <c r="I20" s="56" t="str">
         <v>leetcode.cn/problems/product-of-array-except-self/</v>
       </c>
-      <c r="J20" s="73"/>
+      <c r="J20" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K20" s="74" t="n">
         <f>LEN(J20)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J20,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" s="71" t="str">
-        <v>思路：求每个数组元素的前缀与后缀乘积，然后令前后缀相乘</v>
+        <v>思路：求每个数组元素的前缀与后缀乘积，然后令前后缀相乘;注意只使用一个列表就可以</v>
       </c>
       <c r="M20" s="71"/>
     </row>
     <row r="21" ht="78" customHeight="1">
       <c r="A21" s="28"/>
-      <c r="B21" s="103" t="str">
+      <c r="B21" s="102" t="str">
         <v>原地哈希</v>
       </c>
       <c r="C21" s="34" t="n">
@@ -1321,13 +1348,15 @@
       <c r="L21" s="71" t="str">
         <v>思想： 看学号为1到n的学生是否坐在了0到n-1的位置上 对于一个长度为n的数组，它的索引范围为[0,n-1],缺失的第一个正数一定在[1,n+1]的范围内，所以对于一个学号为nums[i]的学生，他应该坐在nums[i-1]位置;</v>
       </c>
-      <c r="M21" s="71"/>
+      <c r="M21" s="71" t="str">
+        <v>while循环里面同时判断当前num是否大于0小于等于n</v>
+      </c>
     </row>
     <row r="22" ht="45.79999923706055" customHeight="1">
       <c r="A22" s="28" t="str">
         <v>矩阵</v>
       </c>
-      <c r="B22" s="103" t="str">
+      <c r="B22" s="102" t="str">
         <v>标记置零</v>
       </c>
       <c r="C22" s="34" t="n">
@@ -1337,7 +1366,7 @@
         <v>73</v>
       </c>
       <c r="E22" s="72" t="str">
-        <v>73. 矩阵置零</v>
+        <v>73.矩阵置零</v>
       </c>
       <c r="F22" s="45" t="str">
         <v>中等</v>
@@ -1358,12 +1387,12 @@
         <v>用首行首列作为标记数组记录含0的行列，再二次遍历置零；注意首行首列本身要先处理;倒序就是为了防止 matrix[0][0] = 0 在处理第 0 列时提前把 matrix[i][0] 改成 0，进而误伤整行。</v>
       </c>
       <c r="M22" s="71" t="str">
-        <v>注意外部循环从1开始</v>
-      </c>
-    </row>
-    <row r="23" ht="36" customHeight="1">
+        <v>注意两次循环中有关行的循环都从从1开始,第二次循环中与列倒序遍历</v>
+      </c>
+    </row>
+    <row r="23" ht="45.79999923706055" customHeight="1">
       <c r="A23" s="28"/>
-      <c r="B23" s="103" t="str">
+      <c r="B23" s="102" t="str">
         <v>边界模拟</v>
       </c>
       <c r="C23" s="34" t="n">
@@ -1383,19 +1412,23 @@
       <c r="I23" s="56" t="str">
         <v>leetcode.cn/problems/spiral-matrix/</v>
       </c>
-      <c r="J23" s="73"/>
+      <c r="J23" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K23" s="74" t="n">
         <f>LEN(J23)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J23,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" s="71" t="str">
         <v>按上、右、下、左四条边界循环收缩；防止m*n为奇数时中心元素遗漏</v>
       </c>
-      <c r="M23" s="71"/>
+      <c r="M23" s="71" t="str">
+        <v>注意条件判断与for循环里面使用的边界不同,比如说判断left &lt;=right成立的时候,里面进行的循环应该是与top,bottom有关的.</v>
+      </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="28"/>
-      <c r="B24" s="103" t="str">
+      <c r="B24" s="102" t="str">
         <v>转置与反转</v>
       </c>
       <c r="C24" s="34" t="n">
@@ -1415,10 +1448,12 @@
       <c r="I24" s="56" t="str">
         <v>leetcode.cn/problems/rotate-image/</v>
       </c>
-      <c r="J24" s="73"/>
+      <c r="J24" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K24" s="74" t="n">
         <f>LEN(J24)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J24,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="71" t="str">
         <v>先转置（沿主对角线），再逐行反转</v>
@@ -1427,7 +1462,7 @@
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="28"/>
-      <c r="B25" s="103" t="str">
+      <c r="B25" s="102" t="str">
         <v>二维有序查找</v>
       </c>
       <c r="C25" s="34" t="n">
@@ -1447,10 +1482,12 @@
       <c r="I25" s="56" t="str">
         <v>https://leetcode.cn/problems/search-a-2d-matrix-ii/</v>
       </c>
-      <c r="J25" s="73"/>
+      <c r="J25" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K25" s="74" t="n">
         <f>LEN(J25)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J25,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" s="71" t="str">
         <v>行、列分别有序，从右上角逐行或逐列排除；区别于74题的整体有序条件。</v>
@@ -1461,7 +1498,7 @@
       <c r="A26" s="28" t="str">
         <v>链表</v>
       </c>
-      <c r="B26" s="103" t="str">
+      <c r="B26" s="102" t="str">
         <v>相交与环</v>
       </c>
       <c r="C26" s="34" t="n">
@@ -1481,19 +1518,21 @@
       <c r="I26" s="56" t="str">
         <v>leetcode.cn/problems/intersection-of-two-linked-lists/</v>
       </c>
-      <c r="J26" s="73"/>
+      <c r="J26" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K26" s="74" t="n">
         <f>LEN(J26)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J26,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" s="71" t="str">
-        <v>使用集合而非列表存储节点，因为在后续的环节，使用列表的话时间复杂度为0(n),而对于集合而言，时间复杂度为0(1),对于集合与字典而言，哪怕是值与后继都相同的两个节点，地址不同的话仍然可以存放进去。 if right i…</v>
+        <v>使用浪漫相遇法,外部循环时while pa != pb</v>
       </c>
       <c r="M26" s="71"/>
     </row>
     <row r="27" ht="50" customHeight="1">
       <c r="A27" s="28"/>
-      <c r="B27" s="103"/>
+      <c r="B27" s="102"/>
       <c r="C27" s="34" t="n">
         <v>2</v>
       </c>
@@ -1511,19 +1550,23 @@
       <c r="I27" s="56" t="str">
         <v>leetcode.cn/problems/linked-list-cycle/</v>
       </c>
-      <c r="J27" s="73"/>
+      <c r="J27" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K27" s="74" t="n">
         <f>LEN(J27)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J27,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" s="71" t="str">
         <v>佛洛依德判圈算法：使用快慢指针检测是否存在环，快指针每次走两步，慢指针每次走一步，如果最终快指针追上慢指针，证明有环。</v>
       </c>
-      <c r="M27" s="71"/>
+      <c r="M27" s="71" t="str">
+        <v>具体做法:外部循环只判断fast是否等于slow,内部判断fast的合法性</v>
+      </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="28"/>
-      <c r="B28" s="103"/>
+      <c r="B28" s="102"/>
       <c r="C28" s="34" t="n">
         <v>3</v>
       </c>
@@ -1541,10 +1584,12 @@
       <c r="I28" s="56" t="str">
         <v>leetcode.cn/problems/linked-list-cycle-ii/</v>
       </c>
-      <c r="J28" s="73"/>
+      <c r="J28" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K28" s="74" t="n">
         <f>LEN(J28)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J28,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" s="71" t="str">
         <v>详见题解</v>
@@ -1553,7 +1598,7 @@
     </row>
     <row r="29" ht="50" customHeight="1">
       <c r="A29" s="28"/>
-      <c r="B29" s="103" t="str">
+      <c r="B29" s="102" t="str">
         <v>链表反转</v>
       </c>
       <c r="C29" s="34" t="n">
@@ -1573,19 +1618,21 @@
       <c r="I29" s="56" t="str">
         <v>leetcode.cn/problems/reverse-linked-list/</v>
       </c>
-      <c r="J29" s="73"/>
+      <c r="J29" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K29" s="74" t="n">
         <f>LEN(J29)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J29,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" s="71" t="str">
         <v>迭代：prev/curr指针逐个反转next；递归：先反转后续，再 head.next.next=head</v>
       </c>
       <c r="M29" s="71"/>
     </row>
-    <row r="30" ht="36" customHeight="1">
+    <row r="30" ht="45.79999923706055" customHeight="1">
       <c r="A30" s="28"/>
-      <c r="B30" s="103"/>
+      <c r="B30" s="102"/>
       <c r="C30" s="34" t="n">
         <v>2</v>
       </c>
@@ -1609,13 +1656,13 @@
         <v>0</v>
       </c>
       <c r="L30" s="71" t="str">
-        <v>注意每个group的pre以及end</v>
+        <v>pre以及end指针最关键,利用这两个指针进行反转,每次反转要处理三步:1.pre与头部反转节点以及的关系;2.反转内部的实现;3.尾部反转节点与下一组之间的关系</v>
       </c>
       <c r="M30" s="71"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="28"/>
-      <c r="B31" s="103" t="str">
+      <c r="B31" s="102" t="str">
         <v>快慢指针</v>
       </c>
       <c r="C31" s="34" t="n">
@@ -1635,10 +1682,12 @@
       <c r="I31" s="56" t="str">
         <v>leetcode.cn/problems/palindrome-linked-list/</v>
       </c>
-      <c r="J31" s="73"/>
+      <c r="J31" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K31" s="74" t="n">
         <f>LEN(J31)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J31,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" s="71" t="str">
         <v>回文链表问题使用快慢指针方法解答最优，其中，慢指针每次走一步，快指针每次走两步。</v>
@@ -1647,7 +1696,7 @@
     </row>
     <row r="32" ht="45.79999923706055" customHeight="1">
       <c r="A32" s="28"/>
-      <c r="B32" s="103"/>
+      <c r="B32" s="102"/>
       <c r="C32" s="34" t="n">
         <v>2</v>
       </c>
@@ -1665,10 +1714,12 @@
       <c r="I32" s="56" t="str">
         <v>leetcode.cn/problems/remove-nth-node-from-end-of-list/description/</v>
       </c>
-      <c r="J32" s="73"/>
+      <c r="J32" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K32" s="74" t="n">
         <f>LEN(J32)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J32,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" s="71" t="str">
         <v>dummy节点的使用,同时注意当右指针指向最后一个结点的时候,左指针指向的是倒数第(1+n)个节点,也就是说左指针的下一个节点就是倒数第n个节点</v>
@@ -1677,7 +1728,7 @@
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="28"/>
-      <c r="B33" s="103" t="str">
+      <c r="B33" s="102" t="str">
         <v>数位运算</v>
       </c>
       <c r="C33" s="34" t="n">
@@ -1697,10 +1748,12 @@
       <c r="I33" s="101" t="str">
         <v>leetcode.cn/problems/add-two-numbers/</v>
       </c>
-      <c r="J33" s="73"/>
+      <c r="J33" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K33" s="74" t="n">
         <f>LEN(J33)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J33,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="71" t="str">
         <v>注意l1.val以及l1.next的赋值方法,里面包含判断,二者紧密结合</v>
@@ -1709,7 +1762,7 @@
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="28"/>
-      <c r="B34" s="103" t="str">
+      <c r="B34" s="102" t="str">
         <v>节点交换</v>
       </c>
       <c r="C34" s="34" t="n">
@@ -1729,10 +1782,12 @@
       <c r="I34" s="56" t="str">
         <v>leetcode.cn/problems/swap-nodes-in-pairs/</v>
       </c>
-      <c r="J34" s="73"/>
+      <c r="J34" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K34" s="74" t="n">
         <f>LEN(J34)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J34,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" s="71" t="str">
         <v>需要dummy节点；pre指向每组前驱，两两交换a、b后移动指针</v>
@@ -1741,7 +1796,7 @@
     </row>
     <row r="35" ht="50" customHeight="1">
       <c r="A35" s="28"/>
-      <c r="B35" s="103" t="str">
+      <c r="B35" s="102" t="str">
         <v>深拷贝</v>
       </c>
       <c r="C35" s="34" t="n">
@@ -1761,19 +1816,21 @@
       <c r="I35" s="56" t="str">
         <v>leetcode.cn/problems/copy-list-with-random-pointer/</v>
       </c>
-      <c r="J35" s="73"/>
+      <c r="J35" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K35" s="74" t="n">
         <f>LEN(J35)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J35,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" s="71" t="str">
-        <v>想要完成链表的深拷贝要求先创建所有的节点，在进行next与random的设置，使用哈希表构建原节点与新节点的映射，在构建新节点的next与random。</v>
+        <v>注意当head为空时,返回None;核心思路在于使用字典创建新的节点,两次循环构建新节点之间的关系,对于字典来说,键为旧节点,值为对应的新节点</v>
       </c>
       <c r="M35" s="71"/>
     </row>
     <row r="36" ht="78" customHeight="1">
       <c r="A36" s="28"/>
-      <c r="B36" s="103" t="str">
+      <c r="B36" s="102" t="str">
         <v>归并排序</v>
       </c>
       <c r="C36" s="34" t="n">
@@ -1793,19 +1850,21 @@
       <c r="I36" s="56" t="str">
         <v>leetcode.cn/problems/sort-list/</v>
       </c>
-      <c r="J36" s="73"/>
+      <c r="J36" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K36" s="74" t="n">
         <f>LEN(J36)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J36,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L36" s="71" t="str">
-        <v>使用快慢指针方法找到中点,然后使用归并排序方法进行排序.</v>
+        <v>使用快慢指针方法找到中点,然后使用归并排序方法(递归)进行排序;记住基本结束条件,内部本质上就是一个排序问题</v>
       </c>
       <c r="M36" s="71"/>
     </row>
     <row r="37" ht="64" customHeight="1">
       <c r="A37" s="28"/>
-      <c r="B37" s="103" t="str">
+      <c r="B37" s="102" t="str">
         <v>多路归并</v>
       </c>
       <c r="C37" s="34" t="n">
@@ -1825,19 +1884,23 @@
       <c r="I37" s="56" t="str">
         <v>leetcode.cn/problems/merge-k-sorted-lists/</v>
       </c>
-      <c r="J37" s="73"/>
+      <c r="J37" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K37" s="74" t="n">
         <f>LEN(J37)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J37,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" s="71" t="str">
         <v>此题的思路与链表的归并排序以及两个链表的合并有关，思想是先对链表数组进行递归拆分，然后将单个链表返回并对返回的链表采用链表的合并策略，总体而言相较于链表的直接归并排序要简单一些，因为不需要自己手动将链表拆解。</v>
       </c>
-      <c r="M37" s="71"/>
-    </row>
-    <row r="38" ht="36" customHeight="1">
+      <c r="M37" s="71" t="str">
+        <v>具体做法既可以利用left与right指针判断当前</v>
+      </c>
+    </row>
+    <row r="38" ht="71" customHeight="1">
       <c r="A38" s="28"/>
-      <c r="B38" s="103" t="str">
+      <c r="B38" s="102" t="str">
         <v>缓存设计</v>
       </c>
       <c r="C38" s="34" t="n">
@@ -1857,21 +1920,23 @@
       <c r="I38" s="56" t="str">
         <v>leetcode.cn/problems/lru-cache/description/</v>
       </c>
-      <c r="J38" s="73"/>
+      <c r="J38" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K38" s="74" t="n">
         <f>LEN(J38)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J38,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" s="71" t="str">
-        <v>注意self.hashtable是一个字典,value为双向链表节点,通过.next以及.pre属性构建双向链表</v>
+        <v>使用self.hashtable存储key与对应节点之间的关系,涉及到插入以及删除的时候需要及时更新;使用doublelink双向链表,self.dummy0后面时最久没有使用过的节点,self.dummy1前面是最近使用过的节点;同时对于delete以及insert操作来说,操作的都是节点,同时注意函数内部对于self.num的操作</v>
       </c>
       <c r="M38" s="71"/>
     </row>
-    <row r="39" ht="58.400001525878906" customHeight="1">
+    <row r="39" ht="71" customHeight="1">
       <c r="A39" s="28" t="str">
         <v>二叉树</v>
       </c>
-      <c r="B39" s="103" t="str">
+      <c r="B39" s="102" t="str">
         <v>遍历</v>
       </c>
       <c r="C39" s="34" t="n">
@@ -1891,19 +1956,21 @@
       <c r="I39" s="56" t="str">
         <v>leetcode.cn/problems/binary-tree-inorder-traversal/description/</v>
       </c>
-      <c r="J39" s="73"/>
+      <c r="J39" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K39" s="74" t="n">
         <f>LEN(J39)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J39,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" s="71" t="str">
-        <v>中序遍历的迭代实现以及前序后序遍历的迭代方法,对于中序方法来说,因为在需要在拆桥(根节点有左子树遍历完)和没有左子树的时候添加,因此可以不使用else,但是对于前序和后序遍历来说,在拆桥的时候不能再次添加,因此需要使用else.</v>
+        <v>中序遍历的迭代实现以及前序后序遍历的迭代方法,对于中序方法来说,因为在需要在拆桥(根节点有左子树遍历完)和没有左子树的时候添加,因此可以不使用else,但是对于前序和后序遍历来说,在拆桥的时候不能再次添加,因此需要使用else,在搭桥以及没有左节点的时候记录</v>
       </c>
       <c r="M39" s="71"/>
     </row>
     <row r="40" ht="64" customHeight="1">
       <c r="A40" s="28"/>
-      <c r="B40" s="103"/>
+      <c r="B40" s="102"/>
       <c r="C40" s="34" t="n">
         <v>2</v>
       </c>
@@ -1921,19 +1988,23 @@
       <c r="I40" s="56" t="str">
         <v>leetcode.cn/problems/binary-tree-level-order-traversal/</v>
       </c>
-      <c r="J40" s="73"/>
+      <c r="J40" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K40" s="74" t="n">
         <f>LEN(J40)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J40,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" s="71" t="str">
         <v>树的层序遍历：树的层序遍历不需要提前知道树的深度 注意：使用 res = [[]nums] 并不能生成一个含有nums个列表的二维列表，应该使用: res = [[] for in range(nums)]</v>
       </c>
-      <c r="M40" s="71"/>
+      <c r="M40" s="71" t="str">
+        <v>注意要判断root是否为None</v>
+      </c>
     </row>
     <row r="41" ht="36" customHeight="1">
       <c r="A41" s="28"/>
-      <c r="B41" s="103" t="str">
+      <c r="B41" s="102" t="str">
         <v>深度与结构</v>
       </c>
       <c r="C41" s="34" t="n">
@@ -1953,10 +2024,12 @@
       <c r="I41" s="56" t="str">
         <v>leetcode.cn/problems/maximum-depth-of-binary-tree/</v>
       </c>
-      <c r="J41" s="73"/>
+      <c r="J41" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K41" s="74" t="n">
         <f>LEN(J41)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J41,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" s="71" t="str">
         <v>递归：max(左子树深度, 右子树深度)+1；空节点返回0</v>
@@ -1965,7 +2038,7 @@
     </row>
     <row r="42" ht="36" customHeight="1">
       <c r="A42" s="28"/>
-      <c r="B42" s="103"/>
+      <c r="B42" s="102"/>
       <c r="C42" s="34" t="n">
         <v>2</v>
       </c>
@@ -1983,10 +2056,12 @@
       <c r="I42" s="56" t="str">
         <v>leetcode.cn/problems/invert-binary-tree/</v>
       </c>
-      <c r="J42" s="73"/>
+      <c r="J42" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K42" s="74" t="n">
         <f>LEN(J42)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J42,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" s="71" t="str">
         <v>递归交换左右孩子；或层序遍历逐层交换</v>
@@ -1995,7 +2070,7 @@
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="28"/>
-      <c r="B43" s="103"/>
+      <c r="B43" s="102"/>
       <c r="C43" s="34" t="n">
         <v>3</v>
       </c>
@@ -2013,10 +2088,12 @@
       <c r="I43" s="56" t="str">
         <v>leetcode.cn/problems/symmetric-tree/</v>
       </c>
-      <c r="J43" s="73"/>
+      <c r="J43" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K43" s="74" t="n">
         <f>LEN(J43)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J43,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" s="71" t="str">
         <v>递归：两棵子树镜像对称（左.左==右.右 且 左.右==右.左）;注意需要判断根节点是否为空</v>
@@ -2025,7 +2102,7 @@
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="28"/>
-      <c r="B44" s="103" t="str">
+      <c r="B44" s="102" t="str">
         <v>树的直径（一般树扩展）</v>
       </c>
       <c r="C44" s="34" t="n">
@@ -2045,10 +2122,12 @@
       <c r="I44" s="56" t="str">
         <v>leetcode.cn/problems/diameter-of-binary-tree/</v>
       </c>
-      <c r="J44" s="73"/>
+      <c r="J44" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K44" s="74" t="n">
         <f>LEN(J44)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J44,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" s="71" t="str">
         <v>递归求每个节点左右子树深度，全局max(左深+右深)；直径不一定要过根</v>
@@ -2057,7 +2136,7 @@
     </row>
     <row r="45" ht="78" customHeight="1">
       <c r="A45" s="28"/>
-      <c r="B45" s="103"/>
+      <c r="B45" s="102"/>
       <c r="C45" s="34" t="n">
         <v>2</v>
       </c>
@@ -2087,7 +2166,7 @@
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="28"/>
-      <c r="B46" s="103"/>
+      <c r="B46" s="102"/>
       <c r="C46" s="34" t="n">
         <v>3</v>
       </c>
@@ -2117,7 +2196,7 @@
     </row>
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="28"/>
-      <c r="B47" s="103"/>
+      <c r="B47" s="102"/>
       <c r="C47" s="34" t="n">
         <v>4</v>
       </c>
@@ -2147,7 +2226,7 @@
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="28"/>
-      <c r="B48" s="103" t="str">
+      <c r="B48" s="102" t="str">
         <v>二叉搜索树</v>
       </c>
       <c r="C48" s="34" t="n">
@@ -2167,61 +2246,61 @@
       <c r="I48" s="56" t="str">
         <v>leetcode.cn/problems/validate-binary-search-tree/</v>
       </c>
-      <c r="J48" s="73"/>
+      <c r="J48" s="73" t="str">
+        <v>√</v>
+      </c>
       <c r="K48" s="74" t="n">
         <f>LEN(J48)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J48,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" s="71" t="str">
         <v>中序遍历结果严格递增；或递归传递(lower, upper)上下界校验</v>
       </c>
       <c r="M48" s="71"/>
     </row>
-    <row r="49" ht="64" customHeight="1">
+    <row r="49" ht="60" customHeight="1">
       <c r="A49" s="28"/>
-      <c r="B49" s="103" t="str">
-        <v>结构变换</v>
-      </c>
+      <c r="B49" s="102"/>
       <c r="C49" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D49" s="34" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E49" s="72" t="str">
-        <v>114. 二叉树展开为链表</v>
-      </c>
-      <c r="F49" s="45" t="str">
-        <v>中等</v>
+        <v>108.将有序数组转换为二叉搜索树</v>
+      </c>
+      <c r="F49" s="80" t="str">
+        <v>简单</v>
       </c>
       <c r="G49" s="51"/>
       <c r="H49" s="51"/>
       <c r="I49" s="56" t="str">
-        <v>leetcode.cn/problems/flatten-binary-tree-to-linked-list/</v>
-      </c>
-      <c r="J49" s="73"/>
+        <v>leetcode.cn/problems/convert-sorted-array-to-binary-search-tree/</v>
+      </c>
+      <c r="J49" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K49" s="74" t="n">
         <f>LEN(J49)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J49,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="71" t="str">
-        <v>while 栈非空: 1. 弹出当前节点 = 栈.pop() 2. 连接操作：if pre: pre.right = 当前节点; pre.left = None 3. 入栈操作：先右后左（因为栈是后进先出）</v>
+        <v>二叉搜索树按照中序遍历是严格递增的,基本结束条件为 left &gt; right,然后就是不断迭代mid,构建节点</v>
       </c>
       <c r="M49" s="71"/>
     </row>
-    <row r="50" ht="78" customHeight="1">
+    <row r="50" ht="60" customHeight="1">
       <c r="A50" s="28"/>
-      <c r="B50" s="103" t="str">
-        <v>构造二叉树</v>
-      </c>
+      <c r="B50" s="102"/>
       <c r="C50" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D50" s="34" t="n">
-        <v>105</v>
+        <v>230</v>
       </c>
       <c r="E50" s="72" t="str">
-        <v>105. 从前序与中序遍历序列构造二叉树</v>
+        <v>230. 二叉搜索树中第 K 小的元素</v>
       </c>
       <c r="F50" s="45" t="str">
         <v>中等</v>
@@ -2229,31 +2308,33 @@
       <c r="G50" s="51"/>
       <c r="H50" s="51"/>
       <c r="I50" s="56" t="str">
-        <v>leetcode.cn/problems/construct-binary-tree-from-preorder-and-inorder-traversal/</v>
-      </c>
-      <c r="J50" s="73"/>
+        <v>leetcode.cn/problems/kth-smallest-element-in-a-bst/</v>
+      </c>
+      <c r="J50" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K50" s="74" t="n">
         <f>LEN(J50)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J50,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" s="71" t="str">
-        <v>方法一： 这个方法从递归的角度入手，先获取先序遍历中根节点在中序遍历中的索引，然后根据索引确定根节点的左子树和右子树有多少节点，在递归调用构建左右子树 例如，对于这个例子而言，根节点3在中序中对应的位置为1，也就说明了左…</v>
+        <v>k:需要跳过多少个节点,才能找到目标节点</v>
       </c>
       <c r="M50" s="71"/>
     </row>
-    <row r="51" ht="83.5999984741211" customHeight="1">
+    <row r="51" ht="64" customHeight="1">
       <c r="A51" s="28"/>
-      <c r="B51" s="103" t="str">
-        <v>前缀和路径</v>
+      <c r="B51" s="102" t="str">
+        <v>结构变换</v>
       </c>
       <c r="C51" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D51" s="34" t="n">
-        <v>437</v>
+        <v>114</v>
       </c>
       <c r="E51" s="72" t="str">
-        <v>437. 路径总和 III</v>
+        <v>114. 二叉树展开为链表</v>
       </c>
       <c r="F51" s="45" t="str">
         <v>中等</v>
@@ -2261,7 +2342,7 @@
       <c r="G51" s="51"/>
       <c r="H51" s="51"/>
       <c r="I51" s="56" t="str">
-        <v>leetcode.cn/problems/path-sum-iii/</v>
+        <v>leetcode.cn/problems/flatten-binary-tree-to-linked-list/</v>
       </c>
       <c r="J51" s="73"/>
       <c r="K51" s="74" t="n">
@@ -2269,23 +2350,23 @@
         <v>0</v>
       </c>
       <c r="L51" s="71" t="str">
-        <v>采用前缀和的思想，最后在单次函数执行完之前(也就意味着这个节点作为路径终点的所有路径遍历完成)，将字典当中从根节点到当前节点的数量-1，避免对其他分支造成影响。此题可以看作是560.和为k的子数组的升级版本;同时对于使用前缀和的题目来说,有两点需要注意:1.首先设置cnt[0]=1,避免漏算 2.先判断时候有cnt[curr_sum - target_sum]存在,在更新cnt.</v>
+        <v>while 栈非空: 1. 弹出当前节点 = 栈.pop() 2. 连接操作：if pre: pre.right = 当前节点; pre.left = None 3. 入栈操作：先右后左（因为栈是后进先出）</v>
       </c>
       <c r="M51" s="71"/>
     </row>
-    <row r="52" ht="45.79999923706055" customHeight="1">
+    <row r="52" ht="78" customHeight="1">
       <c r="A52" s="28"/>
-      <c r="B52" s="103" t="str">
-        <v>最近公共祖先</v>
+      <c r="B52" s="102" t="str">
+        <v>构造二叉树</v>
       </c>
       <c r="C52" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D52" s="34" t="n">
-        <v>236</v>
+        <v>105</v>
       </c>
       <c r="E52" s="72" t="str">
-        <v>236. 二叉树的最近公共祖先</v>
+        <v>105. 从前序与中序遍历序列构造二叉树</v>
       </c>
       <c r="F52" s="45" t="str">
         <v>中等</v>
@@ -2293,7 +2374,7 @@
       <c r="G52" s="51"/>
       <c r="H52" s="51"/>
       <c r="I52" s="56" t="str">
-        <v>leetcode.cn/problems/lowest-common-ancestor-of-a-binary-tree/</v>
+        <v>leetcode.cn/problems/construct-binary-tree-from-preorder-and-inorder-traversal/</v>
       </c>
       <c r="J52" s="73"/>
       <c r="K52" s="74" t="n">
@@ -2301,21 +2382,23 @@
         <v>0</v>
       </c>
       <c r="L52" s="71" t="str">
-        <v>递归：节点为p或q为空都返回自身；左右子树返回值均非空时当前节点即最近公共祖先;否则执行return left if left else right判断</v>
+        <v>方法一： 这个方法从递归的角度入手，先获取先序遍历中根节点在中序遍历中的索引，然后根据索引确定根节点的左子树和右子树有多少节点，在递归调用构建左右子树 例如，对于这个例子而言，根节点3在中序中对应的位置为1，也就说明了左…</v>
       </c>
       <c r="M52" s="71"/>
     </row>
-    <row r="53" ht="36" customHeight="1">
+    <row r="53" ht="83.5999984741211" customHeight="1">
       <c r="A53" s="28"/>
-      <c r="B53" s="103"/>
+      <c r="B53" s="102" t="str">
+        <v>前缀和路径</v>
+      </c>
       <c r="C53" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D53" s="34" t="n">
-        <v>235</v>
+        <v>437</v>
       </c>
       <c r="E53" s="72" t="str">
-        <v>235. 二叉搜索树的最近公共祖先</v>
+        <v>437. 路径总和 III</v>
       </c>
       <c r="F53" s="45" t="str">
         <v>中等</v>
@@ -2323,7 +2406,7 @@
       <c r="G53" s="51"/>
       <c r="H53" s="51"/>
       <c r="I53" s="56" t="str">
-        <v>https://leetcode.cn/problems/lowest-common-ancestor-of-a-binary-search-tree/</v>
+        <v>leetcode.cn/problems/path-sum-iii/</v>
       </c>
       <c r="J53" s="73"/>
       <c r="K53" s="74" t="n">
@@ -2331,31 +2414,31 @@
         <v>0</v>
       </c>
       <c r="L53" s="71" t="str">
-        <v>利用BST有序性：p、q都较小时向左，都较大时向右，否则当前节点为最近公共祖先。</v>
+        <v>采用前缀和的思想，最后在单次函数执行完之前(也就意味着这个节点作为路径终点的所有路径遍历完成)，将字典当中从根节点到当前节点的数量-1，避免对其他分支造成影响。此题可以看作是560.和为k的子数组的升级版本;同时对于使用前缀和的题目来说,有两点需要注意:1.首先设置cnt[0]=1,避免漏算 2.先判断时候有cnt[curr_sum - target_sum]存在,在更新cnt.</v>
       </c>
       <c r="M53" s="71"/>
     </row>
-    <row r="54" ht="36" customHeight="1">
+    <row r="54" ht="45.79999923706055" customHeight="1">
       <c r="A54" s="28"/>
-      <c r="B54" s="103" t="str">
-        <v>树形DP</v>
+      <c r="B54" s="102" t="str">
+        <v>最近公共祖先</v>
       </c>
       <c r="C54" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D54" s="34" t="n">
-        <v>124</v>
+        <v>236</v>
       </c>
       <c r="E54" s="72" t="str">
-        <v>124. 二叉树中的最大路径和</v>
-      </c>
-      <c r="F54" s="91" t="str">
-        <v>困难</v>
+        <v>236. 二叉树的最近公共祖先</v>
+      </c>
+      <c r="F54" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G54" s="51"/>
       <c r="H54" s="51"/>
       <c r="I54" s="56" t="str">
-        <v>leetcode.cn/problems/binary-tree-maximum-path-sum/</v>
+        <v>leetcode.cn/problems/lowest-common-ancestor-of-a-binary-tree/</v>
       </c>
       <c r="J54" s="73"/>
       <c r="K54" s="74" t="n">
@@ -2363,21 +2446,21 @@
         <v>0</v>
       </c>
       <c r="L54" s="71" t="str">
-        <v>递归返回单边最大路径和 node.val+max(左,右,0)；全局max记录经过当前节点的最大路径和</v>
+        <v>递归：节点为p或q为空都返回自身；左右子树返回值均非空时当前节点即最近公共祖先;否则执行return left if left else right判断</v>
       </c>
       <c r="M54" s="71"/>
     </row>
     <row r="55" ht="36" customHeight="1">
       <c r="A55" s="28"/>
-      <c r="B55" s="103"/>
+      <c r="B55" s="102"/>
       <c r="C55" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D55" s="34" t="n">
-        <v>337</v>
+        <v>235</v>
       </c>
       <c r="E55" s="72" t="str">
-        <v>337. 打家劫舍 III</v>
+        <v>235. 二叉搜索树的最近公共祖先</v>
       </c>
       <c r="F55" s="45" t="str">
         <v>中等</v>
@@ -2385,7 +2468,7 @@
       <c r="G55" s="51"/>
       <c r="H55" s="51"/>
       <c r="I55" s="56" t="str">
-        <v>leetcode.cn/problems/house-robber-iii/</v>
+        <v>https://leetcode.cn/problems/lowest-common-ancestor-of-a-binary-search-tree/</v>
       </c>
       <c r="J55" s="73"/>
       <c r="K55" s="74" t="n">
@@ -2393,21 +2476,23 @@
         <v>0</v>
       </c>
       <c r="L55" s="71" t="str">
-        <v>树形DP：每个节点返回[偷,不偷]；偷则子节点不能偷，不偷取子节点最大值；后序遍历</v>
+        <v>利用BST有序性：p、q都较小时向左，都较大时向右，否则当前节点为最近公共祖先。</v>
       </c>
       <c r="M55" s="71"/>
     </row>
-    <row r="56" ht="78" customHeight="1">
+    <row r="56" ht="36" customHeight="1">
       <c r="A56" s="28"/>
-      <c r="B56" s="103"/>
+      <c r="B56" s="102" t="str">
+        <v>树形DP</v>
+      </c>
       <c r="C56" s="34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D56" s="34" t="n">
-        <v>968</v>
+        <v>124</v>
       </c>
       <c r="E56" s="72" t="str">
-        <v>968. 监控二叉树</v>
+        <v>124. 二叉树中的最大路径和</v>
       </c>
       <c r="F56" s="91" t="str">
         <v>困难</v>
@@ -2415,7 +2500,7 @@
       <c r="G56" s="51"/>
       <c r="H56" s="51"/>
       <c r="I56" s="56" t="str">
-        <v>leetcode.cn/problems/binary-tree-cameras/</v>
+        <v>leetcode.cn/problems/binary-tree-maximum-path-sum/</v>
       </c>
       <c r="J56" s="73"/>
       <c r="K56" s="74" t="n">
@@ -2423,25 +2508,21 @@
         <v>0</v>
       </c>
       <c r="L56" s="71" t="str">
-        <v>此题的核心是针对每个节点，从节点的不同状态入手，分析节点在不同状态下的最小数目或者最小点权和。 分析一下红色节点的处理逻辑，对于红色节点而言，它必须有一个子节点是蓝色节点，而对于黄色节点而言，它的子节点是由红色与蓝色构成…</v>
+        <v>递归返回单边最大路径和 node.val+max(左,右,0)；全局max记录经过当前节点的最大路径和</v>
       </c>
       <c r="M56" s="71"/>
     </row>
-    <row r="57" ht="78" customHeight="1">
-      <c r="A57" s="28" t="str">
-        <v>图论</v>
-      </c>
-      <c r="B57" s="103" t="str">
-        <v>连通块遍历</v>
-      </c>
+    <row r="57" ht="36" customHeight="1">
+      <c r="A57" s="28"/>
+      <c r="B57" s="102"/>
       <c r="C57" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D57" s="34" t="n">
-        <v>200</v>
+        <v>337</v>
       </c>
       <c r="E57" s="72" t="str">
-        <v>200. 岛屿数量</v>
+        <v>337. 打家劫舍 III</v>
       </c>
       <c r="F57" s="45" t="str">
         <v>中等</v>
@@ -2449,7 +2530,7 @@
       <c r="G57" s="51"/>
       <c r="H57" s="51"/>
       <c r="I57" s="56" t="str">
-        <v>leetcode.cn/problems/number-of-islands/</v>
+        <v>leetcode.cn/problems/house-robber-iii/</v>
       </c>
       <c r="J57" s="73"/>
       <c r="K57" s="74" t="n">
@@ -2457,31 +2538,29 @@
         <v>0</v>
       </c>
       <c r="L57" s="71" t="str">
-        <v>方法一：DFS 方法二：BFS ,对于BFS算法来说,队列的创建放在bfs函数里面,同时队列里面存储的是已经被探索过的岛屿元素,值由1变为0</v>
+        <v>树形DP：每个节点返回[偷,不偷]；偷则子节点不能偷，不偷取子节点最大值；后序遍历</v>
       </c>
       <c r="M57" s="71"/>
     </row>
-    <row r="58" ht="140" customHeight="1">
+    <row r="58" ht="78" customHeight="1">
       <c r="A58" s="28"/>
-      <c r="B58" s="103" t="str">
-        <v>多源 BFS</v>
-      </c>
+      <c r="B58" s="102"/>
       <c r="C58" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D58" s="34" t="n">
-        <v>994</v>
+        <v>968</v>
       </c>
       <c r="E58" s="72" t="str">
-        <v>994. 腐烂的橘子</v>
-      </c>
-      <c r="F58" s="45" t="str">
-        <v>中等</v>
+        <v>968. 监控二叉树</v>
+      </c>
+      <c r="F58" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G58" s="51"/>
       <c r="H58" s="51"/>
       <c r="I58" s="56" t="str">
-        <v>leetcode.cn/problems/rotting-oranges/</v>
+        <v>leetcode.cn/problems/binary-tree-cameras/</v>
       </c>
       <c r="J58" s="73"/>
       <c r="K58" s="74" t="n">
@@ -2489,25 +2568,25 @@
         <v>0</v>
       </c>
       <c r="L58" s="71" t="str">
-        <v>多源 BFS：先扫描整个网格，将所有腐烂橘子入队并统计新鲜橘子 num；每层处理当前队列长度，对应 1 分钟。新鲜橘子入队时立即标记为腐烂并将 num 减一，避免重复入队。</v>
-      </c>
-      <c r="M58" s="96" t="str">
-        <v>【曾错重点】首次完整遍历网格后、进入 while queue 前，先判断 num == 0（即 if not num），为 0 立即 return 0！不能只在 BFS 内判断：如 [[0]] 没有新鲜橘子，队列也为空，BFS 不执行，会误走末尾 return -1。</v>
-      </c>
-    </row>
-    <row r="59" ht="83.5999984741211" customHeight="1">
-      <c r="A59" s="28"/>
-      <c r="B59" s="103" t="str">
-        <v>拓扑排序</v>
+        <v>此题的核心是针对每个节点，从节点的不同状态入手，分析节点在不同状态下的最小数目或者最小点权和。 分析一下红色节点的处理逻辑，对于红色节点而言，它必须有一个子节点是蓝色节点，而对于黄色节点而言，它的子节点是由红色与蓝色构成…</v>
+      </c>
+      <c r="M58" s="71"/>
+    </row>
+    <row r="59" ht="78" customHeight="1">
+      <c r="A59" s="28" t="str">
+        <v>图论</v>
+      </c>
+      <c r="B59" s="102" t="str">
+        <v>连通块遍历</v>
       </c>
       <c r="C59" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D59" s="34" t="n">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="E59" s="72" t="str">
-        <v>207. 课程表</v>
+        <v>200. 岛屿数量</v>
       </c>
       <c r="F59" s="45" t="str">
         <v>中等</v>
@@ -2515,31 +2594,31 @@
       <c r="G59" s="51"/>
       <c r="H59" s="51"/>
       <c r="I59" s="56" t="str">
-        <v>leetcode.cn/problems/course-schedule/</v>
+        <v>leetcode.cn/problems/number-of-islands/</v>
       </c>
       <c r="J59" s="73"/>
       <c r="K59" s="74" t="n">
         <f>LEN(J59)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J59,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L59" s="96" t="str">
-        <v>核心在于构建映射表(从parent到child),然后记录每个child的入度,当一个child的入读为0的时候,将其加入到queue队列当中,然后遍历这个节点作为parent的所有子节点,将他们的入读减1,然后判断是否有入度为0的元素,如果有那么将其加入到队列中;同时需要注意记录数量的时候应该是当讲一个元素从队列中弹出时,而不是加入时</v>
+      <c r="L59" s="71" t="str">
+        <v>方法一：DFS 方法二：BFS ,对于BFS算法来说,队列的创建放在bfs函数里面,同时队列里面存储的是已经被探索过的岛屿元素,值由1变为0</v>
       </c>
       <c r="M59" s="71"/>
     </row>
-    <row r="60" ht="45.79999923706055" customHeight="1">
+    <row r="60" ht="140" customHeight="1">
       <c r="A60" s="28"/>
-      <c r="B60" s="103" t="str">
-        <v>前缀树</v>
+      <c r="B60" s="102" t="str">
+        <v>多源 BFS</v>
       </c>
       <c r="C60" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="34" t="n">
-        <v>208</v>
+        <v>994</v>
       </c>
       <c r="E60" s="72" t="str">
-        <v>208. 实现 Trie (前缀树)</v>
+        <v>994. 腐烂的橘子</v>
       </c>
       <c r="F60" s="45" t="str">
         <v>中等</v>
@@ -2547,7 +2626,7 @@
       <c r="G60" s="51"/>
       <c r="H60" s="51"/>
       <c r="I60" s="56" t="str">
-        <v>leetcode.cn/problems/implement-trie-prefix-tree/</v>
+        <v>leetcode.cn/problems/rotting-oranges/</v>
       </c>
       <c r="J60" s="73"/>
       <c r="K60" s="74" t="n">
@@ -2555,25 +2634,25 @@
         <v>0</v>
       </c>
       <c r="L60" s="71" t="str">
-        <v>TrieNode节点的构建很关键,对于该节点的属性hashtable来说,存储以某个字符为前缀的其他Tridnode,然后flag属性用于判断某个字符是不是结尾.</v>
-      </c>
-      <c r="M60" s="71"/>
-    </row>
-    <row r="61" ht="78" customHeight="1">
-      <c r="A61" s="28" t="str">
-        <v>回溯</v>
-      </c>
-      <c r="B61" s="103" t="str">
-        <v>排列</v>
+        <v>多源 BFS：先扫描整个网格，将所有腐烂橘子入队并统计新鲜橘子 num；每层处理当前队列长度，对应 1 分钟。新鲜橘子入队时立即标记为腐烂并将 num 减一，避免重复入队。</v>
+      </c>
+      <c r="M60" s="96" t="str">
+        <v>【曾错重点】首次完整遍历网格后、进入 while queue 前，先判断 num == 0（即 if not num），为 0 立即 return 0！不能只在 BFS 内判断：如 [[0]] 没有新鲜橘子，队列也为空，BFS 不执行，会误走末尾 return -1。</v>
+      </c>
+    </row>
+    <row r="61" ht="83.5999984741211" customHeight="1">
+      <c r="A61" s="28"/>
+      <c r="B61" s="102" t="str">
+        <v>拓扑排序</v>
       </c>
       <c r="C61" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="34" t="n">
-        <v>46</v>
+        <v>207</v>
       </c>
       <c r="E61" s="72" t="str">
-        <v>46. 全排列</v>
+        <v>207. 课程表</v>
       </c>
       <c r="F61" s="45" t="str">
         <v>中等</v>
@@ -2581,31 +2660,31 @@
       <c r="G61" s="51"/>
       <c r="H61" s="51"/>
       <c r="I61" s="56" t="str">
-        <v>leetcode.cn/problems/permutations/</v>
+        <v>leetcode.cn/problems/course-schedule/</v>
       </c>
       <c r="J61" s="73"/>
       <c r="K61" s="74" t="n">
         <f>LEN(J61)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J61,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L61" s="71" t="str">
-        <v>（时间复杂度为O(en!)） 在全排列问题当中，始终都是对path这个列表进行处理，如果添加的是path的话只是对原列表的引用，因此当对path进行修改时，也会影响到加入到res当中的列表，正确的做法是添加当前列表的副本…</v>
+      <c r="L61" s="96" t="str">
+        <v>核心在于构建映射表(从parent到child),然后记录每个child的入度,当一个child的入读为0的时候,将其加入到queue队列当中,然后遍历这个节点作为parent的所有子节点,将他们的入读减1,然后判断是否有入度为0的元素,如果有那么将其加入到队列中;同时需要注意记录数量的时候应该是当讲一个元素从队列中弹出时,而不是加入时</v>
       </c>
       <c r="M61" s="71"/>
     </row>
-    <row r="62" ht="78" customHeight="1">
+    <row r="62" ht="45.79999923706055" customHeight="1">
       <c r="A62" s="28"/>
-      <c r="B62" s="103" t="str">
-        <v>子集</v>
+      <c r="B62" s="102" t="str">
+        <v>前缀树</v>
       </c>
       <c r="C62" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D62" s="34" t="n">
-        <v>78</v>
+        <v>208</v>
       </c>
       <c r="E62" s="72" t="str">
-        <v>78. 子集</v>
+        <v>208. 实现 Trie (前缀树)</v>
       </c>
       <c r="F62" s="45" t="str">
         <v>中等</v>
@@ -2613,7 +2692,7 @@
       <c r="G62" s="51"/>
       <c r="H62" s="51"/>
       <c r="I62" s="56" t="str">
-        <v>leetcode.cn/problems/subsets/</v>
+        <v>leetcode.cn/problems/implement-trie-prefix-tree/</v>
       </c>
       <c r="J62" s="73"/>
       <c r="K62" s="74" t="n">
@@ -2621,23 +2700,25 @@
         <v>0</v>
       </c>
       <c r="L62" s="71" t="str">
-        <v>模板一：每个数的选与不选 回溯三问为： 1.当前的操作是什么：是否选择索引值为i的值并将其加入到path中 2.子问题是什么：索引值=i的剩余数的选择问题 3.下一个子问题：索引值=i+1的剩余数的选择问题 模板二：站在…</v>
+        <v>TrieNode节点的构建很关键,对于该节点的属性hashtable来说,存储以某个字符为前缀的其他Tridnode,然后flag属性用于判断某个字符是不是结尾.</v>
       </c>
       <c r="M62" s="71"/>
     </row>
     <row r="63" ht="78" customHeight="1">
-      <c r="A63" s="28"/>
-      <c r="B63" s="103" t="str">
-        <v>组合枚举</v>
+      <c r="A63" s="28" t="str">
+        <v>回溯</v>
+      </c>
+      <c r="B63" s="102" t="str">
+        <v>排列</v>
       </c>
       <c r="C63" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D63" s="34" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="E63" s="72" t="str">
-        <v>17. 电话号码的字母组合</v>
+        <v>46. 全排列</v>
       </c>
       <c r="F63" s="45" t="str">
         <v>中等</v>
@@ -2645,31 +2726,31 @@
       <c r="G63" s="51"/>
       <c r="H63" s="51"/>
       <c r="I63" s="56" t="str">
-        <v>leetcode.cn/problems/letter-combinations-of-a-phone-number/</v>
+        <v>leetcode.cn/problems/permutations/</v>
       </c>
       <c r="J63" s="73"/>
       <c r="K63" s="74" t="n">
         <f>LEN(J63)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J63,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L63" s="71" t="str">
-        <v>对这个题而言，回溯三问为： 1.当前正在进行的操作是什么：枚举第i个数字的字母（需要使用循环达到枚举的效果） 2.子问题是什么：构建索引值大于等于i的字符串 3.下一个子问题是什么：构建索引值大于等于i+1的字符串</v>
+      <c r="L63" s="96" t="str">
+        <v>定长问题,对于这样的问题来说,先构建一个定长的数组用于存储结果,同时注意path[:]而不是path,传递的是副本而不是原件,如果传原件的话后续会被修改;内部循环是for i in s,其中s为集合.</v>
       </c>
       <c r="M63" s="71"/>
     </row>
     <row r="64" ht="78" customHeight="1">
       <c r="A64" s="28"/>
-      <c r="B64" s="103" t="str">
-        <v>组合总和</v>
+      <c r="B64" s="102" t="str">
+        <v>子集</v>
       </c>
       <c r="C64" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D64" s="34" t="n">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="E64" s="72" t="str">
-        <v>39. 组合总和</v>
+        <v>78. 子集</v>
       </c>
       <c r="F64" s="45" t="str">
         <v>中等</v>
@@ -2677,29 +2758,31 @@
       <c r="G64" s="51"/>
       <c r="H64" s="51"/>
       <c r="I64" s="56" t="str">
-        <v>leetcode.cn/problems/combination-sum/</v>
+        <v>leetcode.cn/problems/subsets/</v>
       </c>
       <c r="J64" s="73"/>
       <c r="K64" s="74" t="n">
         <f>LEN(J64)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J64,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L64" s="71" t="str">
-        <v>回溯三问为： 1.当前操作：从大于等于i的索引中选取一个数，索引为j 2.子问题：从大于等于索引i的数组中选数加入到总和中看是否等于target 3.下一个子问题：从大于等于索引j的数组中选数加入到总和中看是否等于tar…</v>
+      <c r="L64" s="96" t="str">
+        <v>不定长问题,通过append与pop操作增加去除path里面的元素,两种解法:1.每个数选与不选 2.枚举选哪个数.注意这两种方法中i的含义不相同,第一种方法中i指的是这个元素的选与不选问题,但是第二种方法中的i指的是从[i,n]范围内容枚举一个数,因此res.append()的位置也有所不同,这一点需要特别注意.</v>
       </c>
       <c r="M64" s="71"/>
     </row>
-    <row r="65" ht="36" customHeight="1">
+    <row r="65" ht="78" customHeight="1">
       <c r="A65" s="28"/>
-      <c r="B65" s="103"/>
+      <c r="B65" s="102" t="str">
+        <v>组合枚举</v>
+      </c>
       <c r="C65" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" s="34" t="n">
-        <v>216</v>
+        <v>17</v>
       </c>
       <c r="E65" s="72" t="str">
-        <v>216. 组合总和 III</v>
+        <v>17. 电话号码的字母组合</v>
       </c>
       <c r="F65" s="45" t="str">
         <v>中等</v>
@@ -2707,31 +2790,34 @@
       <c r="G65" s="51"/>
       <c r="H65" s="51"/>
       <c r="I65" s="56" t="str">
-        <v>leetcode.cn/problems/combination-sum-iii/</v>
+        <v>leetcode.cn/problems/letter-combinations-of-a-phone-number/</v>
       </c>
       <c r="J65" s="73"/>
       <c r="K65" s="74" t="n">
         <f>LEN(J65)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J65,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L65" s="71" t="str">
-        <v>回溯组合：从1~9选k个数和为n；可剪枝（剩余个数不足或和超target）</v>
+      <c r="L65" s="96" t="str">
+        <v>定长问题, 对这个题而言，回溯三问为：
+    1.当前正在进行的操作是什么：枚举第i个数字的字母（需要使用循环达到枚举的效果）
+    2.子问题是什么：构建索引值大于等于i的字符串
+    3.下一个子问题是什么：构建索引值大于等于i+1的字符串</v>
       </c>
       <c r="M65" s="71"/>
     </row>
-    <row r="66" ht="36" customHeight="1">
+    <row r="66" ht="78" customHeight="1">
       <c r="A66" s="28"/>
-      <c r="B66" s="103" t="str">
-        <v>括号构造</v>
+      <c r="B66" s="102" t="str">
+        <v>组合总和</v>
       </c>
       <c r="C66" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D66" s="34" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="E66" s="72" t="str">
-        <v>22. 括号生成</v>
+        <v>39. 组合总和</v>
       </c>
       <c r="F66" s="45" t="str">
         <v>中等</v>
@@ -2739,31 +2825,29 @@
       <c r="G66" s="51"/>
       <c r="H66" s="51"/>
       <c r="I66" s="56" t="str">
-        <v>leetcode.cn/problems/generate-parentheses/</v>
+        <v>leetcode.cn/problems/combination-sum/</v>
       </c>
       <c r="J66" s="73"/>
       <c r="K66" s="74" t="n">
         <f>LEN(J66)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J66,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L66" s="71" t="str">
-        <v>回溯选与不选：左括号数&lt;n才可加'('，右括号数&lt;左括号数才可加')'</v>
+      <c r="L66" s="96" t="str">
+        <v>不定长问题,回溯三问为： 1.当前操作：从大于等于i的索引中选取一个数，索引为j 2.子问题：从大于等于索引i的数组中选数加入到总和中看是否等于target 3.下一个子问题：从大于等于索引j的数组中选数加入到总和中看是否等于target</v>
       </c>
       <c r="M66" s="71"/>
     </row>
-    <row r="67" ht="64" customHeight="1">
+    <row r="67" ht="45.79999923706055" customHeight="1">
       <c r="A67" s="28"/>
-      <c r="B67" s="103" t="str">
-        <v>分割</v>
-      </c>
+      <c r="B67" s="102"/>
       <c r="C67" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D67" s="34" t="n">
-        <v>131</v>
+        <v>216</v>
       </c>
       <c r="E67" s="72" t="str">
-        <v>131. 分割回文串</v>
+        <v>216. 组合总和 III</v>
       </c>
       <c r="F67" s="45" t="str">
         <v>中等</v>
@@ -2771,65 +2855,63 @@
       <c r="G67" s="51"/>
       <c r="H67" s="51"/>
       <c r="I67" s="56" t="str">
-        <v>leetcode.cn/problems/palindrome-partitioning/</v>
+        <v>leetcode.cn/problems/combination-sum-iii/</v>
       </c>
       <c r="J67" s="73"/>
       <c r="K67" s="74" t="n">
         <f>LEN(J67)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J67,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L67" s="71" t="str">
-        <v>回溯三问为: 1.当前操作：从索引i开始找一个[i,j]的字符串，判断它是不是回文串 2.子问题：从当前索引开始查找回文子串（枚举从i开始的字符串） 3.下一个子问题：从索引j+1开始查找回文串</v>
+      <c r="L67" s="96" t="str">
+        <v>不定长问题,回溯组合：从1~9选k个数和为n；可剪枝（剩余个数不足或和超target）;if t &lt; 0 or t &gt; (i + i -d + 1) * d // 2,dfs里面先判断这个,后面再接d == 0</v>
       </c>
       <c r="M67" s="71"/>
     </row>
     <row r="68" ht="36" customHeight="1">
       <c r="A68" s="28"/>
-      <c r="B68" s="103" t="str">
-        <v>排列与约束</v>
+      <c r="B68" s="102" t="str">
+        <v>括号构造</v>
       </c>
       <c r="C68" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D68" s="34" t="n">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="E68" s="72" t="str">
-        <v>51. N 皇后</v>
-      </c>
-      <c r="F68" s="91" t="str">
-        <v>困难</v>
+        <v>22. 括号生成</v>
+      </c>
+      <c r="F68" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G68" s="51"/>
       <c r="H68" s="51"/>
       <c r="I68" s="56" t="str">
-        <v>leetcode.cn/problems/n-queens/</v>
+        <v>leetcode.cn/problems/generate-parentheses/</v>
       </c>
       <c r="J68" s="73"/>
       <c r="K68" s="74" t="n">
         <f>LEN(J68)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J68,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L68" s="71" t="str">
-        <v>回溯逐行放皇后；用列、主对角线(i-j)、副对角线(i+j)集合剪枝</v>
+      <c r="L68" s="96" t="str">
+        <v>回溯选与不选,定长问题：左括号数&lt;n才可加'('，右括号数&lt;左括号数才可加')';能加左就加左括号,不行在右括号</v>
       </c>
       <c r="M68" s="71"/>
     </row>
-    <row r="69" ht="36" customHeight="1">
-      <c r="A69" s="28" t="str">
-        <v>二分查找</v>
-      </c>
-      <c r="B69" s="103" t="str">
-        <v>二维有序查找</v>
+    <row r="69" ht="105" customHeight="1">
+      <c r="A69" s="28"/>
+      <c r="B69" s="102" t="str">
+        <v>网格搜索</v>
       </c>
       <c r="C69" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D69" s="34" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E69" s="72" t="str">
-        <v>74. 搜索二维矩阵</v>
+        <v>79. 单词搜索</v>
       </c>
       <c r="F69" s="45" t="str">
         <v>中等</v>
@@ -2837,7 +2919,7 @@
       <c r="G69" s="51"/>
       <c r="H69" s="51"/>
       <c r="I69" s="56" t="str">
-        <v>leetcode.cn/problems/search-a-2d-matrix/</v>
+        <v>leetcode.cn/problems/word-search/</v>
       </c>
       <c r="J69" s="73"/>
       <c r="K69" s="74" t="n">
@@ -2845,23 +2927,25 @@
         <v>0</v>
       </c>
       <c r="L69" s="71" t="str">
-        <v>把二维矩阵拉成一维即可,mid对应矩阵的位置为[mid//column][mid%column]</v>
-      </c>
-      <c r="M69" s="71"/>
-    </row>
-    <row r="70" ht="50" customHeight="1">
+        <v>网格回溯：从每个格子出发匹配 word[k:]，当前字符匹配后标记访问，枚举四邻格递归匹配 k+1；失败后恢复现场，同一路径不能重复使用格子。先比较字符频次剪枝，必要时反转单词，从较稀少的端点开始搜索。</v>
+      </c>
+      <c r="M69" s="71" t="str">
+        <v>注意区分下标：子集/组合正序且不可重复选时，选 j 后递归从 j+1 开始；单词搜索推进的是字符下标 k+1，同时移动到相邻未访问格子。</v>
+      </c>
+    </row>
+    <row r="70" ht="64" customHeight="1">
       <c r="A70" s="28"/>
-      <c r="B70" s="103" t="str">
-        <v>边界查找</v>
+      <c r="B70" s="102" t="str">
+        <v>分割</v>
       </c>
       <c r="C70" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D70" s="34" t="n">
-        <v>34</v>
+        <v>131</v>
       </c>
       <c r="E70" s="72" t="str">
-        <v>34. 在排序数组中查找元素的第一个和最后一个位置</v>
+        <v>131. 分割回文串</v>
       </c>
       <c r="F70" s="45" t="str">
         <v>中等</v>
@@ -2869,39 +2953,39 @@
       <c r="G70" s="51"/>
       <c r="H70" s="51"/>
       <c r="I70" s="56" t="str">
-        <v>leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/</v>
+        <v>leetcode.cn/problems/palindrome-partitioning/</v>
       </c>
       <c r="J70" s="73"/>
       <c r="K70" s="74" t="n">
         <f>LEN(J70)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J70,"√",""),"×",""),"✓",""))</f>
         <v>0</v>
       </c>
-      <c r="L70" s="71" t="str">
-        <v>使用lower_bound方法,lower_bound(x)找到第一个大于等于x的值,使用lower_bound(x+1)-1找到最后一个大于等于0的值,然后再判断是不是目标值;额外关注left的取值范围为[0,len(nums)]</v>
+      <c r="L70" s="96" t="str">
+        <v>不定长问题,回溯三问为: 1.当前操作：从索引i开始找一个[i,j]的字符串，判断它是不是回文串 2.子问题：从当前索引开始查找回文子串（枚举从i开始的字符串） 3.下一个子问题：从索引j+1开始查找回文串</v>
       </c>
       <c r="M70" s="71"/>
     </row>
-    <row r="71" ht="45.79999923706055" customHeight="1">
+    <row r="71" ht="36" customHeight="1">
       <c r="A71" s="28"/>
-      <c r="B71" s="103" t="str">
-        <v>旋转数组与局部性质</v>
+      <c r="B71" s="102" t="str">
+        <v>排列与约束</v>
       </c>
       <c r="C71" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D71" s="34" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="E71" s="72" t="str">
-        <v>33. 搜索旋转排序数组</v>
-      </c>
-      <c r="F71" s="45" t="str">
-        <v>中等</v>
+        <v>51. N 皇后</v>
+      </c>
+      <c r="F71" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G71" s="51"/>
       <c r="H71" s="51"/>
       <c r="I71" s="56" t="str">
-        <v>leetcode.cn/problems/search-in-rotated-sorted-array/</v>
+        <v>leetcode.cn/problems/n-queens/</v>
       </c>
       <c r="J71" s="73"/>
       <c r="K71" s="74" t="n">
@@ -2909,21 +2993,25 @@
         <v>0</v>
       </c>
       <c r="L71" s="71" t="str">
-        <v>红蓝染色/二分：判断mid在target的左侧还是右侧,然后进行染色,最终返回的left就应该是target出现的位置,但同时需要进行判断验证left的合理性.</v>
+        <v>定长问题,回溯逐行放皇后；用列、主对角线(i-j)、副对角线(i+j)集合剪枝</v>
       </c>
       <c r="M71" s="71"/>
     </row>
-    <row r="72" ht="64" customHeight="1">
-      <c r="A72" s="28"/>
-      <c r="B72" s="103"/>
+    <row r="72" ht="36" customHeight="1">
+      <c r="A72" s="28" t="str">
+        <v>二分查找</v>
+      </c>
+      <c r="B72" s="102" t="str">
+        <v>二维有序查找</v>
+      </c>
       <c r="C72" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D72" s="34" t="n">
-        <v>153</v>
+        <v>74</v>
       </c>
       <c r="E72" s="72" t="str">
-        <v>153. 寻找旋转排序数组中的最小值</v>
+        <v>74. 搜索二维矩阵</v>
       </c>
       <c r="F72" s="45" t="str">
         <v>中等</v>
@@ -2931,7 +3019,7 @@
       <c r="G72" s="51"/>
       <c r="H72" s="51"/>
       <c r="I72" s="56" t="str">
-        <v>leetcode.cn/problems/find-minimum-in-rotated-sorted-array/</v>
+        <v>leetcode.cn/problems/search-a-2d-matrix/</v>
       </c>
       <c r="J72" s="73"/>
       <c r="K72" s="74" t="n">
@@ -2939,21 +3027,23 @@
         <v>0</v>
       </c>
       <c r="L72" s="71" t="str">
-        <v>旋转数组左半部分的元素一定大于右半部分，令中间值与末尾值进行比较，如果中间值大于end，意味着中间值及其左侧的值都在最小值的左侧，染成红色，否则为蓝色，蓝色代表着最小值及其右侧。</v>
+        <v>把二维矩阵拉成一维即可,mid对应矩阵的位置为[mid//column][mid%column]</v>
       </c>
       <c r="M72" s="71"/>
     </row>
-    <row r="73" ht="36" customHeight="1">
+    <row r="73" ht="50" customHeight="1">
       <c r="A73" s="28"/>
-      <c r="B73" s="103"/>
+      <c r="B73" s="102" t="str">
+        <v>边界查找</v>
+      </c>
       <c r="C73" s="34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D73" s="34" t="n">
-        <v>162</v>
+        <v>34</v>
       </c>
       <c r="E73" s="72" t="str">
-        <v>162. 寻找峰值</v>
+        <v>34. 在排序数组中查找元素的第一个和最后一个位置</v>
       </c>
       <c r="F73" s="45" t="str">
         <v>中等</v>
@@ -2961,7 +3051,7 @@
       <c r="G73" s="51"/>
       <c r="H73" s="51"/>
       <c r="I73" s="56" t="str">
-        <v>leetcode.cn/problems/find-peak-element/</v>
+        <v>leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/</v>
       </c>
       <c r="J73" s="73"/>
       <c r="K73" s="74" t="n">
@@ -2969,31 +3059,31 @@
         <v>0</v>
       </c>
       <c r="L73" s="71" t="str">
-        <v>红蓝染色：nums[mid]&lt;nums[mid+1] 说明峰在右侧，否则峰在左侧</v>
+        <v>使用lower_bound方法,lower_bound(x)找到第一个大于等于x的值,使用lower_bound(x+1)-1找到最后一个大于等于0的值,然后再判断是不是目标值;额外关注left的取值范围为[0,len(nums)]</v>
       </c>
       <c r="M73" s="71"/>
     </row>
     <row r="74" ht="45.79999923706055" customHeight="1">
       <c r="A74" s="28"/>
-      <c r="B74" s="103" t="str">
-        <v>中位数划分</v>
+      <c r="B74" s="102" t="str">
+        <v>旋转数组与局部性质</v>
       </c>
       <c r="C74" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D74" s="34" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="E74" s="72" t="str">
-        <v>4. 寻找两个正序数组的中位数</v>
-      </c>
-      <c r="F74" s="91" t="str">
-        <v>困难</v>
+        <v>33. 搜索旋转排序数组</v>
+      </c>
+      <c r="F74" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G74" s="51"/>
       <c r="H74" s="51"/>
       <c r="I74" s="56" t="str">
-        <v>leetcode.cn/problems/median-of-two-sorted-arrays/</v>
+        <v>leetcode.cn/problems/search-in-rotated-sorted-array/</v>
       </c>
       <c r="J74" s="73"/>
       <c r="K74" s="74" t="n">
@@ -3001,25 +3091,21 @@
         <v>0</v>
       </c>
       <c r="L74" s="71" t="str">
-        <v>二分排除：在较短数组上二分划分，保证左半最大&lt;右半最小；注意奇偶长度中位数处理;对于左侧来说,存在a[i]&lt;=b[j+1],右侧则是a[i]&gt;b[j+1</v>
+        <v>红蓝染色/二分：判断mid在target的左侧还是右侧,然后进行染色,最终返回的left就应该是target出现的位置,但同时需要进行判断验证left的合理性.</v>
       </c>
       <c r="M74" s="71"/>
     </row>
-    <row r="75" ht="36" customHeight="1">
-      <c r="A75" s="28" t="str">
-        <v>栈</v>
-      </c>
-      <c r="B75" s="103" t="str">
-        <v>辅助栈</v>
-      </c>
+    <row r="75" ht="64" customHeight="1">
+      <c r="A75" s="28"/>
+      <c r="B75" s="102"/>
       <c r="C75" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D75" s="34" t="n">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E75" s="72" t="str">
-        <v>155. 最小栈</v>
+        <v>153. 寻找旋转排序数组中的最小值</v>
       </c>
       <c r="F75" s="45" t="str">
         <v>中等</v>
@@ -3027,7 +3113,7 @@
       <c r="G75" s="51"/>
       <c r="H75" s="51"/>
       <c r="I75" s="56" t="str">
-        <v>leetcode.cn/problems/min-stack/</v>
+        <v>leetcode.cn/problems/find-minimum-in-rotated-sorted-array/</v>
       </c>
       <c r="J75" s="73"/>
       <c r="K75" s="74" t="n">
@@ -3035,23 +3121,21 @@
         <v>0</v>
       </c>
       <c r="L75" s="71" t="str">
-        <v>辅助栈同步压入当前最小值；或每个元素存(值, 当前最小值)</v>
+        <v>旋转数组左半部分的元素一定大于右半部分，令中间值与末尾值进行比较，如果中间值大于end，意味着中间值及其左侧的值都在最小值的左侧，染成红色，否则为蓝色，蓝色代表着最小值及其右侧。</v>
       </c>
       <c r="M75" s="71"/>
     </row>
-    <row r="76" ht="78" customHeight="1">
+    <row r="76" ht="36" customHeight="1">
       <c r="A76" s="28"/>
-      <c r="B76" s="103" t="str">
-        <v>嵌套解析</v>
-      </c>
+      <c r="B76" s="102"/>
       <c r="C76" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D76" s="34" t="n">
-        <v>394</v>
+        <v>162</v>
       </c>
       <c r="E76" s="72" t="str">
-        <v>394. 字符串解码</v>
+        <v>162. 寻找峰值</v>
       </c>
       <c r="F76" s="45" t="str">
         <v>中等</v>
@@ -3059,7 +3143,7 @@
       <c r="G76" s="51"/>
       <c r="H76" s="51"/>
       <c r="I76" s="56" t="str">
-        <v>leetcode.cn/problems/decode-string/</v>
+        <v>leetcode.cn/problems/find-peak-element/</v>
       </c>
       <c r="J76" s="73"/>
       <c r="K76" s="74" t="n">
@@ -3067,31 +3151,31 @@
         <v>0</v>
       </c>
       <c r="L76" s="71" t="str">
-        <v>此题的巧妙之处在于使用currsum与currstr来存储会遇到的数字与字符，而不是直接将其加入到栈中，正确的做法是当需要二者入栈的时候，处理到新的字符串（即遇到[时）再将其入栈。 char.isdigit()用来判断一…</v>
+        <v>红蓝染色：nums[mid]&lt;nums[mid+1] 说明峰在右侧，否则峰在左侧</v>
       </c>
       <c r="M76" s="71"/>
     </row>
-    <row r="77" ht="78" customHeight="1">
+    <row r="77" ht="45.79999923706055" customHeight="1">
       <c r="A77" s="28"/>
-      <c r="B77" s="103" t="str">
-        <v>单调栈</v>
+      <c r="B77" s="102" t="str">
+        <v>中位数划分</v>
       </c>
       <c r="C77" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D77" s="34" t="n">
-        <v>739</v>
+        <v>4</v>
       </c>
       <c r="E77" s="72" t="str">
-        <v>739. 每日温度</v>
-      </c>
-      <c r="F77" s="45" t="str">
-        <v>中等</v>
+        <v>4. 寻找两个正序数组的中位数</v>
+      </c>
+      <c r="F77" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G77" s="51"/>
       <c r="H77" s="51"/>
       <c r="I77" s="56" t="str">
-        <v>leetcode.cn/problems/daily-temperatures/</v>
+        <v>leetcode.cn/problems/median-of-two-sorted-arrays/</v>
       </c>
       <c r="J77" s="73"/>
       <c r="K77" s="74" t="n">
@@ -3099,29 +3183,33 @@
         <v>0</v>
       </c>
       <c r="L77" s="71" t="str">
-        <v>上一个更大更小是通过单调栈的属性判断出来的，下一个更大更小是通过while循环中的比较判断出来的 判断单调栈是递增还是递减就看在什么情况下会弹栈就行 此题的求解要特别留意数组中每个元素的索引值的作用，用索引值相减来得到天…</v>
+        <v>二分排除：在较短数组上二分划分，保证左半最大&lt;右半最小；注意奇偶长度中位数处理;对于左侧来说,存在a[i]&lt;=b[j+1],右侧则是a[i]&gt;b[j+1</v>
       </c>
       <c r="M77" s="71"/>
     </row>
     <row r="78" ht="36" customHeight="1">
-      <c r="A78" s="28"/>
-      <c r="B78" s="103"/>
+      <c r="A78" s="28" t="str">
+        <v>栈</v>
+      </c>
+      <c r="B78" s="102" t="str">
+        <v>辅助栈</v>
+      </c>
       <c r="C78" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" s="34" t="n">
-        <v>84</v>
+        <v>155</v>
       </c>
       <c r="E78" s="72" t="str">
-        <v>84. 柱状图中最大的矩形</v>
-      </c>
-      <c r="F78" s="91" t="str">
-        <v>困难</v>
+        <v>155. 最小栈</v>
+      </c>
+      <c r="F78" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G78" s="51"/>
       <c r="H78" s="51"/>
       <c r="I78" s="56" t="str">
-        <v>leetcode.cn/problems/largest-rectangle-in-histogram/</v>
+        <v>leetcode.cn/problems/min-stack/</v>
       </c>
       <c r="J78" s="73"/>
       <c r="K78" s="74" t="n">
@@ -3129,91 +3217,93 @@
         <v>0</v>
       </c>
       <c r="L78" s="71" t="str">
-        <v>思想：枚举每个高度，找到它左右两边最小的值 记住两个-1操作</v>
+        <v>辅助栈同步压入当前最小值；或每个元素存(值, 当前最小值)</v>
       </c>
       <c r="M78" s="71"/>
     </row>
-    <row r="79" ht="36" customHeight="1">
-      <c r="A79" s="28" t="str">
-        <v>堆</v>
-      </c>
-      <c r="B79" s="103" t="str">
-        <v>第K大与快速选择</v>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="28"/>
+      <c r="B79" s="102" t="str">
+        <v>括号匹配</v>
       </c>
       <c r="C79" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D79" s="34" t="n">
-        <v>215</v>
+        <v>20</v>
       </c>
       <c r="E79" s="72" t="str">
-        <v>215. 数组中的第 K 个最大元素</v>
-      </c>
-      <c r="F79" s="45" t="str">
-        <v>中等</v>
+        <v>20.有效括号</v>
+      </c>
+      <c r="F79" s="80" t="str">
+        <v>简单</v>
       </c>
       <c r="G79" s="51"/>
       <c r="H79" s="51"/>
       <c r="I79" s="56" t="str">
-        <v>leetcode.cn/problems/kth-largest-element-in-an-array/</v>
-      </c>
-      <c r="J79" s="73"/>
+        <v>leetcode.cn/problems/valid-parentheses/</v>
+      </c>
+      <c r="J79" s="73" t="str">
+        <v>×</v>
+      </c>
       <c r="K79" s="74" t="n">
         <f>LEN(J79)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J79,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" s="71" t="str">
-        <v>快速选择partition（随机pivot）期望O(n)；或维护大小为k的小顶堆</v>
+        <v>使用stack保存各种左括号,当遇到一个右括号的时候,如果stack为空或者说stack.pop()与右括号不匹配的话,那么返回False,请注意判断条件里面的stack.pop(),遇到一个右括号,无论能不能匹配,都要弹出</v>
       </c>
       <c r="M79" s="71"/>
     </row>
     <row r="80" ht="78" customHeight="1">
       <c r="A80" s="28"/>
-      <c r="B80" s="103" t="str">
-        <v>对顶堆</v>
+      <c r="B80" s="102" t="str">
+        <v>嵌套解析</v>
       </c>
       <c r="C80" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D80" s="34" t="n">
-        <v>295</v>
+        <v>394</v>
       </c>
       <c r="E80" s="72" t="str">
-        <v>295. 数据流的中位数</v>
-      </c>
-      <c r="F80" s="91" t="str">
-        <v>困难</v>
+        <v>394. 字符串解码</v>
+      </c>
+      <c r="F80" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G80" s="51"/>
       <c r="H80" s="51"/>
       <c r="I80" s="56" t="str">
-        <v>leetcode.cn/problems/find-median-from-data-stream/</v>
-      </c>
-      <c r="J80" s="73"/>
+        <v>leetcode.cn/problems/decode-string/</v>
+      </c>
+      <c r="J80" s="73" t="str">
+        <v>××</v>
+      </c>
       <c r="K80" s="74" t="n">
         <f>LEN(J80)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J80,"√",""),"×",""),"✓",""))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L80" s="71" t="str">
-        <v>此题的思路时使用最大堆与最小堆存储数据，但因为python只有最小堆，因此采用存储相反数的形式来实现最大堆，取出时记得将数取反即可。 当左右堆大小相等的时候，不要直接向左堆中加入数据，应该先加入到右堆中，然后取出新的右堆…</v>
-      </c>
-      <c r="M80" s="71"/>
-    </row>
-    <row r="81" ht="36" customHeight="1">
-      <c r="A81" s="28" t="str">
-        <v>贪心算法</v>
-      </c>
-      <c r="B81" s="103" t="str">
-        <v>股票买卖（状态机DP扩展）</v>
+        <v>使用[来进行当前字符串以及下一个字符串次数的保存,使用]取出当前字符串出现的次数以及上一个字符串进行拼接,curr_num 保存的是当前层的重复次数,curr_str保存的是当前层正在构造的字符串</v>
+      </c>
+      <c r="M80" s="71" t="str">
+        <v>else条件为:curr_str += char</v>
+      </c>
+    </row>
+    <row r="81" ht="78" customHeight="1">
+      <c r="A81" s="28"/>
+      <c r="B81" s="102" t="str">
+        <v>单调栈</v>
       </c>
       <c r="C81" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D81" s="34" t="n">
-        <v>122</v>
+        <v>739</v>
       </c>
       <c r="E81" s="72" t="str">
-        <v>122. 买卖股票的最佳时机 II</v>
+        <v>739. 每日温度</v>
       </c>
       <c r="F81" s="45" t="str">
         <v>中等</v>
@@ -3221,7 +3311,7 @@
       <c r="G81" s="51"/>
       <c r="H81" s="51"/>
       <c r="I81" s="56" t="str">
-        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/</v>
+        <v>leetcode.cn/problems/daily-temperatures/</v>
       </c>
       <c r="J81" s="73"/>
       <c r="K81" s="74" t="n">
@@ -3229,21 +3319,21 @@
         <v>0</v>
       </c>
       <c r="L81" s="71" t="str">
-        <v>状态机DP：dp[i][0]不持有、dp[i][1]持有；不限制交易次数，答案=dp[n-1][0]</v>
+        <v>单调递减的栈,对于这种问题来说,每个元素都会入栈,但是不是所有元素都会出栈,同时因为是单减栈,如果新的元素比旧元素要大,因为新元素是一定要入栈的,因此就需要将所有比新元素小的元素出栈才能保证栈的单调递减属性.</v>
       </c>
       <c r="M81" s="71"/>
     </row>
-    <row r="82" ht="36" customHeight="1">
+    <row r="82" ht="58.400001525878906" customHeight="1">
       <c r="A82" s="28"/>
-      <c r="B82" s="103"/>
+      <c r="B82" s="102"/>
       <c r="C82" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D82" s="34" t="n">
-        <v>188</v>
+        <v>84</v>
       </c>
       <c r="E82" s="72" t="str">
-        <v>188. 买卖股票的最佳时机 IV</v>
+        <v>84. 柱状图中最大的矩形</v>
       </c>
       <c r="F82" s="91" t="str">
         <v>困难</v>
@@ -3251,7 +3341,7 @@
       <c r="G82" s="51"/>
       <c r="H82" s="51"/>
       <c r="I82" s="56" t="str">
-        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/</v>
+        <v>leetcode.cn/problems/largest-rectangle-in-histogram/</v>
       </c>
       <c r="J82" s="73"/>
       <c r="K82" s="74" t="n">
@@ -3259,21 +3349,25 @@
         <v>0</v>
       </c>
       <c r="L82" s="71" t="str">
-        <v>至多k笔：dp[i][j][0/1]，j为已交易次数；j&lt;0不合法，需k+2维空间</v>
+        <v>单增栈,思想：枚举每个高度，找到它左右两边最小的值 记住两个-1操作;令每一个元素都能够弹出,同时计算以他为最小高度时矩阵的面积;left以及right指向的值比这个元素还要小,因此使用right-left-1操作,不包含left以及right处的值.</v>
       </c>
       <c r="M82" s="71"/>
     </row>
-    <row r="83" ht="36" customHeight="1">
-      <c r="A83" s="28"/>
-      <c r="B83" s="103"/>
+    <row r="83" ht="58.400001525878906" customHeight="1">
+      <c r="A83" s="28" t="str">
+        <v>堆</v>
+      </c>
+      <c r="B83" s="102" t="str">
+        <v>第K大与快速选择</v>
+      </c>
       <c r="C83" s="34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D83" s="34" t="n">
-        <v>309</v>
+        <v>215</v>
       </c>
       <c r="E83" s="72" t="str">
-        <v>309. 买卖股票的最佳时机含冷冻期</v>
+        <v>215. 数组中的第 K 个最大元素</v>
       </c>
       <c r="F83" s="45" t="str">
         <v>中等</v>
@@ -3281,7 +3375,7 @@
       <c r="G83" s="51"/>
       <c r="H83" s="51"/>
       <c r="I83" s="56" t="str">
-        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/</v>
+        <v>leetcode.cn/problems/kth-largest-element-in-an-array/</v>
       </c>
       <c r="J83" s="73"/>
       <c r="K83" s="74" t="n">
@@ -3289,23 +3383,23 @@
         <v>0</v>
       </c>
       <c r="L83" s="71" t="str">
-        <v>含冷冻期：买入只能从两天前(f2)转移；f0卖出/f1持有/f2冷冻 滚动更新</v>
+        <v>使用快速选择算法,对于partition函数来说,维护两个闭指针,对于left来说,其左侧元素都是小于等于pivot的,对于右侧指针来说反之,因此在进行完一次函数执行后,我们能够知道pivot这个元素所处的位置,从而不断地进行判断最终找到第k大的元素.</v>
       </c>
       <c r="M83" s="71"/>
     </row>
-    <row r="84" ht="36" customHeight="1">
+    <row r="84" ht="60" customHeight="1">
       <c r="A84" s="28"/>
-      <c r="B84" s="103" t="str">
-        <v>覆盖范围</v>
+      <c r="B84" s="102" t="str">
+        <v>Top K 高频</v>
       </c>
       <c r="C84" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D84" s="34" t="n">
-        <v>55</v>
+        <v>347</v>
       </c>
       <c r="E84" s="72" t="str">
-        <v>55. 跳跃游戏</v>
+        <v>347.前k个高频元素</v>
       </c>
       <c r="F84" s="45" t="str">
         <v>中等</v>
@@ -3313,7 +3407,7 @@
       <c r="G84" s="51"/>
       <c r="H84" s="51"/>
       <c r="I84" s="56" t="str">
-        <v>leetcode.cn/problems/jump-game/</v>
+        <v>leetcode.cn/problems/top-k-frequent-elements/</v>
       </c>
       <c r="J84" s="73"/>
       <c r="K84" s="74" t="n">
@@ -3321,29 +3415,31 @@
         <v>0</v>
       </c>
       <c r="L84" s="71" t="str">
-        <v>贪心：维护能到达的最远位置reach，遍历时更新；reach&gt;=n-1即成功</v>
+        <v>先用哈希表统计每个元素的出现频次，再用小顶堆维护频次最高的 K 个元素；也可按频次分桶。</v>
       </c>
       <c r="M84" s="71"/>
     </row>
-    <row r="85" ht="36" customHeight="1">
+    <row r="85" ht="78" customHeight="1">
       <c r="A85" s="28"/>
-      <c r="B85" s="103"/>
+      <c r="B85" s="102" t="str">
+        <v>对顶堆</v>
+      </c>
       <c r="C85" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D85" s="34" t="n">
-        <v>45</v>
+        <v>295</v>
       </c>
       <c r="E85" s="72" t="str">
-        <v>45. 跳跃游戏 II</v>
-      </c>
-      <c r="F85" s="45" t="str">
-        <v>中等</v>
+        <v>295. 数据流的中位数</v>
+      </c>
+      <c r="F85" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G85" s="51"/>
       <c r="H85" s="51"/>
       <c r="I85" s="56" t="str">
-        <v>leetcode.cn/problems/jump-game-ii/</v>
+        <v>leetcode.cn/problems/find-median-from-data-stream/</v>
       </c>
       <c r="J85" s="73"/>
       <c r="K85" s="74" t="n">
@@ -3351,25 +3447,25 @@
         <v>0</v>
       </c>
       <c r="L85" s="71" t="str">
-        <v>条件:从头走到尾 最小子序列:走过的步数最少，涉及到的元素的个数最少，也即最小子序列</v>
+        <v>self.left为最大堆,self.right为最小堆,因为python只有最小堆实现,因此对于最大堆来说,通过加入弹出nums的相反数实现最大堆效果,同时始终保证len(left)最多比len(right)大1与最大堆的最大值比最小堆的最小值还要小这个特点.</v>
       </c>
       <c r="M85" s="71"/>
     </row>
-    <row r="86" ht="64" customHeight="1">
+    <row r="86" ht="36" customHeight="1">
       <c r="A86" s="28" t="str">
-        <v>动态规划</v>
-      </c>
-      <c r="B86" s="103" t="str">
-        <v>计数递推</v>
+        <v>贪心算法</v>
+      </c>
+      <c r="B86" s="102" t="str">
+        <v>股票买卖（状态机DP扩展）</v>
       </c>
       <c r="C86" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D86" s="34" t="n">
-        <v>2266</v>
+        <v>122</v>
       </c>
       <c r="E86" s="72" t="str">
-        <v>2266. 统计打字方案数</v>
+        <v>122. 买卖股票的最佳时机 II</v>
       </c>
       <c r="F86" s="45" t="str">
         <v>中等</v>
@@ -3377,7 +3473,7 @@
       <c r="G86" s="51"/>
       <c r="H86" s="51"/>
       <c r="I86" s="56" t="str">
-        <v>leetcode.cn/problems/count-number-of-texts/</v>
+        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/</v>
       </c>
       <c r="J86" s="73"/>
       <c r="K86" s="74" t="n">
@@ -3385,31 +3481,29 @@
         <v>0</v>
       </c>
       <c r="L86" s="71" t="str">
-        <v>组合计数+DP：连续相同数字分组，每组按键方案满足dp[i]=dp[i-1]+dp[i-2]+dp[i-3]+(4字母键再加dp[i-4])；结果取模1e9+7</v>
+        <v>状态机DP：dp[i][0]不持有、dp[i][1]持有；不限制交易次数，答案=dp[n-1][0]</v>
       </c>
       <c r="M86" s="71"/>
     </row>
-    <row r="87" ht="78" customHeight="1">
+    <row r="87" ht="36" customHeight="1">
       <c r="A87" s="28"/>
-      <c r="B87" s="103" t="str">
-        <v>线性递推</v>
-      </c>
+      <c r="B87" s="102"/>
       <c r="C87" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D87" s="34" t="n">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="E87" s="72" t="str">
-        <v>198. 打家劫舍</v>
-      </c>
-      <c r="F87" s="45" t="str">
-        <v>中等</v>
+        <v>188. 买卖股票的最佳时机 IV</v>
+      </c>
+      <c r="F87" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G87" s="51"/>
       <c r="H87" s="51"/>
       <c r="I87" s="56" t="str">
-        <v>leetcode.cn/problems/house-robber/</v>
+        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/</v>
       </c>
       <c r="J87" s="73"/>
       <c r="K87" s="74" t="n">
@@ -3417,23 +3511,21 @@
         <v>0</v>
       </c>
       <c r="L87" s="71" t="str">
-        <v>使用动态规划的方法，而对于偷前i个房子的问题，它的最大值为偷取前i-1个房子与偷取前i-2个房子加上当前房子的价格的最大值，因此实际上只需使用两个变量记录i-1与i-2的值，不需要使用一个列表来完整记录每个索引的最大值</v>
+        <v>至多k笔：dp[i][j][0/1]，j为已交易次数；j&lt;0不合法，需k+2维空间</v>
       </c>
       <c r="M87" s="71"/>
     </row>
-    <row r="88" ht="50" customHeight="1">
+    <row r="88" ht="36" customHeight="1">
       <c r="A88" s="28"/>
-      <c r="B88" s="103" t="str">
-        <v>背包</v>
-      </c>
+      <c r="B88" s="102"/>
       <c r="C88" s="34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D88" s="34" t="n">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="E88" s="72" t="str">
-        <v>322. 零钱兑换</v>
+        <v>309. 买卖股票的最佳时机含冷冻期</v>
       </c>
       <c r="F88" s="45" t="str">
         <v>中等</v>
@@ -3441,7 +3533,7 @@
       <c r="G88" s="51"/>
       <c r="H88" s="51"/>
       <c r="I88" s="56" t="str">
-        <v>leetcode.cn/problems/coin-change/</v>
+        <v>leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/</v>
       </c>
       <c r="J88" s="73"/>
       <c r="K88" s="74" t="n">
@@ -3449,21 +3541,23 @@
         <v>0</v>
       </c>
       <c r="L88" s="71" t="str">
-        <v>完全背包：f[i]=min(f[i], f[i-coin]+1)；f初始化为inf、f[0]=0，返回时判断是否可达</v>
+        <v>含冷冻期：买入只能从两天前(f2)转移；f0卖出/f1持有/f2冷冻 滚动更新</v>
       </c>
       <c r="M88" s="71"/>
     </row>
     <row r="89" ht="36" customHeight="1">
       <c r="A89" s="28"/>
-      <c r="B89" s="103"/>
+      <c r="B89" s="102" t="str">
+        <v>覆盖范围</v>
+      </c>
       <c r="C89" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D89" s="34" t="n">
-        <v>494</v>
+        <v>55</v>
       </c>
       <c r="E89" s="72" t="str">
-        <v>494. 目标和</v>
+        <v>309. 买卖股票的最佳时机含冷冻期</v>
       </c>
       <c r="F89" s="45" t="str">
         <v>中等</v>
@@ -3471,7 +3565,7 @@
       <c r="G89" s="51"/>
       <c r="H89" s="51"/>
       <c r="I89" s="56" t="str">
-        <v>leetcode.cn/problems/target-sum/</v>
+        <v>leetcode.cn/problems/jump-game/</v>
       </c>
       <c r="J89" s="73"/>
       <c r="K89" s="74" t="n">
@@ -3479,23 +3573,21 @@
         <v>0</v>
       </c>
       <c r="L89" s="71" t="str">
-        <v>01背包：target += sum(nums)，求恰好等于target的方案数（每个数选或不选）</v>
+        <v>贪心：维护能到达的最远位置reach，遍历时更新；reach&gt;=n-1即成功</v>
       </c>
       <c r="M89" s="71"/>
     </row>
     <row r="90" ht="36" customHeight="1">
       <c r="A90" s="28"/>
-      <c r="B90" s="103" t="str">
-        <v>字符串划分</v>
-      </c>
+      <c r="B90" s="102"/>
       <c r="C90" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D90" s="34" t="n">
-        <v>139</v>
+        <v>45</v>
       </c>
       <c r="E90" s="72" t="str">
-        <v>139. 单词拆分</v>
+        <v>45. 跳跃游戏 II</v>
       </c>
       <c r="F90" s="45" t="str">
         <v>中等</v>
@@ -3503,7 +3595,7 @@
       <c r="G90" s="51"/>
       <c r="H90" s="51"/>
       <c r="I90" s="56" t="str">
-        <v>leetcode.cn/problems/word-break/</v>
+        <v>leetcode.cn/problems/jump-game-ii/</v>
       </c>
       <c r="J90" s="73"/>
       <c r="K90" s="74" t="n">
@@ -3511,23 +3603,25 @@
         <v>0</v>
       </c>
       <c r="L90" s="71" t="str">
-        <v>f数组代表着索引i之前的字符串能否被拆分，因此只需考虑f[n]是否为True即可。</v>
+        <v>条件:从头走到尾 最小子序列:走过的步数最少，涉及到的元素的个数最少，也即最小子序列</v>
       </c>
       <c r="M90" s="71"/>
     </row>
-    <row r="91" ht="50" customHeight="1">
-      <c r="A91" s="28"/>
-      <c r="B91" s="103" t="str">
-        <v>递增子序列</v>
+    <row r="91" ht="64" customHeight="1">
+      <c r="A91" s="28" t="str">
+        <v>动态规划</v>
+      </c>
+      <c r="B91" s="102" t="str">
+        <v>计数递推</v>
       </c>
       <c r="C91" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D91" s="34" t="n">
-        <v>300</v>
+        <v>2266</v>
       </c>
       <c r="E91" s="72" t="str">
-        <v>300. 最长递增子序列</v>
+        <v>2266. 统计打字方案数</v>
       </c>
       <c r="F91" s="45" t="str">
         <v>中等</v>
@@ -3535,7 +3629,7 @@
       <c r="G91" s="51"/>
       <c r="H91" s="51"/>
       <c r="I91" s="56" t="str">
-        <v>leetcode.cn/problems/longest-increasing-subsequence/</v>
+        <v>leetcode.cn/problems/count-number-of-texts/</v>
       </c>
       <c r="J91" s="73"/>
       <c r="K91" s="74" t="n">
@@ -3543,29 +3637,31 @@
         <v>0</v>
       </c>
       <c r="L91" s="71" t="str">
-        <v>方法一：使用子集型回溯的枚举选哪个思路 方法二： 在LS相同的情况下我们只保存末尾元素最小的那个值，因为末尾元素越小，后续LS的长度才有可能越大</v>
+        <v>组合计数+DP：连续相同数字分组，每组按键方案满足dp[i]=dp[i-1]+dp[i-2]+dp[i-3]+(4字母键再加dp[i-4])；结果取模1e9+7</v>
       </c>
       <c r="M91" s="71"/>
     </row>
-    <row r="92" ht="50" customHeight="1">
+    <row r="92" ht="78" customHeight="1">
       <c r="A92" s="28"/>
-      <c r="B92" s="103"/>
+      <c r="B92" s="102" t="str">
+        <v>线性递推</v>
+      </c>
       <c r="C92" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D92" s="34" t="n">
-        <v>1187</v>
+        <v>198</v>
       </c>
       <c r="E92" s="72" t="str">
-        <v>1187. 使数组严格递增</v>
-      </c>
-      <c r="F92" s="91" t="str">
-        <v>困难</v>
+        <v>198. 打家劫舍</v>
+      </c>
+      <c r="F92" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G92" s="51"/>
       <c r="H92" s="51"/>
       <c r="I92" s="56" t="str">
-        <v>leetcode.cn/problems/make-array-strictly-increasing/</v>
+        <v>leetcode.cn/problems/house-robber/</v>
       </c>
       <c r="J92" s="73"/>
       <c r="K92" s="74" t="n">
@@ -3573,29 +3669,31 @@
         <v>0</v>
       </c>
       <c r="L92" s="71" t="str">
-        <v>f[i] 表示：以 a[i] 结尾（且 a[i] 不被替换）时，前 i+1 个元素中最多能保留多少个不替换的元素</v>
+        <v>使用动态规划的方法，而对于偷前i个房子的问题，它的最大值为偷取前i-1个房子与偷取前i-2个房子加上当前房子的价格的最大值，因此实际上只需使用两个变量记录i-1与i-2的值，不需要使用一个列表来完整记录每个索引的最大值</v>
       </c>
       <c r="M92" s="71"/>
     </row>
-    <row r="93" ht="50" customHeight="1">
+    <row r="93" ht="78" customHeight="1">
       <c r="A93" s="28"/>
-      <c r="B93" s="103"/>
+      <c r="B93" s="102" t="str">
+        <v>打家劫舍题组</v>
+      </c>
       <c r="C93" s="34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D93" s="34" t="n">
-        <v>1671</v>
+        <v>213</v>
       </c>
       <c r="E93" s="72" t="str">
-        <v>1671. 得到山形数组的最少删除次数</v>
-      </c>
-      <c r="F93" s="91" t="str">
-        <v>困难</v>
+        <v>213. 打家劫舍 II</v>
+      </c>
+      <c r="F93" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G93" s="51"/>
       <c r="H93" s="51"/>
       <c r="I93" s="56" t="str">
-        <v>leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/</v>
+        <v>leetcode.cn/problems/house-robber-ii/</v>
       </c>
       <c r="J93" s="73"/>
       <c r="K93" s="74" t="n">
@@ -3603,29 +3701,31 @@
         <v>0</v>
       </c>
       <c r="L93" s="71" t="str">
-        <v>山形数组：LIS+LDS，枚举峰顶，删除数=n-max(LIS[i]+LDS[i]-1)；峰两侧都需有元素</v>
+        <v>房屋首尾相邻，分别计算不选最后一间和不选第一间的线性打家劫舍结果，取两者最大值。</v>
       </c>
       <c r="M93" s="71"/>
     </row>
     <row r="94" ht="50" customHeight="1">
       <c r="A94" s="28"/>
-      <c r="B94" s="103"/>
+      <c r="B94" s="102" t="str">
+        <v>背包</v>
+      </c>
       <c r="C94" s="34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D94" s="34" t="n">
-        <v>1964</v>
+        <v>322</v>
       </c>
       <c r="E94" s="72" t="str">
-        <v>1964. 找出到每个位置为止的最长合法障碍赛跑路线</v>
-      </c>
-      <c r="F94" s="91" t="str">
-        <v>困难</v>
+        <v>322. 零钱兑换</v>
+      </c>
+      <c r="F94" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G94" s="51"/>
       <c r="H94" s="51"/>
       <c r="I94" s="56" t="str">
-        <v>leetcode.cn/problems/longest-obstacle-course-at-each-position/</v>
+        <v>leetcode.cn/problems/coin-change/</v>
       </c>
       <c r="J94" s="73"/>
       <c r="K94" s="74" t="n">
@@ -3633,23 +3733,23 @@
         <v>0</v>
       </c>
       <c r="L94" s="71" t="str">
-        <v>此题与LIS问题的不同之处在于求解的是以某个元素为止的非递减序列的长度，而不是整个数组的最长递增子序列的长度</v>
+        <v>完全背包：f[i]=min(f[i], f[i-coin]+1)；f初始化为inf、f[0]=0，返回时判断是否可达</v>
       </c>
       <c r="M94" s="71"/>
     </row>
-    <row r="95" ht="78" customHeight="1">
+    <row r="95" ht="60" customHeight="1">
       <c r="A95" s="28"/>
-      <c r="B95" s="103" t="str">
-        <v>连续子数组</v>
+      <c r="B95" s="102" t="str">
+        <v>0-1 背包</v>
       </c>
       <c r="C95" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D95" s="34" t="n">
-        <v>152</v>
+        <v>416</v>
       </c>
       <c r="E95" s="72" t="str">
-        <v>152. 乘积最大子数组</v>
+        <v>416.分割等和子集</v>
       </c>
       <c r="F95" s="45" t="str">
         <v>中等</v>
@@ -3657,7 +3757,7 @@
       <c r="G95" s="51"/>
       <c r="H95" s="51"/>
       <c r="I95" s="56" t="str">
-        <v>leetcode.cn/problems/maximum-product-subarray/</v>
+        <v>leetcode.cn/problems/partition-equal-subset-sum/</v>
       </c>
       <c r="J95" s="73"/>
       <c r="K95" s="74" t="n">
@@ -3665,31 +3765,31 @@
         <v>0</v>
       </c>
       <c r="L95" s="71" t="str">
-        <v>这个问题的思路与求解最大连续子数组和很像，不同的点在于不仅要记录当前最大值，还要记录当前最小值，因为如果当前的数是一个负数的话，那么它乘以小值反而得到一个更大的值，因此在遇到负数的情况下，首先需要将之前的大值与小值互换…</v>
+        <v>0,1背包问题,内部循环要倒序遍历,与零钱兑换以及完全平方和数不同</v>
       </c>
       <c r="M95" s="71"/>
     </row>
     <row r="96" ht="36" customHeight="1">
       <c r="A96" s="28"/>
-      <c r="B96" s="103" t="str">
-        <v>括号匹配</v>
+      <c r="B96" s="102" t="str">
+        <v>背包</v>
       </c>
       <c r="C96" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D96" s="34" t="n">
-        <v>32</v>
+        <v>494</v>
       </c>
       <c r="E96" s="72" t="str">
-        <v>32. 最长有效括号</v>
-      </c>
-      <c r="F96" s="91" t="str">
-        <v>困难</v>
+        <v>494. 目标和</v>
+      </c>
+      <c r="F96" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G96" s="51"/>
       <c r="H96" s="51"/>
       <c r="I96" s="56" t="str">
-        <v>leetcode.cn/problems/longest-valid-parentheses/</v>
+        <v>leetcode.cn/problems/target-sum/</v>
       </c>
       <c r="J96" s="73"/>
       <c r="K96" s="74" t="n">
@@ -3697,33 +3797,31 @@
         <v>0</v>
       </c>
       <c r="L96" s="71" t="str">
-        <v>栈存左括号下标，栈底保留最后一个未匹配的')'作哨兵；遇')'弹出并更新ans</v>
+        <v>01背包：target += sum(nums)，求恰好等于target的方案数（每个数选或不选）;</v>
       </c>
       <c r="M96" s="71"/>
     </row>
-    <row r="97" ht="78" customHeight="1">
-      <c r="A97" s="28" t="str">
-        <v>多维动态规划</v>
-      </c>
-      <c r="B97" s="103" t="str">
-        <v>多维状态与路径</v>
+    <row r="97" ht="36" customHeight="1">
+      <c r="A97" s="28"/>
+      <c r="B97" s="102" t="str">
+        <v>字符串划分</v>
       </c>
       <c r="C97" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D97" s="34" t="n">
-        <v>1770</v>
+        <v>139</v>
       </c>
       <c r="E97" s="72" t="str">
-        <v>1770. 执行乘法运算的最大分数</v>
-      </c>
-      <c r="F97" s="91" t="str">
-        <v>困难</v>
+        <v>139. 单词拆分</v>
+      </c>
+      <c r="F97" s="45" t="str">
+        <v>中等</v>
       </c>
       <c r="G97" s="51"/>
       <c r="H97" s="51"/>
       <c r="I97" s="56" t="str">
-        <v>leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/</v>
+        <v>leetcode.cn/problems/word-break/</v>
       </c>
       <c r="J97" s="73"/>
       <c r="K97" s="74" t="n">
@@ -3731,23 +3829,23 @@
         <v>0</v>
       </c>
       <c r="L97" s="71" t="str">
-        <v>这个题最难的点在于f数组的理解，f[i][j]计算的是剩余操作的最大分数，也就是从第i+1步操作到第m步的最大分数，而j代表着已经选取了j个左侧的值，同时也指明了当前左指针正指向j这个元素，选取的值不论左右，是不会计入到…</v>
+        <v>f数组代表着索引i之前的字符串能否被拆分，数组有效范围为[j,i),其中不包含i,因此在遍历j的时候应该从i-1开始倒序遍历.</v>
       </c>
       <c r="M97" s="71"/>
     </row>
-    <row r="98" ht="36" customHeight="1">
+    <row r="98" ht="50" customHeight="1">
       <c r="A98" s="28"/>
-      <c r="B98" s="103" t="str">
-        <v>回文与区间DP</v>
+      <c r="B98" s="102" t="str">
+        <v>递增子序列</v>
       </c>
       <c r="C98" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D98" s="34" t="n">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="E98" s="72" t="str">
-        <v>5. 最长回文子串</v>
+        <v>300. 最长递增子序列</v>
       </c>
       <c r="F98" s="45" t="str">
         <v>中等</v>
@@ -3755,7 +3853,7 @@
       <c r="G98" s="51"/>
       <c r="H98" s="51"/>
       <c r="I98" s="56" t="str">
-        <v>leetcode.cn/problems/longest-palindromic-substring/</v>
+        <v>leetcode.cn/problems/longest-increasing-subsequence/</v>
       </c>
       <c r="J98" s="73"/>
       <c r="K98" s="74" t="n">
@@ -3763,29 +3861,29 @@
         <v>0</v>
       </c>
       <c r="L98" s="71" t="str">
-        <v>使用这种方法通过一次循环就实现了对每个位置的奇回文串与偶回文串的检查</v>
+        <v>方法一：使用子集型回溯的枚举选哪个思路 方法二： 在LS相同的情况下我们只保存末尾元素最小的那个值，因为末尾元素越小，后续LS的长度才有可能越大</v>
       </c>
       <c r="M98" s="71"/>
     </row>
     <row r="99" ht="50" customHeight="1">
       <c r="A99" s="28"/>
-      <c r="B99" s="103"/>
+      <c r="B99" s="102"/>
       <c r="C99" s="34" t="n">
         <v>2</v>
       </c>
       <c r="D99" s="34" t="n">
-        <v>516</v>
+        <v>1187</v>
       </c>
       <c r="E99" s="72" t="str">
-        <v>516. 最长回文子序列</v>
-      </c>
-      <c r="F99" s="45" t="str">
-        <v>中等</v>
+        <v>1187. 使数组严格递增</v>
+      </c>
+      <c r="F99" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G99" s="51"/>
       <c r="H99" s="51"/>
       <c r="I99" s="56" t="str">
-        <v>leetcode.cn/problems/longest-palindromic-subsequence/</v>
+        <v>leetcode.cn/problems/make-array-strictly-increasing/</v>
       </c>
       <c r="J99" s="73"/>
       <c r="K99" s="74" t="n">
@@ -3793,29 +3891,29 @@
         <v>0</v>
       </c>
       <c r="L99" s="71" t="str">
-        <v>区间DP：f[i][j]表示s[i..j]的最长回文子序列；s[i]==s[j]则+2，否则取max(去左,去右)</v>
+        <v>f[i] 表示：以 a[i] 结尾（且 a[i] 不被替换）时，前 i+1 个元素中最多能保留多少个不替换的元素</v>
       </c>
       <c r="M99" s="71"/>
     </row>
-    <row r="100" ht="78" customHeight="1">
+    <row r="100" ht="50" customHeight="1">
       <c r="A100" s="28"/>
-      <c r="B100" s="103"/>
+      <c r="B100" s="102"/>
       <c r="C100" s="34" t="n">
         <v>3</v>
       </c>
       <c r="D100" s="34" t="n">
-        <v>647</v>
+        <v>1671</v>
       </c>
       <c r="E100" s="72" t="str">
-        <v>647. 回文子串</v>
-      </c>
-      <c r="F100" s="45" t="str">
-        <v>中等</v>
+        <v>1671. 得到山形数组的最少删除次数</v>
+      </c>
+      <c r="F100" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G100" s="51"/>
       <c r="H100" s="51"/>
       <c r="I100" s="56" t="str">
-        <v>leetcode.cn/problems/palindromic-substrings/</v>
+        <v>leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/</v>
       </c>
       <c r="J100" s="73"/>
       <c r="K100" s="74" t="n">
@@ -3823,29 +3921,29 @@
         <v>0</v>
       </c>
       <c r="L100" s="71" t="str">
-        <v>是用动态规划思路解答这个问题的关键在于想清楚dp数组的含义，[i,j]的含义不是从i到j的字符字串中含有多少回文子串，而是判断这个子串是不是一个回文串，因此dp数组有True与False构成，通过统计True的数量来判断…</v>
+        <v>山形数组：LIS+LDS，枚举峰顶，删除数=n-max(LIS[i]+LDS[i]-1)；峰两侧都需有元素</v>
       </c>
       <c r="M100" s="71"/>
     </row>
     <row r="101" ht="50" customHeight="1">
       <c r="A101" s="28"/>
-      <c r="B101" s="103"/>
+      <c r="B101" s="102"/>
       <c r="C101" s="34" t="n">
         <v>4</v>
       </c>
       <c r="D101" s="34" t="n">
-        <v>1039</v>
+        <v>1964</v>
       </c>
       <c r="E101" s="72" t="str">
-        <v>1039. 多边形三角剖分的最低得分</v>
-      </c>
-      <c r="F101" s="45" t="str">
-        <v>中等</v>
+        <v>1964. 找出到每个位置为止的最长合法障碍赛跑路线</v>
+      </c>
+      <c r="F101" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G101" s="51"/>
       <c r="H101" s="51"/>
       <c r="I101" s="56" t="str">
-        <v>leetcode.cn/problems/minimum-score-triangulation-of-polygon/</v>
+        <v>leetcode.cn/problems/longest-obstacle-course-at-each-position/</v>
       </c>
       <c r="J101" s="73"/>
       <c r="K101" s="74" t="n">
@@ -3853,23 +3951,23 @@
         <v>0</v>
       </c>
       <c r="L101" s="71" t="str">
-        <v>回溯三问： 1.当前操作：在(i，j)的范围内枚举一个数k 2.子问题：求解(i,j)的最低得分 3.下一个子问题：求解(i,k)与(k,j)的最低得分</v>
+        <v>此题与LIS问题的不同之处在于求解的是以某个元素为止的非递减序列的长度，而不是整个数组的最长递增子序列的长度</v>
       </c>
       <c r="M101" s="71"/>
     </row>
-    <row r="102" ht="50" customHeight="1">
+    <row r="102" ht="78" customHeight="1">
       <c r="A102" s="28"/>
-      <c r="B102" s="103" t="str">
-        <v>双序列</v>
+      <c r="B102" s="102" t="str">
+        <v>连续子数组</v>
       </c>
       <c r="C102" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D102" s="34" t="n">
-        <v>1143</v>
+        <v>152</v>
       </c>
       <c r="E102" s="72" t="str">
-        <v>1143. 最长公共子序列</v>
+        <v>152. 乘积最大子数组</v>
       </c>
       <c r="F102" s="45" t="str">
         <v>中等</v>
@@ -3877,7 +3975,7 @@
       <c r="G102" s="51"/>
       <c r="H102" s="51"/>
       <c r="I102" s="56" t="str">
-        <v>leetcode.cn/problems/longest-common-subsequence/</v>
+        <v>leetcode.cn/problems/maximum-product-subarray/</v>
       </c>
       <c r="J102" s="73"/>
       <c r="K102" s="74" t="n">
@@ -3885,29 +3983,31 @@
         <v>0</v>
       </c>
       <c r="L102" s="71" t="str">
-        <v>二维DP：text1[i]==text2[j]则f[i][j]=f[i-1][j-1]+1，否则取max(f[i-1][j], f[i][j-1])</v>
+        <v>需要同时记录curr_min与curr_max,当遇到一个负值的时候,需要将curr_min与curr_max调换,与最大连续子数组和思路相同;同时循环的起始值决定了curr_max,curr_min以及max_num的初始值.</v>
       </c>
       <c r="M102" s="71"/>
     </row>
     <row r="103" ht="36" customHeight="1">
       <c r="A103" s="28"/>
-      <c r="B103" s="103"/>
+      <c r="B103" s="102" t="str">
+        <v>括号匹配</v>
+      </c>
       <c r="C103" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D103" s="34" t="n">
-        <v>712</v>
+        <v>32</v>
       </c>
       <c r="E103" s="72" t="str">
-        <v>712. 两个字符串的最小ASCII删除和</v>
-      </c>
-      <c r="F103" s="45" t="str">
-        <v>中等</v>
+        <v>32. 最长有效括号</v>
+      </c>
+      <c r="F103" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G103" s="51"/>
       <c r="H103" s="51"/>
       <c r="I103" s="56" t="str">
-        <v>leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/</v>
+        <v>leetcode.cn/problems/longest-valid-parentheses/</v>
       </c>
       <c r="J103" s="73"/>
       <c r="K103" s="74" t="n">
@@ -3915,29 +4015,33 @@
         <v>0</v>
       </c>
       <c r="L103" s="71" t="str">
-        <v>LCS变式：总ASCII和-2×LCS；或直接DP，两字符不同时取删s1[i]或删s2[j]的较小值</v>
+        <v>栈存左括号下标，栈底保留最后一个未匹配的')'作哨兵；遇')'弹出并更新ans</v>
       </c>
       <c r="M103" s="71"/>
     </row>
-    <row r="104" ht="36" customHeight="1">
-      <c r="A104" s="28"/>
-      <c r="B104" s="103"/>
+    <row r="104" ht="78" customHeight="1">
+      <c r="A104" s="28" t="str">
+        <v>多维动态规划</v>
+      </c>
+      <c r="B104" s="102" t="str">
+        <v>多维状态与路径</v>
+      </c>
       <c r="C104" s="34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D104" s="34" t="n">
-        <v>72</v>
+        <v>1770</v>
       </c>
       <c r="E104" s="72" t="str">
-        <v>72. 编辑距离</v>
-      </c>
-      <c r="F104" s="45" t="str">
-        <v>中等</v>
+        <v>1770. 执行乘法运算的最大分数</v>
+      </c>
+      <c r="F104" s="91" t="str">
+        <v>困难</v>
       </c>
       <c r="G104" s="51"/>
       <c r="H104" s="51"/>
       <c r="I104" s="56" t="str">
-        <v>leetcode.cn/problems/edit-distance/</v>
+        <v>leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/</v>
       </c>
       <c r="J104" s="73"/>
       <c r="K104" s="74" t="n">
@@ -3945,33 +4049,31 @@
         <v>0</v>
       </c>
       <c r="L104" s="71" t="str">
-        <v>DP：f[i][j]编辑距离；末尾字符相同直接继承，不同则取增/删/改三者最小值+1</v>
+        <v>这个题最难的点在于f数组的理解，f[i][j]计算的是剩余操作的最大分数，也就是从第i+1步操作到第m步的最大分数，而j代表着已经选取了j个左侧的值，同时也指明了当前左指针正指向j这个元素，选取的值不论左右，是不会计入到…</v>
       </c>
       <c r="M104" s="71"/>
     </row>
-    <row r="105" ht="36" customHeight="1">
-      <c r="A105" s="28" t="str">
-        <v>技巧</v>
-      </c>
-      <c r="B105" s="103" t="str">
-        <v>三路划分</v>
+    <row r="105" ht="78" customHeight="1">
+      <c r="A105" s="28"/>
+      <c r="B105" s="102" t="str">
+        <v>网格路径</v>
       </c>
       <c r="C105" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D105" s="34" t="n">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="E105" s="72" t="str">
-        <v>75. 颜色分类</v>
-      </c>
-      <c r="F105" s="45" t="str">
+        <v>62. 不同路径</v>
+      </c>
+      <c r="F105" s="91" t="str">
         <v>中等</v>
       </c>
       <c r="G105" s="51"/>
       <c r="H105" s="51"/>
       <c r="I105" s="56" t="str">
-        <v>leetcode.cn/problems/sort-colors/</v>
+        <v>leetcode.cn/problems/unique-paths/</v>
       </c>
       <c r="J105" s="73"/>
       <c r="K105" s="74" t="n">
@@ -3979,31 +4081,29 @@
         <v>0</v>
       </c>
       <c r="L105" s="71" t="str">
-        <v>荷兰国旗三指针：[0,zero]全0、[two,n-1]全2、中间为1；partition交换</v>
+        <v>网格动态规划：到达 (i,j) 的路径数等于从上方和左方到达的路径数之和；首行和首列初始化为 1。</v>
       </c>
       <c r="M105" s="71"/>
     </row>
-    <row r="106" ht="64" customHeight="1">
+    <row r="106" ht="78" customHeight="1">
       <c r="A106" s="28"/>
-      <c r="B106" s="103" t="str">
-        <v>排列变换</v>
-      </c>
+      <c r="B106" s="102"/>
       <c r="C106" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D106" s="34" t="n">
-        <v>31</v>
+        <v>64</v>
       </c>
       <c r="E106" s="72" t="str">
-        <v>31. 下一个排列</v>
-      </c>
-      <c r="F106" s="45" t="str">
+        <v>64.最小路径和</v>
+      </c>
+      <c r="F106" s="91" t="str">
         <v>中等</v>
       </c>
       <c r="G106" s="51"/>
       <c r="H106" s="51"/>
       <c r="I106" s="56" t="str">
-        <v>leetcode.cn/problems/next-permutation/</v>
+        <v>leetcode.cn/problems/minimum-path-sum/</v>
       </c>
       <c r="J106" s="73"/>
       <c r="K106" s="74" t="n">
@@ -4011,23 +4111,23 @@
         <v>0</v>
       </c>
       <c r="L106" s="71" t="str">
-        <v>思路： 1.从右向左，找第一个小于右侧相邻数字的数 x 2.找 x 右边最小的大于 x 的数 y，交换 x 和 y 3.反转 y 右边的数，把右边的数变成最小的排列</v>
+        <v>注意f[0]的处理:f[0] += grid[i][0],同时内部循环从1开始.使用一维数组便可以解决问题</v>
       </c>
       <c r="M106" s="71"/>
     </row>
-    <row r="107" ht="78" customHeight="1">
+    <row r="107" ht="45.79999923706055" customHeight="1">
       <c r="A107" s="28"/>
-      <c r="B107" s="103" t="str">
-        <v>判圈</v>
+      <c r="B107" s="102" t="str">
+        <v>回文与区间DP</v>
       </c>
       <c r="C107" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D107" s="34" t="n">
-        <v>287</v>
+        <v>5</v>
       </c>
       <c r="E107" s="72" t="str">
-        <v>287. 寻找重复数</v>
+        <v>5. 最长回文子串</v>
       </c>
       <c r="F107" s="45" t="str">
         <v>中等</v>
@@ -4035,7 +4135,7 @@
       <c r="G107" s="51"/>
       <c r="H107" s="51"/>
       <c r="I107" s="56" t="str">
-        <v>leetcode.cn/problems/find-the-duplicate-number/</v>
+        <v>leetcode.cn/problems/longest-palindromic-substring/</v>
       </c>
       <c r="J107" s="73"/>
       <c r="K107" s="74" t="n">
@@ -4043,9 +4143,323 @@
         <v>0</v>
       </c>
       <c r="L107" s="71" t="str">
+        <v>以每个字符作为中心进行排查,寻找最长字串;注意循环里面使用的l与r都是开指针,但是ans_left是闭指针,因此赋值的时候应该是ans_left = left + 1</v>
+      </c>
+      <c r="M107" s="71"/>
+    </row>
+    <row r="108" ht="50" customHeight="1">
+      <c r="A108" s="28"/>
+      <c r="B108" s="102"/>
+      <c r="C108" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D108" s="34" t="n">
+        <v>516</v>
+      </c>
+      <c r="E108" s="72" t="str">
+        <v>516. 最长回文子序列</v>
+      </c>
+      <c r="F108" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G108" s="51"/>
+      <c r="H108" s="51"/>
+      <c r="I108" s="56" t="str">
+        <v>leetcode.cn/problems/longest-palindromic-subsequence/</v>
+      </c>
+      <c r="J108" s="73"/>
+      <c r="K108" s="74" t="n">
+        <f>LEN(J108)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J108,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L108" s="71" t="str">
+        <v>区间DP：f[i][j]表示s[i..j]的最长回文子序列；s[i]==s[j]则+2，否则取max(去左,去右)</v>
+      </c>
+      <c r="M108" s="71"/>
+    </row>
+    <row r="109" ht="78" customHeight="1">
+      <c r="A109" s="28"/>
+      <c r="B109" s="102"/>
+      <c r="C109" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D109" s="34" t="n">
+        <v>647</v>
+      </c>
+      <c r="E109" s="72" t="str">
+        <v>647. 回文子串</v>
+      </c>
+      <c r="F109" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G109" s="51"/>
+      <c r="H109" s="51"/>
+      <c r="I109" s="56" t="str">
+        <v>leetcode.cn/problems/palindromic-substrings/</v>
+      </c>
+      <c r="J109" s="73"/>
+      <c r="K109" s="74" t="n">
+        <f>LEN(J109)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J109,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L109" s="71" t="str">
+        <v>是用动态规划思路解答这个问题的关键在于想清楚dp数组的含义，[i,j]的含义不是从i到j的字符字串中含有多少回文子串，而是判断这个子串是不是一个回文串，因此dp数组有True与False构成，通过统计True的数量来判断…</v>
+      </c>
+      <c r="M109" s="71"/>
+    </row>
+    <row r="110" ht="50" customHeight="1">
+      <c r="A110" s="28"/>
+      <c r="B110" s="102"/>
+      <c r="C110" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="D110" s="34" t="n">
+        <v>1039</v>
+      </c>
+      <c r="E110" s="72" t="str">
+        <v>1039. 多边形三角剖分的最低得分</v>
+      </c>
+      <c r="F110" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G110" s="51"/>
+      <c r="H110" s="51"/>
+      <c r="I110" s="56" t="str">
+        <v>leetcode.cn/problems/minimum-score-triangulation-of-polygon/</v>
+      </c>
+      <c r="J110" s="73"/>
+      <c r="K110" s="74" t="n">
+        <f>LEN(J110)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J110,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L110" s="71" t="str">
+        <v>回溯三问： 1.当前操作：在(i，j)的范围内枚举一个数k 2.子问题：求解(i,j)的最低得分 3.下一个子问题：求解(i,k)与(k,j)的最低得分</v>
+      </c>
+      <c r="M110" s="71"/>
+    </row>
+    <row r="111" ht="50" customHeight="1">
+      <c r="A111" s="28"/>
+      <c r="B111" s="102" t="str">
+        <v>双序列</v>
+      </c>
+      <c r="C111" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" s="34" t="n">
+        <v>1143</v>
+      </c>
+      <c r="E111" s="72" t="str">
+        <v>1143. 最长公共子序列</v>
+      </c>
+      <c r="F111" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G111" s="51"/>
+      <c r="H111" s="51"/>
+      <c r="I111" s="56" t="str">
+        <v>leetcode.cn/problems/longest-common-subsequence/</v>
+      </c>
+      <c r="J111" s="73"/>
+      <c r="K111" s="74" t="n">
+        <f>LEN(J111)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J111,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L111" s="71" t="str">
+        <v>二维DP：text1[i]==text2[j]则f[i][j]=f[i-1][j-1]+1，否则取max(f[i-1][j], f[i][j-1])</v>
+      </c>
+      <c r="M111" s="71"/>
+    </row>
+    <row r="112" ht="36" customHeight="1">
+      <c r="A112" s="28"/>
+      <c r="B112" s="102"/>
+      <c r="C112" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D112" s="34" t="n">
+        <v>712</v>
+      </c>
+      <c r="E112" s="72" t="str">
+        <v>712. 两个字符串的最小ASCII删除和</v>
+      </c>
+      <c r="F112" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G112" s="51"/>
+      <c r="H112" s="51"/>
+      <c r="I112" s="56" t="str">
+        <v>leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/</v>
+      </c>
+      <c r="J112" s="73"/>
+      <c r="K112" s="74" t="n">
+        <f>LEN(J112)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J112,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L112" s="71" t="str">
+        <v>LCS变式：总ASCII和-2×LCS；或直接DP，两字符不同时取删s1[i]或删s2[j]的较小值</v>
+      </c>
+      <c r="M112" s="71"/>
+    </row>
+    <row r="113" ht="36" customHeight="1">
+      <c r="A113" s="28"/>
+      <c r="B113" s="102"/>
+      <c r="C113" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D113" s="34" t="n">
+        <v>72</v>
+      </c>
+      <c r="E113" s="72" t="str">
+        <v>72. 编辑距离</v>
+      </c>
+      <c r="F113" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G113" s="51"/>
+      <c r="H113" s="51"/>
+      <c r="I113" s="56" t="str">
+        <v>leetcode.cn/problems/edit-distance/</v>
+      </c>
+      <c r="J113" s="73"/>
+      <c r="K113" s="74" t="n">
+        <f>LEN(J113)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J113,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L113" s="71" t="str">
+        <v>DP：f[i][j]编辑距离；末尾字符相同直接继承，不同则取增/删/改三者最小值+1</v>
+      </c>
+      <c r="M113" s="71" t="str">
+        <v>注意f数组的初始化不是全0.</v>
+      </c>
+    </row>
+    <row r="114" ht="45.79999923706055" customHeight="1">
+      <c r="A114" s="28" t="str">
+        <v>技巧</v>
+      </c>
+      <c r="B114" s="102" t="str">
+        <v>三路划分</v>
+      </c>
+      <c r="C114" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="34" t="n">
+        <v>75</v>
+      </c>
+      <c r="E114" s="72" t="str">
+        <v>75. 颜色分类</v>
+      </c>
+      <c r="F114" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G114" s="51"/>
+      <c r="H114" s="51"/>
+      <c r="I114" s="56" t="str">
+        <v>leetcode.cn/problems/sort-colors/</v>
+      </c>
+      <c r="J114" s="73"/>
+      <c r="K114" s="74" t="n">
+        <f>LEN(J114)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J114,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L114" s="71" t="str">
+        <v>荷兰国旗三指针:三个指针分别为lt,i,rt,其中[0,lt]元素全为0,[lt+1,i)元素全为1;(i,rt)为探索区域;[rt,right]内部元素全为2.其中[]代表包含对应元素,()代表不包含</v>
+      </c>
+      <c r="M114" s="71"/>
+    </row>
+    <row r="115" ht="60" customHeight="1">
+      <c r="A115" s="28"/>
+      <c r="B115" s="102" t="str">
+        <v>位运算</v>
+      </c>
+      <c r="C115" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" s="34" t="n">
+        <v>136</v>
+      </c>
+      <c r="E115" s="72" t="str">
+        <v>136. 只出现一次的数字</v>
+      </c>
+      <c r="F115" s="80" t="str">
+        <v>简单</v>
+      </c>
+      <c r="G115" s="51"/>
+      <c r="H115" s="51"/>
+      <c r="I115" s="56" t="str">
+        <v>leetcode.cn/problems/single-number/</v>
+      </c>
+      <c r="J115" s="73"/>
+      <c r="K115" s="74" t="n">
+        <f>LEN(J115)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J115,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L115" s="71" t="str">
+        <v>异或思路:python当中的异或操作按位计算</v>
+      </c>
+      <c r="M115" s="71"/>
+    </row>
+    <row r="116" ht="64" customHeight="1">
+      <c r="A116" s="28"/>
+      <c r="B116" s="102" t="str">
+        <v>排列变换</v>
+      </c>
+      <c r="C116" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" s="34" t="n">
+        <v>31</v>
+      </c>
+      <c r="E116" s="72" t="str">
+        <v>31. 下一个排列</v>
+      </c>
+      <c r="F116" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G116" s="51"/>
+      <c r="H116" s="51"/>
+      <c r="I116" s="56" t="str">
+        <v>leetcode.cn/problems/next-permutation/</v>
+      </c>
+      <c r="J116" s="73"/>
+      <c r="K116" s="74" t="n">
+        <f>LEN(J116)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J116,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L116" s="71" t="str">
+        <v>思路： 1.从右向左，找第一个小于右侧相邻数字的数 x 2.找 x 右边最小的大于 x 的数 y，交换 x 和 y 3.反转 y 右边的数，把右边的数变成最小的排列</v>
+      </c>
+      <c r="M116" s="71"/>
+    </row>
+    <row r="117" ht="78" customHeight="1">
+      <c r="A117" s="28"/>
+      <c r="B117" s="102" t="str">
+        <v>判圈</v>
+      </c>
+      <c r="C117" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D117" s="34" t="n">
+        <v>287</v>
+      </c>
+      <c r="E117" s="72" t="str">
+        <v>287. 寻找重复数</v>
+      </c>
+      <c r="F117" s="45" t="str">
+        <v>中等</v>
+      </c>
+      <c r="G117" s="51"/>
+      <c r="H117" s="51"/>
+      <c r="I117" s="56" t="str">
+        <v>leetcode.cn/problems/find-the-duplicate-number/</v>
+      </c>
+      <c r="J117" s="73"/>
+      <c r="K117" s="74" t="n">
+        <f>LEN(J117)-LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J117,"√",""),"×",""),"✓",""))</f>
+        <v>0</v>
+      </c>
+      <c r="L117" s="71" t="str">
         <v>这题的关键在于给出一个包含n+1个数字的数组，且数组的取值位于[1,n],可以这么看待问题，把这n+1个数对应的索引看成是n+1个节点，标号从0到n，构建从i到nums[i]的映射，nums[i]的值就代表了i这个节点指…</v>
       </c>
-      <c r="M107" s="71"/>
+      <c r="M117" s="71"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -4058,16 +4472,16 @@
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="A22:A25"/>
     <mergeCell ref="A26:A38"/>
-    <mergeCell ref="A39:A56"/>
-    <mergeCell ref="A57:A60"/>
-    <mergeCell ref="A61:A68"/>
-    <mergeCell ref="A69:A74"/>
-    <mergeCell ref="A75:A78"/>
-    <mergeCell ref="A79:A80"/>
-    <mergeCell ref="A81:A85"/>
-    <mergeCell ref="A86:A96"/>
-    <mergeCell ref="A97:A104"/>
-    <mergeCell ref="A105:A107"/>
+    <mergeCell ref="A39:A58"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="A63:A71"/>
+    <mergeCell ref="A72:A77"/>
+    <mergeCell ref="A78:A82"/>
+    <mergeCell ref="A83:A85"/>
+    <mergeCell ref="A86:A90"/>
+    <mergeCell ref="A91:A103"/>
+    <mergeCell ref="A104:A113"/>
+    <mergeCell ref="A114:A117"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="B26:B28"/>
@@ -4076,20 +4490,21 @@
     <mergeCell ref="B39:B40"/>
     <mergeCell ref="B41:B43"/>
     <mergeCell ref="B44:B47"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="B71:B73"/>
-    <mergeCell ref="B77:B78"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="B88:B89"/>
-    <mergeCell ref="B91:B94"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="B56:B58"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="B74:B76"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="B86:B88"/>
+    <mergeCell ref="B89:B90"/>
     <mergeCell ref="B98:B101"/>
-    <mergeCell ref="B102:B104"/>
+    <mergeCell ref="B105:B106"/>
+    <mergeCell ref="B107:B110"/>
+    <mergeCell ref="B111:B113"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="custom" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="只填写做题结果" error="请只填写√或×（兼容✓）。每个符号代表做了一次，例如√×√。" promptTitle="追加本次结果" prompt="双击或F2编辑，在末尾追加√或×。例如√×√表示3次；不要覆盖已有记录。" sqref="J4:J107">
+    <dataValidation type="custom" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="只填写做题结果" error="请只填写√或×（兼容✓）。每个符号代表做了一次，例如√×√。" promptTitle="追加本次结果" prompt="双击或F2编辑，在末尾追加√或×。例如√×√表示3次；不要覆盖已有记录。" sqref="J4:J117">
       <formula1>LEN(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(J4,"√",""),"×",""),"✓",""))=0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4130,7 +4545,7 @@
     <hyperlink ref="I20" display="leetcode.cn/problems/product-of-array-except-self/" r:id="codexHyperlink34"/>
     <hyperlink ref="E21" display="41. 缺失的第一个正数" tooltip="05_普通数组.ipynb / lc-41" r:id="codexHyperlink35"/>
     <hyperlink ref="I21" display="leetcode.cn/problems/first-missing-positive/" r:id="codexHyperlink36"/>
-    <hyperlink ref="E22" display="73. 矩阵置零" tooltip="06_矩阵.ipynb / lc-73" r:id="codexHyperlink37"/>
+    <hyperlink ref="E22" display="73.矩阵置零" tooltip="06_矩阵.ipynb / lc-73" r:id="codexHyperlink37"/>
     <hyperlink ref="I22" display="leetcode.cn/problems/set-matrix-zeroes/" r:id="codexHyperlink38"/>
     <hyperlink ref="E23" display="54. 螺旋矩阵" tooltip="06_矩阵.ipynb / lc-54" r:id="codexHyperlink39"/>
     <hyperlink ref="I23" display="leetcode.cn/problems/spiral-matrix/" r:id="codexHyperlink40"/>
@@ -4184,124 +4599,144 @@
     <hyperlink ref="I47" display="leetcode.cn/problems/difference-between-maximum-and-minimum-price-sum/" r:id="codexHyperlink88"/>
     <hyperlink ref="E48" display="98. 验证二叉搜索树" tooltip="08_二叉树.ipynb / lc-98" r:id="codexHyperlink89"/>
     <hyperlink ref="I48" display="leetcode.cn/problems/validate-binary-search-tree/" r:id="codexHyperlink90"/>
-    <hyperlink ref="E49" display="114. 二叉树展开为链表" tooltip="08_二叉树.ipynb / lc-114" r:id="codexHyperlink91"/>
-    <hyperlink ref="I49" display="leetcode.cn/problems/flatten-binary-tree-to-linked-list/" r:id="codexHyperlink92"/>
-    <hyperlink ref="E50" display="105. 从前序与中序遍历序列构造二叉树" tooltip="08_二叉树.ipynb / lc-105" r:id="codexHyperlink93"/>
-    <hyperlink ref="I50" display="leetcode.cn/problems/construct-binary-tree-from-preorder-and-inorder-traversal/" r:id="codexHyperlink94"/>
-    <hyperlink ref="E51" display="437. 路径总和 III" tooltip="08_二叉树.ipynb / lc-437" r:id="codexHyperlink95"/>
-    <hyperlink ref="I51" display="leetcode.cn/problems/path-sum-iii/" r:id="codexHyperlink96"/>
-    <hyperlink ref="E52" display="236. 二叉树的最近公共祖先" tooltip="08_二叉树.ipynb / lc-236" r:id="codexHyperlink97"/>
-    <hyperlink ref="I52" display="leetcode.cn/problems/lowest-common-ancestor-of-a-binary-tree/" r:id="codexHyperlink98"/>
-    <hyperlink ref="E53" display="235. 二叉搜索树的最近公共祖先" tooltip="08_二叉树.ipynb / lc-235" r:id="codexHyperlink99"/>
-    <hyperlink ref="I53" display="https://leetcode.cn/problems/lowest-common-ancestor-of-a-binary-search-tree/" r:id="codexHyperlink100"/>
-    <hyperlink ref="E54" display="124. 二叉树中的最大路径和" tooltip="08_二叉树.ipynb / lc-124" r:id="codexHyperlink101"/>
-    <hyperlink ref="I54" display="leetcode.cn/problems/binary-tree-maximum-path-sum/" r:id="codexHyperlink102"/>
-    <hyperlink ref="E55" display="337. 打家劫舍 III" tooltip="08_二叉树.ipynb / lc-337" r:id="codexHyperlink103"/>
-    <hyperlink ref="I55" display="leetcode.cn/problems/house-robber-iii/" r:id="codexHyperlink104"/>
-    <hyperlink ref="E56" display="968. 监控二叉树" tooltip="08_二叉树.ipynb / lc-968" r:id="codexHyperlink105"/>
-    <hyperlink ref="I56" display="leetcode.cn/problems/binary-tree-cameras/" r:id="codexHyperlink106"/>
-    <hyperlink ref="E57" display="200. 岛屿数量" tooltip="09_图论.ipynb / lc-200" r:id="codexHyperlink107"/>
-    <hyperlink ref="I57" display="leetcode.cn/problems/number-of-islands/" r:id="codexHyperlink108"/>
-    <hyperlink ref="E58" display="994. 腐烂的橘子" tooltip="09_图论.ipynb / lc-994" r:id="codexHyperlink109"/>
-    <hyperlink ref="I58" display="leetcode.cn/problems/rotting-oranges/" r:id="codexHyperlink110"/>
-    <hyperlink ref="E59" display="207. 课程表" tooltip="09_图论.ipynb / lc-207" r:id="codexHyperlink111"/>
-    <hyperlink ref="I59" display="leetcode.cn/problems/course-schedule/" r:id="codexHyperlink112"/>
-    <hyperlink ref="E60" display="208. 实现 Trie (前缀树)" tooltip="09_图论.ipynb / lc-208" r:id="codexHyperlink113"/>
-    <hyperlink ref="I60" display="leetcode.cn/problems/implement-trie-prefix-tree/" r:id="codexHyperlink114"/>
-    <hyperlink ref="E61" display="46. 全排列" tooltip="10_回溯.ipynb / lc-46" r:id="codexHyperlink115"/>
-    <hyperlink ref="I61" display="leetcode.cn/problems/permutations/" r:id="codexHyperlink116"/>
-    <hyperlink ref="E62" display="78. 子集" tooltip="10_回溯.ipynb / lc-78" r:id="codexHyperlink117"/>
-    <hyperlink ref="I62" display="leetcode.cn/problems/subsets/" r:id="codexHyperlink118"/>
-    <hyperlink ref="E63" display="17. 电话号码的字母组合" tooltip="10_回溯.ipynb / lc-17" r:id="codexHyperlink119"/>
-    <hyperlink ref="I63" display="leetcode.cn/problems/letter-combinations-of-a-phone-number/" r:id="codexHyperlink120"/>
-    <hyperlink ref="E64" display="39. 组合总和" tooltip="10_回溯.ipynb / lc-39" r:id="codexHyperlink121"/>
-    <hyperlink ref="I64" display="leetcode.cn/problems/combination-sum/" r:id="codexHyperlink122"/>
-    <hyperlink ref="E65" display="216. 组合总和 III" tooltip="10_回溯.ipynb / lc-216" r:id="codexHyperlink123"/>
-    <hyperlink ref="I65" display="leetcode.cn/problems/combination-sum-iii/" r:id="codexHyperlink124"/>
-    <hyperlink ref="E66" display="22. 括号生成" tooltip="10_回溯.ipynb / lc-22" r:id="codexHyperlink125"/>
-    <hyperlink ref="I66" display="leetcode.cn/problems/generate-parentheses/" r:id="codexHyperlink126"/>
-    <hyperlink ref="E67" display="131. 分割回文串" tooltip="10_回溯.ipynb / lc-131" r:id="codexHyperlink127"/>
-    <hyperlink ref="I67" display="leetcode.cn/problems/palindrome-partitioning/" r:id="codexHyperlink128"/>
-    <hyperlink ref="E68" display="51. N 皇后" tooltip="10_回溯.ipynb / lc-51" r:id="codexHyperlink129"/>
-    <hyperlink ref="I68" display="leetcode.cn/problems/n-queens/" r:id="codexHyperlink130"/>
-    <hyperlink ref="E69" display="74. 搜索二维矩阵" tooltip="11_二分查找.ipynb / lc-74" r:id="codexHyperlink131"/>
-    <hyperlink ref="I69" display="leetcode.cn/problems/search-a-2d-matrix/" r:id="codexHyperlink132"/>
-    <hyperlink ref="E70" display="34. 在排序数组中查找元素的第一个和最后一个位置" tooltip="11_二分查找.ipynb / lc-34" r:id="codexHyperlink133"/>
-    <hyperlink ref="I70" display="leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/" r:id="codexHyperlink134"/>
-    <hyperlink ref="E71" display="33. 搜索旋转排序数组" tooltip="11_二分查找.ipynb / lc-33" r:id="codexHyperlink135"/>
-    <hyperlink ref="I71" display="leetcode.cn/problems/search-in-rotated-sorted-array/" r:id="codexHyperlink136"/>
-    <hyperlink ref="E72" display="153. 寻找旋转排序数组中的最小值" tooltip="11_二分查找.ipynb / lc-153" r:id="codexHyperlink137"/>
-    <hyperlink ref="I72" display="leetcode.cn/problems/find-minimum-in-rotated-sorted-array/" r:id="codexHyperlink138"/>
-    <hyperlink ref="E73" display="162. 寻找峰值" tooltip="11_二分查找.ipynb / lc-162" r:id="codexHyperlink139"/>
-    <hyperlink ref="I73" display="leetcode.cn/problems/find-peak-element/" r:id="codexHyperlink140"/>
-    <hyperlink ref="E74" display="4. 寻找两个正序数组的中位数" tooltip="11_二分查找.ipynb / lc-4" r:id="codexHyperlink141"/>
-    <hyperlink ref="I74" display="leetcode.cn/problems/median-of-two-sorted-arrays/" r:id="codexHyperlink142"/>
-    <hyperlink ref="E75" display="155. 最小栈" tooltip="12_栈.ipynb / lc-155" r:id="codexHyperlink143"/>
-    <hyperlink ref="I75" display="leetcode.cn/problems/min-stack/" r:id="codexHyperlink144"/>
-    <hyperlink ref="E76" display="394. 字符串解码" tooltip="12_栈.ipynb / lc-394" r:id="codexHyperlink145"/>
-    <hyperlink ref="I76" display="leetcode.cn/problems/decode-string/" r:id="codexHyperlink146"/>
-    <hyperlink ref="E77" display="739. 每日温度" tooltip="12_栈.ipynb / lc-739" r:id="codexHyperlink147"/>
-    <hyperlink ref="I77" display="leetcode.cn/problems/daily-temperatures/" r:id="codexHyperlink148"/>
-    <hyperlink ref="E78" display="84. 柱状图中最大的矩形" tooltip="12_栈.ipynb / lc-84" r:id="codexHyperlink149"/>
-    <hyperlink ref="I78" display="leetcode.cn/problems/largest-rectangle-in-histogram/" r:id="codexHyperlink150"/>
-    <hyperlink ref="E79" display="215. 数组中的第 K 个最大元素" tooltip="13_堆.ipynb / lc-215" r:id="codexHyperlink151"/>
-    <hyperlink ref="I79" display="leetcode.cn/problems/kth-largest-element-in-an-array/" r:id="codexHyperlink152"/>
-    <hyperlink ref="E80" display="295. 数据流的中位数" tooltip="13_堆.ipynb / lc-295" r:id="codexHyperlink153"/>
-    <hyperlink ref="I80" display="leetcode.cn/problems/find-median-from-data-stream/" r:id="codexHyperlink154"/>
-    <hyperlink ref="E81" display="122. 买卖股票的最佳时机 II" tooltip="14_贪心算法.ipynb / lc-122" r:id="codexHyperlink155"/>
-    <hyperlink ref="I81" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/" r:id="codexHyperlink156"/>
-    <hyperlink ref="E82" display="188. 买卖股票的最佳时机 IV" tooltip="14_贪心算法.ipynb / lc-188" r:id="codexHyperlink157"/>
-    <hyperlink ref="I82" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/" r:id="codexHyperlink158"/>
-    <hyperlink ref="E83" display="309. 买卖股票的最佳时机含冷冻期" tooltip="14_贪心算法.ipynb / lc-309" r:id="codexHyperlink159"/>
-    <hyperlink ref="I83" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/" r:id="codexHyperlink160"/>
-    <hyperlink ref="E84" display="55. 跳跃游戏" tooltip="14_贪心算法.ipynb / lc-55" r:id="codexHyperlink161"/>
-    <hyperlink ref="I84" display="leetcode.cn/problems/jump-game/" r:id="codexHyperlink162"/>
-    <hyperlink ref="E85" display="45. 跳跃游戏 II" tooltip="14_贪心算法.ipynb / lc-45" r:id="codexHyperlink163"/>
-    <hyperlink ref="I85" display="leetcode.cn/problems/jump-game-ii/" r:id="codexHyperlink164"/>
-    <hyperlink ref="E86" display="2266. 统计打字方案数" tooltip="15_动态规划.ipynb / lc-2266" r:id="codexHyperlink165"/>
-    <hyperlink ref="I86" display="leetcode.cn/problems/count-number-of-texts/" r:id="codexHyperlink166"/>
-    <hyperlink ref="E87" display="198. 打家劫舍" tooltip="15_动态规划.ipynb / lc-198" r:id="codexHyperlink167"/>
-    <hyperlink ref="I87" display="leetcode.cn/problems/house-robber/" r:id="codexHyperlink168"/>
-    <hyperlink ref="E88" display="322. 零钱兑换" tooltip="15_动态规划.ipynb / lc-322" r:id="codexHyperlink169"/>
-    <hyperlink ref="I88" display="leetcode.cn/problems/coin-change/" r:id="codexHyperlink170"/>
-    <hyperlink ref="E89" display="494. 目标和" tooltip="15_动态规划.ipynb / lc-494" r:id="codexHyperlink171"/>
-    <hyperlink ref="I89" display="leetcode.cn/problems/target-sum/" r:id="codexHyperlink172"/>
-    <hyperlink ref="E90" display="139. 单词拆分" tooltip="15_动态规划.ipynb / lc-139" r:id="codexHyperlink173"/>
-    <hyperlink ref="I90" display="leetcode.cn/problems/word-break/" r:id="codexHyperlink174"/>
-    <hyperlink ref="E91" display="300. 最长递增子序列" tooltip="15_动态规划.ipynb / lc-300" r:id="codexHyperlink175"/>
-    <hyperlink ref="I91" display="leetcode.cn/problems/longest-increasing-subsequence/" r:id="codexHyperlink176"/>
-    <hyperlink ref="E92" display="1187. 使数组严格递增" tooltip="15_动态规划.ipynb / lc-1187" r:id="codexHyperlink177"/>
-    <hyperlink ref="I92" display="leetcode.cn/problems/make-array-strictly-increasing/" r:id="codexHyperlink178"/>
-    <hyperlink ref="E93" display="1671. 得到山形数组的最少删除次数" tooltip="15_动态规划.ipynb / lc-1671" r:id="codexHyperlink179"/>
-    <hyperlink ref="I93" display="leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/" r:id="codexHyperlink180"/>
-    <hyperlink ref="E94" display="1964. 找出到每个位置为止的最长合法障碍赛跑路线" tooltip="15_动态规划.ipynb / lc-1964" r:id="codexHyperlink181"/>
-    <hyperlink ref="I94" display="leetcode.cn/problems/longest-obstacle-course-at-each-position/" r:id="codexHyperlink182"/>
-    <hyperlink ref="E95" display="152. 乘积最大子数组" tooltip="15_动态规划.ipynb / lc-152" r:id="codexHyperlink183"/>
-    <hyperlink ref="I95" display="leetcode.cn/problems/maximum-product-subarray/" r:id="codexHyperlink184"/>
-    <hyperlink ref="E96" display="32. 最长有效括号" tooltip="15_动态规划.ipynb / lc-32" r:id="codexHyperlink185"/>
-    <hyperlink ref="I96" display="leetcode.cn/problems/longest-valid-parentheses/" r:id="codexHyperlink186"/>
-    <hyperlink ref="E97" display="1770. 执行乘法运算的最大分数" tooltip="16_多维动态规划.ipynb / lc-1770" r:id="codexHyperlink187"/>
-    <hyperlink ref="I97" display="leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/" r:id="codexHyperlink188"/>
-    <hyperlink ref="E98" display="5. 最长回文子串" tooltip="16_多维动态规划.ipynb / lc-5" r:id="codexHyperlink189"/>
-    <hyperlink ref="I98" display="leetcode.cn/problems/longest-palindromic-substring/" r:id="codexHyperlink190"/>
-    <hyperlink ref="E99" display="516. 最长回文子序列" tooltip="16_多维动态规划.ipynb / lc-516" r:id="codexHyperlink191"/>
-    <hyperlink ref="I99" display="leetcode.cn/problems/longest-palindromic-subsequence/" r:id="codexHyperlink192"/>
-    <hyperlink ref="E100" display="647. 回文子串" tooltip="16_多维动态规划.ipynb / lc-647" r:id="codexHyperlink193"/>
-    <hyperlink ref="I100" display="leetcode.cn/problems/palindromic-substrings/" r:id="codexHyperlink194"/>
-    <hyperlink ref="E101" display="1039. 多边形三角剖分的最低得分" tooltip="16_多维动态规划.ipynb / lc-1039" r:id="codexHyperlink195"/>
-    <hyperlink ref="I101" display="leetcode.cn/problems/minimum-score-triangulation-of-polygon/" r:id="codexHyperlink196"/>
-    <hyperlink ref="E102" display="1143. 最长公共子序列" tooltip="16_多维动态规划.ipynb / lc-1143" r:id="codexHyperlink197"/>
-    <hyperlink ref="I102" display="leetcode.cn/problems/longest-common-subsequence/" r:id="codexHyperlink198"/>
-    <hyperlink ref="E103" display="712. 两个字符串的最小ASCII删除和" tooltip="16_多维动态规划.ipynb / lc-712" r:id="codexHyperlink199"/>
-    <hyperlink ref="I103" display="leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/" r:id="codexHyperlink200"/>
-    <hyperlink ref="E104" display="72. 编辑距离" tooltip="16_多维动态规划.ipynb / lc-72" r:id="codexHyperlink201"/>
-    <hyperlink ref="I104" display="leetcode.cn/problems/edit-distance/" r:id="codexHyperlink202"/>
-    <hyperlink ref="E105" display="75. 颜色分类" tooltip="17_技巧.ipynb / lc-75" r:id="codexHyperlink203"/>
-    <hyperlink ref="I105" display="leetcode.cn/problems/sort-colors/" r:id="codexHyperlink204"/>
-    <hyperlink ref="E106" display="31. 下一个排列" tooltip="17_技巧.ipynb / lc-31" r:id="codexHyperlink205"/>
-    <hyperlink ref="I106" display="leetcode.cn/problems/next-permutation/" r:id="codexHyperlink206"/>
-    <hyperlink ref="E107" display="287. 寻找重复数" tooltip="17_技巧.ipynb / lc-287" r:id="codexHyperlink207"/>
-    <hyperlink ref="I107" display="leetcode.cn/problems/find-the-duplicate-number/" r:id="codexHyperlink208"/>
+    <hyperlink ref="E49" display="108.将有序数组转换为二叉搜索树" tooltip="08_二叉树.ipynb / lc-108" r:id="codexHyperlink91"/>
+    <hyperlink ref="I49" display="leetcode.cn/problems/convert-sorted-array-to-binary-search-tree/" r:id="codexHyperlink92"/>
+    <hyperlink ref="E50" display="230. 二叉搜索树中第 K 小的元素" tooltip="08_二叉树.ipynb / lc-230" r:id="codexHyperlink93"/>
+    <hyperlink ref="I50" display="leetcode.cn/problems/kth-smallest-element-in-a-bst/" r:id="codexHyperlink94"/>
+    <hyperlink ref="E51" display="114. 二叉树展开为链表" tooltip="08_二叉树.ipynb / lc-114" r:id="codexHyperlink95"/>
+    <hyperlink ref="I51" display="leetcode.cn/problems/flatten-binary-tree-to-linked-list/" r:id="codexHyperlink96"/>
+    <hyperlink ref="E52" display="105. 从前序与中序遍历序列构造二叉树" tooltip="08_二叉树.ipynb / lc-105" r:id="codexHyperlink97"/>
+    <hyperlink ref="I52" display="leetcode.cn/problems/construct-binary-tree-from-preorder-and-inorder-traversal/" r:id="codexHyperlink98"/>
+    <hyperlink ref="E53" display="437. 路径总和 III" tooltip="08_二叉树.ipynb / lc-437" r:id="codexHyperlink99"/>
+    <hyperlink ref="I53" display="leetcode.cn/problems/path-sum-iii/" r:id="codexHyperlink100"/>
+    <hyperlink ref="E54" display="236. 二叉树的最近公共祖先" tooltip="08_二叉树.ipynb / lc-236" r:id="codexHyperlink101"/>
+    <hyperlink ref="I54" display="leetcode.cn/problems/lowest-common-ancestor-of-a-binary-tree/" r:id="codexHyperlink102"/>
+    <hyperlink ref="E55" display="235. 二叉搜索树的最近公共祖先" tooltip="08_二叉树.ipynb / lc-235" r:id="codexHyperlink103"/>
+    <hyperlink ref="I55" display="https://leetcode.cn/problems/lowest-common-ancestor-of-a-binary-search-tree/" r:id="codexHyperlink104"/>
+    <hyperlink ref="E56" display="124. 二叉树中的最大路径和" tooltip="08_二叉树.ipynb / lc-124" r:id="codexHyperlink105"/>
+    <hyperlink ref="I56" display="leetcode.cn/problems/binary-tree-maximum-path-sum/" r:id="codexHyperlink106"/>
+    <hyperlink ref="E57" display="337. 打家劫舍 III" tooltip="08_二叉树.ipynb / lc-337" r:id="codexHyperlink107"/>
+    <hyperlink ref="I57" display="leetcode.cn/problems/house-robber-iii/" r:id="codexHyperlink108"/>
+    <hyperlink ref="E58" display="968. 监控二叉树" tooltip="08_二叉树.ipynb / lc-968" r:id="codexHyperlink109"/>
+    <hyperlink ref="I58" display="leetcode.cn/problems/binary-tree-cameras/" r:id="codexHyperlink110"/>
+    <hyperlink ref="E59" display="200. 岛屿数量" tooltip="09_图论.ipynb / lc-200" r:id="codexHyperlink111"/>
+    <hyperlink ref="I59" display="leetcode.cn/problems/number-of-islands/" r:id="codexHyperlink112"/>
+    <hyperlink ref="E60" display="994. 腐烂的橘子" tooltip="09_图论.ipynb / lc-994" r:id="codexHyperlink113"/>
+    <hyperlink ref="I60" display="leetcode.cn/problems/rotting-oranges/" r:id="codexHyperlink114"/>
+    <hyperlink ref="E61" display="207. 课程表" tooltip="09_图论.ipynb / lc-207" r:id="codexHyperlink115"/>
+    <hyperlink ref="I61" display="leetcode.cn/problems/course-schedule/" r:id="codexHyperlink116"/>
+    <hyperlink ref="E62" display="208. 实现 Trie (前缀树)" tooltip="09_图论.ipynb / lc-208" r:id="codexHyperlink117"/>
+    <hyperlink ref="I62" display="leetcode.cn/problems/implement-trie-prefix-tree/" r:id="codexHyperlink118"/>
+    <hyperlink ref="E63" display="46. 全排列" tooltip="10_回溯.ipynb / lc-46" r:id="codexHyperlink119"/>
+    <hyperlink ref="I63" display="leetcode.cn/problems/permutations/" r:id="codexHyperlink120"/>
+    <hyperlink ref="E64" display="78. 子集" tooltip="10_回溯.ipynb / lc-78" r:id="codexHyperlink121"/>
+    <hyperlink ref="I64" display="leetcode.cn/problems/subsets/" r:id="codexHyperlink122"/>
+    <hyperlink ref="E65" display="17. 电话号码的字母组合" tooltip="10_回溯.ipynb / lc-17" r:id="codexHyperlink123"/>
+    <hyperlink ref="I65" display="leetcode.cn/problems/letter-combinations-of-a-phone-number/" r:id="codexHyperlink124"/>
+    <hyperlink ref="E66" display="39. 组合总和" tooltip="10_回溯.ipynb / lc-39" r:id="codexHyperlink125"/>
+    <hyperlink ref="I66" display="leetcode.cn/problems/combination-sum/" r:id="codexHyperlink126"/>
+    <hyperlink ref="E67" display="216. 组合总和 III" tooltip="10_回溯.ipynb / lc-216" r:id="codexHyperlink127"/>
+    <hyperlink ref="I67" display="leetcode.cn/problems/combination-sum-iii/" r:id="codexHyperlink128"/>
+    <hyperlink ref="E68" display="22. 括号生成" tooltip="10_回溯.ipynb / lc-22" r:id="codexHyperlink129"/>
+    <hyperlink ref="I68" display="leetcode.cn/problems/generate-parentheses/" r:id="codexHyperlink130"/>
+    <hyperlink ref="E69" display="79. 单词搜索" tooltip="10_回溯.ipynb / lc-79" r:id="codexHyperlink131"/>
+    <hyperlink ref="I69" display="leetcode.cn/problems/word-search/" r:id="codexHyperlink132"/>
+    <hyperlink ref="E70" display="131. 分割回文串" tooltip="10_回溯.ipynb / lc-131" r:id="codexHyperlink133"/>
+    <hyperlink ref="I70" display="leetcode.cn/problems/palindrome-partitioning/" r:id="codexHyperlink134"/>
+    <hyperlink ref="E71" display="51. N 皇后" tooltip="10_回溯.ipynb / lc-51" r:id="codexHyperlink135"/>
+    <hyperlink ref="I71" display="leetcode.cn/problems/n-queens/" r:id="codexHyperlink136"/>
+    <hyperlink ref="E72" display="74. 搜索二维矩阵" tooltip="11_二分查找.ipynb / lc-74" r:id="codexHyperlink137"/>
+    <hyperlink ref="I72" display="leetcode.cn/problems/search-a-2d-matrix/" r:id="codexHyperlink138"/>
+    <hyperlink ref="E73" display="34. 在排序数组中查找元素的第一个和最后一个位置" tooltip="11_二分查找.ipynb / lc-34" r:id="codexHyperlink139"/>
+    <hyperlink ref="I73" display="leetcode.cn/problems/find-first-and-last-position-of-element-in-sorted-array/" r:id="codexHyperlink140"/>
+    <hyperlink ref="E74" display="33. 搜索旋转排序数组" tooltip="11_二分查找.ipynb / lc-33" r:id="codexHyperlink141"/>
+    <hyperlink ref="I74" display="leetcode.cn/problems/search-in-rotated-sorted-array/" r:id="codexHyperlink142"/>
+    <hyperlink ref="E75" display="153. 寻找旋转排序数组中的最小值" tooltip="11_二分查找.ipynb / lc-153" r:id="codexHyperlink143"/>
+    <hyperlink ref="I75" display="leetcode.cn/problems/find-minimum-in-rotated-sorted-array/" r:id="codexHyperlink144"/>
+    <hyperlink ref="E76" display="162. 寻找峰值" tooltip="11_二分查找.ipynb / lc-162" r:id="codexHyperlink145"/>
+    <hyperlink ref="I76" display="leetcode.cn/problems/find-peak-element/" r:id="codexHyperlink146"/>
+    <hyperlink ref="E77" display="4. 寻找两个正序数组的中位数" tooltip="11_二分查找.ipynb / lc-4" r:id="codexHyperlink147"/>
+    <hyperlink ref="I77" display="leetcode.cn/problems/median-of-two-sorted-arrays/" r:id="codexHyperlink148"/>
+    <hyperlink ref="E78" display="155. 最小栈" tooltip="12_栈.ipynb / lc-155" r:id="codexHyperlink149"/>
+    <hyperlink ref="I78" display="leetcode.cn/problems/min-stack/" r:id="codexHyperlink150"/>
+    <hyperlink ref="E79" display="20.有效括号" tooltip="12_栈.ipynb / lc-20" r:id="codexHyperlink151"/>
+    <hyperlink ref="I79" display="leetcode.cn/problems/valid-parentheses/" r:id="codexHyperlink152"/>
+    <hyperlink ref="E80" display="394. 字符串解码" tooltip="12_栈.ipynb / lc-394" r:id="codexHyperlink153"/>
+    <hyperlink ref="I80" display="leetcode.cn/problems/decode-string/" r:id="codexHyperlink154"/>
+    <hyperlink ref="E81" display="739. 每日温度" tooltip="12_栈.ipynb / lc-739" r:id="codexHyperlink155"/>
+    <hyperlink ref="I81" display="leetcode.cn/problems/daily-temperatures/" r:id="codexHyperlink156"/>
+    <hyperlink ref="E82" display="84. 柱状图中最大的矩形" tooltip="12_栈.ipynb / lc-84" r:id="codexHyperlink157"/>
+    <hyperlink ref="I82" display="leetcode.cn/problems/largest-rectangle-in-histogram/" r:id="codexHyperlink158"/>
+    <hyperlink ref="E83" display="215. 数组中的第 K 个最大元素" tooltip="13_堆.ipynb / lc-215" r:id="codexHyperlink159"/>
+    <hyperlink ref="I83" display="leetcode.cn/problems/kth-largest-element-in-an-array/" r:id="codexHyperlink160"/>
+    <hyperlink ref="E84" display="347.前k个高频元素" tooltip="13_堆.ipynb / lc-347" r:id="codexHyperlink161"/>
+    <hyperlink ref="I84" display="leetcode.cn/problems/top-k-frequent-elements/" r:id="codexHyperlink162"/>
+    <hyperlink ref="E85" display="295. 数据流的中位数" tooltip="13_堆.ipynb / lc-295" r:id="codexHyperlink163"/>
+    <hyperlink ref="I85" display="leetcode.cn/problems/find-median-from-data-stream/" r:id="codexHyperlink164"/>
+    <hyperlink ref="E86" display="122. 买卖股票的最佳时机 II" tooltip="14_贪心算法.ipynb / lc-122" r:id="codexHyperlink165"/>
+    <hyperlink ref="I86" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-ii/" r:id="codexHyperlink166"/>
+    <hyperlink ref="E87" display="188. 买卖股票的最佳时机 IV" tooltip="14_贪心算法.ipynb / lc-188" r:id="codexHyperlink167"/>
+    <hyperlink ref="I87" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-iv/" r:id="codexHyperlink168"/>
+    <hyperlink ref="E88" display="309. 买卖股票的最佳时机含冷冻期" tooltip="14_贪心算法.ipynb / lc-309" r:id="codexHyperlink169"/>
+    <hyperlink ref="I88" display="leetcode.cn/problems/best-time-to-buy-and-sell-stock-with-cooldown/" r:id="codexHyperlink170"/>
+    <hyperlink ref="E89" display="309. 买卖股票的最佳时机含冷冻期" tooltip="14_贪心算法.ipynb / lc-55" r:id="codexHyperlink171"/>
+    <hyperlink ref="I89" display="leetcode.cn/problems/jump-game/" r:id="codexHyperlink172"/>
+    <hyperlink ref="E90" display="45. 跳跃游戏 II" tooltip="14_贪心算法.ipynb / lc-45" r:id="codexHyperlink173"/>
+    <hyperlink ref="I90" display="leetcode.cn/problems/jump-game-ii/" r:id="codexHyperlink174"/>
+    <hyperlink ref="E91" display="2266. 统计打字方案数" tooltip="15_动态规划.ipynb / lc-2266" r:id="codexHyperlink175"/>
+    <hyperlink ref="I91" display="leetcode.cn/problems/count-number-of-texts/" r:id="codexHyperlink176"/>
+    <hyperlink ref="E92" display="198. 打家劫舍" tooltip="15_动态规划.ipynb / lc-198" r:id="codexHyperlink177"/>
+    <hyperlink ref="I92" display="leetcode.cn/problems/house-robber/" r:id="codexHyperlink178"/>
+    <hyperlink ref="E93" display="213. 打家劫舍 II" tooltip="15_动态规划.ipynb / lc-213" r:id="codexHyperlink179"/>
+    <hyperlink ref="I93" display="leetcode.cn/problems/house-robber-ii/" r:id="codexHyperlink180"/>
+    <hyperlink ref="E94" display="322. 零钱兑换" tooltip="15_动态规划.ipynb / lc-322" r:id="codexHyperlink181"/>
+    <hyperlink ref="I94" display="leetcode.cn/problems/coin-change/" r:id="codexHyperlink182"/>
+    <hyperlink ref="E95" display="416.分割等和子集" tooltip="15_动态规划.ipynb / lc-416" r:id="codexHyperlink183"/>
+    <hyperlink ref="I95" display="leetcode.cn/problems/partition-equal-subset-sum/" r:id="codexHyperlink184"/>
+    <hyperlink ref="E96" display="494. 目标和" tooltip="15_动态规划.ipynb / lc-494" r:id="codexHyperlink185"/>
+    <hyperlink ref="I96" display="leetcode.cn/problems/target-sum/" r:id="codexHyperlink186"/>
+    <hyperlink ref="E97" display="139. 单词拆分" tooltip="15_动态规划.ipynb / lc-139" r:id="codexHyperlink187"/>
+    <hyperlink ref="I97" display="leetcode.cn/problems/word-break/" r:id="codexHyperlink188"/>
+    <hyperlink ref="E98" display="300. 最长递增子序列" tooltip="15_动态规划.ipynb / lc-300" r:id="codexHyperlink189"/>
+    <hyperlink ref="I98" display="leetcode.cn/problems/longest-increasing-subsequence/" r:id="codexHyperlink190"/>
+    <hyperlink ref="E99" display="1187. 使数组严格递增" tooltip="15_动态规划.ipynb / lc-1187" r:id="codexHyperlink191"/>
+    <hyperlink ref="I99" display="leetcode.cn/problems/make-array-strictly-increasing/" r:id="codexHyperlink192"/>
+    <hyperlink ref="E100" display="1671. 得到山形数组的最少删除次数" tooltip="15_动态规划.ipynb / lc-1671" r:id="codexHyperlink193"/>
+    <hyperlink ref="I100" display="leetcode.cn/problems/minimum-number-of-removals-to-make-mountain-array/" r:id="codexHyperlink194"/>
+    <hyperlink ref="E101" display="1964. 找出到每个位置为止的最长合法障碍赛跑路线" tooltip="15_动态规划.ipynb / lc-1964" r:id="codexHyperlink195"/>
+    <hyperlink ref="I101" display="leetcode.cn/problems/longest-obstacle-course-at-each-position/" r:id="codexHyperlink196"/>
+    <hyperlink ref="E102" display="152. 乘积最大子数组" tooltip="15_动态规划.ipynb / lc-152" r:id="codexHyperlink197"/>
+    <hyperlink ref="I102" display="leetcode.cn/problems/maximum-product-subarray/" r:id="codexHyperlink198"/>
+    <hyperlink ref="E103" display="32. 最长有效括号" tooltip="15_动态规划.ipynb / lc-32" r:id="codexHyperlink199"/>
+    <hyperlink ref="I103" display="leetcode.cn/problems/longest-valid-parentheses/" r:id="codexHyperlink200"/>
+    <hyperlink ref="E104" display="1770. 执行乘法运算的最大分数" tooltip="16_多维动态规划.ipynb / lc-1770" r:id="codexHyperlink201"/>
+    <hyperlink ref="I104" display="leetcode.cn/problems/maximum-score-from-performing-multiplication-operations/" r:id="codexHyperlink202"/>
+    <hyperlink ref="E105" display="62. 不同路径" tooltip="16_多维动态规划.ipynb / lc-62" r:id="codexHyperlink203"/>
+    <hyperlink ref="I105" display="leetcode.cn/problems/unique-paths/" r:id="codexHyperlink204"/>
+    <hyperlink ref="E106" display="64.最小路径和" tooltip="16_多维动态规划.ipynb / lc-64" r:id="codexHyperlink205"/>
+    <hyperlink ref="I106" display="leetcode.cn/problems/minimum-path-sum/" r:id="codexHyperlink206"/>
+    <hyperlink ref="E107" display="5. 最长回文子串" tooltip="16_多维动态规划.ipynb / lc-5" r:id="codexHyperlink207"/>
+    <hyperlink ref="I107" display="leetcode.cn/problems/longest-palindromic-substring/" r:id="codexHyperlink208"/>
+    <hyperlink ref="E108" display="516. 最长回文子序列" tooltip="16_多维动态规划.ipynb / lc-516" r:id="codexHyperlink209"/>
+    <hyperlink ref="I108" display="leetcode.cn/problems/longest-palindromic-subsequence/" r:id="codexHyperlink210"/>
+    <hyperlink ref="E109" display="647. 回文子串" tooltip="16_多维动态规划.ipynb / lc-647" r:id="codexHyperlink211"/>
+    <hyperlink ref="I109" display="leetcode.cn/problems/palindromic-substrings/" r:id="codexHyperlink212"/>
+    <hyperlink ref="E110" display="1039. 多边形三角剖分的最低得分" tooltip="16_多维动态规划.ipynb / lc-1039" r:id="codexHyperlink213"/>
+    <hyperlink ref="I110" display="leetcode.cn/problems/minimum-score-triangulation-of-polygon/" r:id="codexHyperlink214"/>
+    <hyperlink ref="E111" display="1143. 最长公共子序列" tooltip="16_多维动态规划.ipynb / lc-1143" r:id="codexHyperlink215"/>
+    <hyperlink ref="I111" display="leetcode.cn/problems/longest-common-subsequence/" r:id="codexHyperlink216"/>
+    <hyperlink ref="E112" display="712. 两个字符串的最小ASCII删除和" tooltip="16_多维动态规划.ipynb / lc-712" r:id="codexHyperlink217"/>
+    <hyperlink ref="I112" display="leetcode.cn/problems/minimum-ascii-delete-sum-for-two-strings/" r:id="codexHyperlink218"/>
+    <hyperlink ref="E113" display="72. 编辑距离" tooltip="16_多维动态规划.ipynb / lc-72" r:id="codexHyperlink219"/>
+    <hyperlink ref="I113" display="leetcode.cn/problems/edit-distance/" r:id="codexHyperlink220"/>
+    <hyperlink ref="E114" display="75. 颜色分类" tooltip="17_技巧.ipynb / lc-75" r:id="codexHyperlink221"/>
+    <hyperlink ref="I114" display="leetcode.cn/problems/sort-colors/" r:id="codexHyperlink222"/>
+    <hyperlink ref="E115" display="136. 只出现一次的数字" tooltip="17_技巧.ipynb / lc-136" r:id="codexHyperlink223"/>
+    <hyperlink ref="I115" display="leetcode.cn/problems/single-number/" r:id="codexHyperlink224"/>
+    <hyperlink ref="E116" display="31. 下一个排列" tooltip="17_技巧.ipynb / lc-31" r:id="codexHyperlink225"/>
+    <hyperlink ref="I116" display="leetcode.cn/problems/next-permutation/" r:id="codexHyperlink226"/>
+    <hyperlink ref="E117" display="287. 寻找重复数" tooltip="17_技巧.ipynb / lc-287" r:id="codexHyperlink227"/>
+    <hyperlink ref="I117" display="leetcode.cn/problems/find-the-duplicate-number/" r:id="codexHyperlink228"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>